<commit_message>
add error response dto
</commit_message>
<xml_diff>
--- a/src/main/resources/templates/summaryReportForm3.xlsx
+++ b/src/main/resources/templates/summaryReportForm3.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="21231"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5E85D29E-8FBD-4F0F-BBEE-E9AF8FCB9C3D}" xr6:coauthVersionLast="40" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5CD995A6-60EE-46AF-91B5-D31C1FC97BA1}" xr6:coauthVersionLast="40" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="402" uniqueCount="233">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="403" uniqueCount="233">
   <si>
     <t>Оперативная информация</t>
   </si>
@@ -1374,27 +1374,174 @@
     <xf numFmtId="1" fontId="3" fillId="0" borderId="34" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="35" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="37" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="34" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="3" fillId="0" borderId="38" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="4" fillId="0" borderId="32" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="49" fontId="4" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="49" fontId="4" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="4" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="4" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="49" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1402,6 +1549,9 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="4" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1410,158 +1560,8 @@
     <xf numFmtId="49" fontId="4" fillId="0" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="49" fontId="4" fillId="0" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="35" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="37" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="31" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="3" fillId="0" borderId="34" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="30" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="3" fillId="0" borderId="38" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="4" fillId="0" borderId="32" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1852,235 +1852,235 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:94" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B1" s="87" t="s">
+      <c r="B1" s="45" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="87"/>
-      <c r="D1" s="87"/>
-      <c r="E1" s="87"/>
-      <c r="F1" s="87"/>
-      <c r="G1" s="87"/>
-      <c r="H1" s="87"/>
-      <c r="I1" s="87"/>
-      <c r="J1" s="87"/>
-      <c r="K1" s="87"/>
-      <c r="L1" s="87"/>
-      <c r="M1" s="87"/>
-      <c r="N1" s="87"/>
-      <c r="O1" s="87"/>
-      <c r="P1" s="87"/>
-      <c r="Q1" s="87"/>
-      <c r="R1" s="87"/>
-      <c r="S1" s="87"/>
-      <c r="T1" s="87"/>
-      <c r="U1" s="87"/>
-      <c r="V1" s="87"/>
-      <c r="W1" s="87"/>
-      <c r="X1" s="87"/>
-      <c r="Y1" s="87"/>
-      <c r="Z1" s="87"/>
-      <c r="AA1" s="87"/>
+      <c r="C1" s="45"/>
+      <c r="D1" s="45"/>
+      <c r="E1" s="45"/>
+      <c r="F1" s="45"/>
+      <c r="G1" s="45"/>
+      <c r="H1" s="45"/>
+      <c r="I1" s="45"/>
+      <c r="J1" s="45"/>
+      <c r="K1" s="45"/>
+      <c r="L1" s="45"/>
+      <c r="M1" s="45"/>
+      <c r="N1" s="45"/>
+      <c r="O1" s="45"/>
+      <c r="P1" s="45"/>
+      <c r="Q1" s="45"/>
+      <c r="R1" s="45"/>
+      <c r="S1" s="45"/>
+      <c r="T1" s="45"/>
+      <c r="U1" s="45"/>
+      <c r="V1" s="45"/>
+      <c r="W1" s="45"/>
+      <c r="X1" s="45"/>
+      <c r="Y1" s="45"/>
+      <c r="Z1" s="45"/>
+      <c r="AA1" s="45"/>
     </row>
     <row r="2" spans="1:94" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B2" s="87" t="s">
+      <c r="B2" s="45" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="87"/>
-      <c r="D2" s="87"/>
-      <c r="E2" s="87"/>
-      <c r="F2" s="87"/>
-      <c r="G2" s="87"/>
-      <c r="H2" s="87"/>
-      <c r="I2" s="87"/>
-      <c r="J2" s="87"/>
-      <c r="K2" s="87"/>
-      <c r="L2" s="87"/>
-      <c r="M2" s="87"/>
-      <c r="N2" s="87"/>
-      <c r="O2" s="87"/>
-      <c r="P2" s="87"/>
-      <c r="Q2" s="87"/>
-      <c r="R2" s="87"/>
-      <c r="S2" s="87"/>
-      <c r="T2" s="87"/>
-      <c r="U2" s="87"/>
-      <c r="V2" s="87"/>
-      <c r="W2" s="87"/>
-      <c r="X2" s="87"/>
-      <c r="Y2" s="87"/>
-      <c r="Z2" s="87"/>
-      <c r="AA2" s="87"/>
+      <c r="C2" s="45"/>
+      <c r="D2" s="45"/>
+      <c r="E2" s="45"/>
+      <c r="F2" s="45"/>
+      <c r="G2" s="45"/>
+      <c r="H2" s="45"/>
+      <c r="I2" s="45"/>
+      <c r="J2" s="45"/>
+      <c r="K2" s="45"/>
+      <c r="L2" s="45"/>
+      <c r="M2" s="45"/>
+      <c r="N2" s="45"/>
+      <c r="O2" s="45"/>
+      <c r="P2" s="45"/>
+      <c r="Q2" s="45"/>
+      <c r="R2" s="45"/>
+      <c r="S2" s="45"/>
+      <c r="T2" s="45"/>
+      <c r="U2" s="45"/>
+      <c r="V2" s="45"/>
+      <c r="W2" s="45"/>
+      <c r="X2" s="45"/>
+      <c r="Y2" s="45"/>
+      <c r="Z2" s="45"/>
+      <c r="AA2" s="45"/>
       <c r="AB2" s="3"/>
     </row>
     <row r="3" spans="1:94" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="L3" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="M3" s="88" t="s">
+      <c r="M3" s="46" t="s">
         <v>232</v>
       </c>
-      <c r="N3" s="88"/>
-      <c r="O3" s="88"/>
-      <c r="P3" s="88"/>
+      <c r="N3" s="46"/>
+      <c r="O3" s="46"/>
+      <c r="P3" s="46"/>
     </row>
     <row r="4" spans="1:94" s="2" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="5" spans="1:94" s="2" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="89" t="s">
+      <c r="A5" s="47" t="s">
         <v>3</v>
       </c>
-      <c r="B5" s="90" t="s">
+      <c r="B5" s="50" t="s">
         <v>4</v>
       </c>
-      <c r="C5" s="68" t="s">
+      <c r="C5" s="53" t="s">
         <v>5</v>
       </c>
-      <c r="D5" s="67"/>
-      <c r="E5" s="67"/>
-      <c r="F5" s="67"/>
-      <c r="G5" s="67"/>
-      <c r="H5" s="67"/>
-      <c r="I5" s="67"/>
-      <c r="J5" s="67"/>
-      <c r="K5" s="67"/>
-      <c r="L5" s="67"/>
-      <c r="M5" s="67"/>
-      <c r="N5" s="67"/>
-      <c r="O5" s="67"/>
-      <c r="P5" s="67"/>
-      <c r="Q5" s="67"/>
-      <c r="R5" s="67"/>
-      <c r="S5" s="67"/>
-      <c r="T5" s="67"/>
-      <c r="U5" s="67"/>
-      <c r="V5" s="67"/>
-      <c r="W5" s="67"/>
-      <c r="X5" s="67"/>
-      <c r="Y5" s="67"/>
-      <c r="Z5" s="67"/>
-      <c r="AA5" s="67"/>
-      <c r="AB5" s="67"/>
-      <c r="AC5" s="67"/>
-      <c r="AD5" s="67"/>
-      <c r="AE5" s="67"/>
-      <c r="AF5" s="67"/>
-      <c r="AG5" s="67"/>
-      <c r="AH5" s="67"/>
-      <c r="AI5" s="61" t="s">
+      <c r="D5" s="54"/>
+      <c r="E5" s="54"/>
+      <c r="F5" s="54"/>
+      <c r="G5" s="54"/>
+      <c r="H5" s="54"/>
+      <c r="I5" s="54"/>
+      <c r="J5" s="54"/>
+      <c r="K5" s="54"/>
+      <c r="L5" s="54"/>
+      <c r="M5" s="54"/>
+      <c r="N5" s="54"/>
+      <c r="O5" s="54"/>
+      <c r="P5" s="54"/>
+      <c r="Q5" s="54"/>
+      <c r="R5" s="54"/>
+      <c r="S5" s="54"/>
+      <c r="T5" s="54"/>
+      <c r="U5" s="54"/>
+      <c r="V5" s="54"/>
+      <c r="W5" s="54"/>
+      <c r="X5" s="54"/>
+      <c r="Y5" s="54"/>
+      <c r="Z5" s="54"/>
+      <c r="AA5" s="54"/>
+      <c r="AB5" s="54"/>
+      <c r="AC5" s="54"/>
+      <c r="AD5" s="54"/>
+      <c r="AE5" s="54"/>
+      <c r="AF5" s="54"/>
+      <c r="AG5" s="54"/>
+      <c r="AH5" s="54"/>
+      <c r="AI5" s="67" t="s">
         <v>6</v>
       </c>
-      <c r="AJ5" s="62"/>
-      <c r="AK5" s="63"/>
-      <c r="AL5" s="61" t="s">
+      <c r="AJ5" s="68"/>
+      <c r="AK5" s="69"/>
+      <c r="AL5" s="67" t="s">
         <v>43</v>
       </c>
-      <c r="AM5" s="62"/>
-      <c r="AN5" s="63"/>
-      <c r="AO5" s="64" t="s">
+      <c r="AM5" s="68"/>
+      <c r="AN5" s="69"/>
+      <c r="AO5" s="70" t="s">
         <v>7</v>
       </c>
-      <c r="AP5" s="65"/>
-      <c r="AQ5" s="66"/>
-      <c r="AR5" s="67" t="s">
+      <c r="AP5" s="71"/>
+      <c r="AQ5" s="72"/>
+      <c r="AR5" s="54" t="s">
         <v>8</v>
       </c>
-      <c r="AS5" s="67"/>
-      <c r="AT5" s="67"/>
-      <c r="AU5" s="67"/>
-      <c r="AV5" s="67"/>
-      <c r="AW5" s="67"/>
-      <c r="AX5" s="67"/>
-      <c r="AY5" s="67"/>
-      <c r="AZ5" s="67"/>
-      <c r="BA5" s="67"/>
-      <c r="BB5" s="67"/>
-      <c r="BC5" s="67"/>
-      <c r="BD5" s="67"/>
-      <c r="BE5" s="67"/>
-      <c r="BF5" s="67"/>
-      <c r="BG5" s="67"/>
-      <c r="BH5" s="68" t="s">
+      <c r="AS5" s="54"/>
+      <c r="AT5" s="54"/>
+      <c r="AU5" s="54"/>
+      <c r="AV5" s="54"/>
+      <c r="AW5" s="54"/>
+      <c r="AX5" s="54"/>
+      <c r="AY5" s="54"/>
+      <c r="AZ5" s="54"/>
+      <c r="BA5" s="54"/>
+      <c r="BB5" s="54"/>
+      <c r="BC5" s="54"/>
+      <c r="BD5" s="54"/>
+      <c r="BE5" s="54"/>
+      <c r="BF5" s="54"/>
+      <c r="BG5" s="54"/>
+      <c r="BH5" s="53" t="s">
         <v>9</v>
       </c>
-      <c r="BI5" s="67"/>
-      <c r="BJ5" s="67"/>
-      <c r="BK5" s="67"/>
-      <c r="BL5" s="67"/>
-      <c r="BM5" s="67"/>
-      <c r="BN5" s="67"/>
-      <c r="BO5" s="67"/>
-      <c r="BP5" s="67"/>
-      <c r="BQ5" s="67"/>
-      <c r="BR5" s="67"/>
-      <c r="BS5" s="67"/>
-      <c r="BT5" s="67"/>
-      <c r="BU5" s="67"/>
-      <c r="BV5" s="67"/>
-      <c r="BW5" s="67"/>
-      <c r="BX5" s="67"/>
-      <c r="BY5" s="67"/>
-      <c r="BZ5" s="67"/>
-      <c r="CA5" s="67"/>
-      <c r="CB5" s="67"/>
-      <c r="CC5" s="67"/>
-      <c r="CD5" s="67"/>
-      <c r="CE5" s="67"/>
-      <c r="CF5" s="67"/>
-      <c r="CG5" s="67"/>
-      <c r="CH5" s="67"/>
-      <c r="CI5" s="69"/>
-      <c r="CJ5" s="70" t="s">
+      <c r="BI5" s="54"/>
+      <c r="BJ5" s="54"/>
+      <c r="BK5" s="54"/>
+      <c r="BL5" s="54"/>
+      <c r="BM5" s="54"/>
+      <c r="BN5" s="54"/>
+      <c r="BO5" s="54"/>
+      <c r="BP5" s="54"/>
+      <c r="BQ5" s="54"/>
+      <c r="BR5" s="54"/>
+      <c r="BS5" s="54"/>
+      <c r="BT5" s="54"/>
+      <c r="BU5" s="54"/>
+      <c r="BV5" s="54"/>
+      <c r="BW5" s="54"/>
+      <c r="BX5" s="54"/>
+      <c r="BY5" s="54"/>
+      <c r="BZ5" s="54"/>
+      <c r="CA5" s="54"/>
+      <c r="CB5" s="54"/>
+      <c r="CC5" s="54"/>
+      <c r="CD5" s="54"/>
+      <c r="CE5" s="54"/>
+      <c r="CF5" s="54"/>
+      <c r="CG5" s="54"/>
+      <c r="CH5" s="54"/>
+      <c r="CI5" s="73"/>
+      <c r="CJ5" s="74" t="s">
         <v>10</v>
       </c>
-      <c r="CK5" s="70"/>
-      <c r="CL5" s="70"/>
-      <c r="CM5" s="70"/>
-      <c r="CN5" s="70"/>
-      <c r="CO5" s="70"/>
-      <c r="CP5" s="71" t="s">
+      <c r="CK5" s="74"/>
+      <c r="CL5" s="74"/>
+      <c r="CM5" s="74"/>
+      <c r="CN5" s="74"/>
+      <c r="CO5" s="74"/>
+      <c r="CP5" s="75" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="6" spans="1:94" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="59"/>
-      <c r="B6" s="50"/>
-      <c r="C6" s="91" t="s">
+      <c r="A6" s="48"/>
+      <c r="B6" s="51"/>
+      <c r="C6" s="55" t="s">
         <v>12</v>
       </c>
-      <c r="D6" s="74"/>
-      <c r="E6" s="74"/>
-      <c r="F6" s="74"/>
-      <c r="G6" s="74"/>
-      <c r="H6" s="74"/>
-      <c r="I6" s="74"/>
-      <c r="J6" s="74"/>
-      <c r="K6" s="74"/>
-      <c r="L6" s="74"/>
-      <c r="M6" s="74"/>
-      <c r="N6" s="74"/>
-      <c r="O6" s="74"/>
-      <c r="P6" s="74"/>
-      <c r="Q6" s="80" t="s">
+      <c r="D6" s="56"/>
+      <c r="E6" s="56"/>
+      <c r="F6" s="56"/>
+      <c r="G6" s="56"/>
+      <c r="H6" s="56"/>
+      <c r="I6" s="56"/>
+      <c r="J6" s="56"/>
+      <c r="K6" s="56"/>
+      <c r="L6" s="56"/>
+      <c r="M6" s="56"/>
+      <c r="N6" s="56"/>
+      <c r="O6" s="56"/>
+      <c r="P6" s="56"/>
+      <c r="Q6" s="57" t="s">
         <v>13</v>
       </c>
-      <c r="R6" s="80"/>
-      <c r="S6" s="80"/>
-      <c r="T6" s="80"/>
-      <c r="U6" s="80"/>
-      <c r="V6" s="80"/>
-      <c r="W6" s="80"/>
-      <c r="X6" s="80"/>
-      <c r="Y6" s="80"/>
-      <c r="Z6" s="80"/>
-      <c r="AA6" s="80"/>
-      <c r="AB6" s="80"/>
-      <c r="AC6" s="80" t="s">
+      <c r="R6" s="57"/>
+      <c r="S6" s="57"/>
+      <c r="T6" s="57"/>
+      <c r="U6" s="57"/>
+      <c r="V6" s="57"/>
+      <c r="W6" s="57"/>
+      <c r="X6" s="57"/>
+      <c r="Y6" s="57"/>
+      <c r="Z6" s="57"/>
+      <c r="AA6" s="57"/>
+      <c r="AB6" s="57"/>
+      <c r="AC6" s="57" t="s">
         <v>14</v>
       </c>
-      <c r="AD6" s="80"/>
-      <c r="AE6" s="80"/>
-      <c r="AF6" s="80"/>
-      <c r="AG6" s="80"/>
-      <c r="AH6" s="76"/>
+      <c r="AD6" s="57"/>
+      <c r="AE6" s="57"/>
+      <c r="AF6" s="57"/>
+      <c r="AG6" s="57"/>
+      <c r="AH6" s="58"/>
       <c r="AI6" s="5" t="s">
         <v>12</v>
       </c>
@@ -2108,94 +2108,94 @@
       <c r="AQ6" s="14" t="s">
         <v>15</v>
       </c>
-      <c r="AR6" s="74" t="s">
+      <c r="AR6" s="56" t="s">
         <v>12</v>
       </c>
-      <c r="AS6" s="74"/>
-      <c r="AT6" s="74"/>
-      <c r="AU6" s="74"/>
-      <c r="AV6" s="74"/>
-      <c r="AW6" s="74"/>
-      <c r="AX6" s="75"/>
-      <c r="AY6" s="76" t="s">
+      <c r="AS6" s="56"/>
+      <c r="AT6" s="56"/>
+      <c r="AU6" s="56"/>
+      <c r="AV6" s="56"/>
+      <c r="AW6" s="56"/>
+      <c r="AX6" s="78"/>
+      <c r="AY6" s="58" t="s">
         <v>13</v>
       </c>
-      <c r="AZ6" s="77"/>
-      <c r="BA6" s="77"/>
-      <c r="BB6" s="77"/>
-      <c r="BC6" s="78"/>
-      <c r="BD6" s="76" t="s">
+      <c r="AZ6" s="61"/>
+      <c r="BA6" s="61"/>
+      <c r="BB6" s="61"/>
+      <c r="BC6" s="62"/>
+      <c r="BD6" s="58" t="s">
         <v>14</v>
       </c>
-      <c r="BE6" s="77"/>
-      <c r="BF6" s="77"/>
+      <c r="BE6" s="61"/>
+      <c r="BF6" s="61"/>
       <c r="BG6" s="6"/>
       <c r="BH6" s="79" t="s">
         <v>12</v>
       </c>
-      <c r="BI6" s="77"/>
-      <c r="BJ6" s="77"/>
-      <c r="BK6" s="77"/>
-      <c r="BL6" s="77"/>
-      <c r="BM6" s="77"/>
-      <c r="BN6" s="77"/>
-      <c r="BO6" s="77"/>
-      <c r="BP6" s="77"/>
-      <c r="BQ6" s="77"/>
-      <c r="BR6" s="78"/>
-      <c r="BS6" s="80" t="s">
+      <c r="BI6" s="61"/>
+      <c r="BJ6" s="61"/>
+      <c r="BK6" s="61"/>
+      <c r="BL6" s="61"/>
+      <c r="BM6" s="61"/>
+      <c r="BN6" s="61"/>
+      <c r="BO6" s="61"/>
+      <c r="BP6" s="61"/>
+      <c r="BQ6" s="61"/>
+      <c r="BR6" s="62"/>
+      <c r="BS6" s="57" t="s">
         <v>13</v>
       </c>
-      <c r="BT6" s="80"/>
-      <c r="BU6" s="80"/>
-      <c r="BV6" s="80"/>
-      <c r="BW6" s="80"/>
-      <c r="BX6" s="80"/>
-      <c r="BY6" s="80"/>
-      <c r="BZ6" s="80"/>
-      <c r="CA6" s="80"/>
-      <c r="CB6" s="80" t="s">
+      <c r="BT6" s="57"/>
+      <c r="BU6" s="57"/>
+      <c r="BV6" s="57"/>
+      <c r="BW6" s="57"/>
+      <c r="BX6" s="57"/>
+      <c r="BY6" s="57"/>
+      <c r="BZ6" s="57"/>
+      <c r="CA6" s="57"/>
+      <c r="CB6" s="57" t="s">
         <v>14</v>
       </c>
-      <c r="CC6" s="80"/>
-      <c r="CD6" s="80"/>
-      <c r="CE6" s="76"/>
-      <c r="CF6" s="76"/>
-      <c r="CG6" s="76"/>
-      <c r="CH6" s="76"/>
-      <c r="CI6" s="86"/>
-      <c r="CJ6" s="81" t="s">
+      <c r="CC6" s="57"/>
+      <c r="CD6" s="57"/>
+      <c r="CE6" s="58"/>
+      <c r="CF6" s="58"/>
+      <c r="CG6" s="58"/>
+      <c r="CH6" s="58"/>
+      <c r="CI6" s="88"/>
+      <c r="CJ6" s="80" t="s">
         <v>16</v>
       </c>
-      <c r="CK6" s="83" t="s">
+      <c r="CK6" s="82" t="s">
         <v>17</v>
       </c>
-      <c r="CL6" s="84"/>
-      <c r="CM6" s="84"/>
-      <c r="CN6" s="85"/>
-      <c r="CO6" s="80" t="s">
+      <c r="CL6" s="83"/>
+      <c r="CM6" s="83"/>
+      <c r="CN6" s="84"/>
+      <c r="CO6" s="57" t="s">
         <v>18</v>
       </c>
-      <c r="CP6" s="72"/>
+      <c r="CP6" s="76"/>
     </row>
     <row r="7" spans="1:94" s="2" customFormat="1" ht="56.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="59"/>
-      <c r="B7" s="50"/>
+      <c r="A7" s="48"/>
+      <c r="B7" s="51"/>
       <c r="C7" s="9" t="s">
         <v>19</v>
       </c>
       <c r="D7" s="8" t="s">
         <v>20</v>
       </c>
-      <c r="E7" s="76" t="s">
+      <c r="E7" s="58" t="s">
         <v>21</v>
       </c>
-      <c r="F7" s="77"/>
-      <c r="G7" s="77"/>
-      <c r="H7" s="77"/>
-      <c r="I7" s="77"/>
-      <c r="J7" s="77"/>
-      <c r="K7" s="78"/>
+      <c r="F7" s="61"/>
+      <c r="G7" s="61"/>
+      <c r="H7" s="61"/>
+      <c r="I7" s="61"/>
+      <c r="J7" s="61"/>
+      <c r="K7" s="62"/>
       <c r="L7" s="8" t="s">
         <v>22</v>
       </c>
@@ -2217,15 +2217,15 @@
       <c r="R7" s="8" t="s">
         <v>20</v>
       </c>
-      <c r="S7" s="76" t="s">
+      <c r="S7" s="58" t="s">
         <v>27</v>
       </c>
-      <c r="T7" s="77"/>
-      <c r="U7" s="77"/>
-      <c r="V7" s="77"/>
-      <c r="W7" s="77"/>
-      <c r="X7" s="77"/>
-      <c r="Y7" s="78"/>
+      <c r="T7" s="61"/>
+      <c r="U7" s="61"/>
+      <c r="V7" s="61"/>
+      <c r="W7" s="61"/>
+      <c r="X7" s="61"/>
+      <c r="Y7" s="62"/>
       <c r="Z7" s="10" t="s">
         <v>24</v>
       </c>
@@ -2253,21 +2253,21 @@
       <c r="AH7" s="15" t="s">
         <v>29</v>
       </c>
-      <c r="AI7" s="52" t="s">
+      <c r="AI7" s="85" t="s">
         <v>27</v>
       </c>
-      <c r="AJ7" s="53"/>
-      <c r="AK7" s="54"/>
-      <c r="AL7" s="52" t="s">
+      <c r="AJ7" s="86"/>
+      <c r="AK7" s="87"/>
+      <c r="AL7" s="85" t="s">
         <v>27</v>
       </c>
-      <c r="AM7" s="53"/>
-      <c r="AN7" s="54"/>
-      <c r="AO7" s="78" t="s">
+      <c r="AM7" s="86"/>
+      <c r="AN7" s="87"/>
+      <c r="AO7" s="62" t="s">
         <v>27</v>
       </c>
-      <c r="AP7" s="80"/>
-      <c r="AQ7" s="86"/>
+      <c r="AP7" s="57"/>
+      <c r="AQ7" s="88"/>
       <c r="AR7" s="7" t="s">
         <v>19</v>
       </c>
@@ -2400,7 +2400,7 @@
       <c r="CI7" s="12" t="s">
         <v>29</v>
       </c>
-      <c r="CJ7" s="82"/>
+      <c r="CJ7" s="81"/>
       <c r="CK7" s="8" t="s">
         <v>34</v>
       </c>
@@ -2413,80 +2413,79 @@
       <c r="CN7" s="8" t="s">
         <v>37</v>
       </c>
-      <c r="CO7" s="80"/>
-      <c r="CP7" s="73"/>
+      <c r="CO7" s="57"/>
+      <c r="CP7" s="77"/>
     </row>
     <row r="8" spans="1:94" s="2" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="59"/>
-      <c r="B8" s="50"/>
-      <c r="C8" s="55" t="s">
+      <c r="A8" s="48"/>
+      <c r="B8" s="51"/>
+      <c r="C8" s="59" t="s">
         <v>38</v>
       </c>
-      <c r="D8" s="92" t="s">
-        <v>44</v>
-      </c>
-      <c r="E8" s="38" t="s">
-        <v>44</v>
-      </c>
-      <c r="F8" s="38" t="s">
+      <c r="D8" s="63" t="s">
+        <v>44</v>
+      </c>
+      <c r="E8" s="65" t="s">
+        <v>44</v>
+      </c>
+      <c r="F8" s="65" t="s">
         <v>35</v>
       </c>
-      <c r="G8" s="38" t="s">
+      <c r="G8" s="65" t="s">
         <v>36</v>
       </c>
-      <c r="H8" s="38" t="s">
+      <c r="H8" s="65" t="s">
         <v>39</v>
       </c>
-      <c r="I8" s="38" t="s">
+      <c r="I8" s="65" t="s">
         <v>40</v>
       </c>
-      <c r="J8" s="38" t="s">
+      <c r="J8" s="65" t="s">
         <v>34</v>
       </c>
-      <c r="K8" s="38" t="s">
+      <c r="K8" s="65" t="s">
         <v>41</v>
       </c>
-      <c r="L8" s="38" t="s">
-        <v>44</v>
-      </c>
-      <c r="M8" s="38" t="s">
-        <v>44</v>
-      </c>
-      <c r="N8" s="38" t="str">
-        <f>$D$8</f>
-        <v>$header_year</v>
-      </c>
-      <c r="O8" s="39" t="s">
+      <c r="L8" s="65" t="s">
+        <v>44</v>
+      </c>
+      <c r="M8" s="65" t="s">
+        <v>44</v>
+      </c>
+      <c r="N8" s="65" t="s">
+        <v>44</v>
+      </c>
+      <c r="O8" s="66" t="s">
         <v>42</v>
       </c>
-      <c r="P8" s="38" t="s">
-        <v>44</v>
-      </c>
-      <c r="Q8" s="38" t="s">
+      <c r="P8" s="65" t="s">
+        <v>44</v>
+      </c>
+      <c r="Q8" s="65" t="s">
         <v>38</v>
       </c>
-      <c r="R8" s="38" t="s">
-        <v>44</v>
-      </c>
-      <c r="S8" s="38" t="s">
-        <v>44</v>
-      </c>
-      <c r="T8" s="38" t="s">
+      <c r="R8" s="65" t="s">
+        <v>44</v>
+      </c>
+      <c r="S8" s="65" t="s">
+        <v>44</v>
+      </c>
+      <c r="T8" s="65" t="s">
         <v>35</v>
       </c>
-      <c r="U8" s="38" t="s">
+      <c r="U8" s="65" t="s">
         <v>36</v>
       </c>
-      <c r="V8" s="38" t="s">
+      <c r="V8" s="65" t="s">
         <v>39</v>
       </c>
-      <c r="W8" s="38" t="s">
+      <c r="W8" s="65" t="s">
         <v>40</v>
       </c>
-      <c r="X8" s="38" t="s">
+      <c r="X8" s="65" t="s">
         <v>34</v>
       </c>
-      <c r="Y8" s="38" t="s">
+      <c r="Y8" s="65" t="s">
         <v>41</v>
       </c>
       <c r="Z8" s="16" t="s">
@@ -2495,16 +2494,16 @@
       <c r="AA8" s="16" t="s">
         <v>42</v>
       </c>
-      <c r="AB8" s="38" t="s">
-        <v>44</v>
-      </c>
-      <c r="AC8" s="38" t="s">
+      <c r="AB8" s="65" t="s">
+        <v>44</v>
+      </c>
+      <c r="AC8" s="65" t="s">
         <v>38</v>
       </c>
-      <c r="AD8" s="38" t="s">
-        <v>44</v>
-      </c>
-      <c r="AE8" s="38" t="s">
+      <c r="AD8" s="65" t="s">
+        <v>44</v>
+      </c>
+      <c r="AE8" s="65" t="s">
         <v>44</v>
       </c>
       <c r="AF8" s="16" t="s">
@@ -2516,43 +2515,43 @@
       <c r="AH8" s="15" t="s">
         <v>42</v>
       </c>
-      <c r="AI8" s="55" t="s">
-        <v>44</v>
-      </c>
-      <c r="AJ8" s="38" t="s">
-        <v>44</v>
-      </c>
-      <c r="AK8" s="48" t="s">
-        <v>44</v>
-      </c>
-      <c r="AL8" s="55" t="s">
-        <v>44</v>
-      </c>
-      <c r="AM8" s="38" t="s">
-        <v>44</v>
-      </c>
-      <c r="AN8" s="48" t="s">
-        <v>44</v>
-      </c>
-      <c r="AO8" s="40" t="s">
-        <v>44</v>
-      </c>
-      <c r="AP8" s="38" t="s">
-        <v>44</v>
-      </c>
-      <c r="AQ8" s="50" t="s">
-        <v>44</v>
-      </c>
-      <c r="AR8" s="40" t="s">
+      <c r="AI8" s="59" t="s">
+        <v>44</v>
+      </c>
+      <c r="AJ8" s="65" t="s">
+        <v>44</v>
+      </c>
+      <c r="AK8" s="98" t="s">
+        <v>44</v>
+      </c>
+      <c r="AL8" s="59" t="s">
+        <v>44</v>
+      </c>
+      <c r="AM8" s="65" t="s">
+        <v>44</v>
+      </c>
+      <c r="AN8" s="98" t="s">
+        <v>44</v>
+      </c>
+      <c r="AO8" s="97" t="s">
+        <v>44</v>
+      </c>
+      <c r="AP8" s="65" t="s">
+        <v>44</v>
+      </c>
+      <c r="AQ8" s="51" t="s">
+        <v>44</v>
+      </c>
+      <c r="AR8" s="97" t="s">
         <v>38</v>
       </c>
-      <c r="AS8" s="38" t="s">
-        <v>44</v>
-      </c>
-      <c r="AT8" s="38" t="s">
-        <v>44</v>
-      </c>
-      <c r="AU8" s="38" t="s">
+      <c r="AS8" s="65" t="s">
+        <v>44</v>
+      </c>
+      <c r="AT8" s="65" t="s">
+        <v>44</v>
+      </c>
+      <c r="AU8" s="65" t="s">
         <v>44</v>
       </c>
       <c r="AV8" s="16" t="s">
@@ -2561,16 +2560,16 @@
       <c r="AW8" s="16" t="s">
         <v>42</v>
       </c>
-      <c r="AX8" s="38" t="s">
-        <v>44</v>
-      </c>
-      <c r="AY8" s="38" t="s">
+      <c r="AX8" s="65" t="s">
+        <v>44</v>
+      </c>
+      <c r="AY8" s="65" t="s">
         <v>38</v>
       </c>
-      <c r="AZ8" s="38" t="s">
-        <v>44</v>
-      </c>
-      <c r="BA8" s="38" t="s">
+      <c r="AZ8" s="65" t="s">
+        <v>44</v>
+      </c>
+      <c r="BA8" s="65" t="s">
         <v>44</v>
       </c>
       <c r="BB8" s="16" t="s">
@@ -2579,34 +2578,34 @@
       <c r="BC8" s="16" t="s">
         <v>42</v>
       </c>
-      <c r="BD8" s="38" t="s">
+      <c r="BD8" s="65" t="s">
         <v>38</v>
       </c>
-      <c r="BE8" s="38" t="s">
-        <v>44</v>
-      </c>
-      <c r="BF8" s="38" t="s">
+      <c r="BE8" s="65" t="s">
+        <v>44</v>
+      </c>
+      <c r="BF8" s="65" t="s">
         <v>44</v>
       </c>
       <c r="BG8" s="15" t="s">
         <v>42</v>
       </c>
-      <c r="BH8" s="59" t="s">
+      <c r="BH8" s="48" t="s">
         <v>38</v>
       </c>
-      <c r="BI8" s="38" t="s">
-        <v>44</v>
-      </c>
-      <c r="BJ8" s="38" t="s">
-        <v>44</v>
-      </c>
-      <c r="BK8" s="42" t="s">
-        <v>44</v>
-      </c>
-      <c r="BL8" s="43"/>
-      <c r="BM8" s="43"/>
-      <c r="BN8" s="41"/>
-      <c r="BO8" s="38" t="s">
+      <c r="BI8" s="65" t="s">
+        <v>44</v>
+      </c>
+      <c r="BJ8" s="65" t="s">
+        <v>44</v>
+      </c>
+      <c r="BK8" s="89" t="s">
+        <v>44</v>
+      </c>
+      <c r="BL8" s="92"/>
+      <c r="BM8" s="92"/>
+      <c r="BN8" s="93"/>
+      <c r="BO8" s="65" t="s">
         <v>44</v>
       </c>
       <c r="BP8" s="16" t="s">
@@ -2615,315 +2614,315 @@
       <c r="BQ8" s="15" t="s">
         <v>42</v>
       </c>
-      <c r="BR8" s="38" t="s">
-        <v>44</v>
-      </c>
-      <c r="BS8" s="38" t="s">
+      <c r="BR8" s="65" t="s">
+        <v>44</v>
+      </c>
+      <c r="BS8" s="65" t="s">
         <v>38</v>
       </c>
-      <c r="BT8" s="38" t="s">
-        <v>44</v>
-      </c>
-      <c r="BU8" s="38" t="s">
-        <v>44</v>
-      </c>
-      <c r="BV8" s="42" t="s">
-        <v>44</v>
-      </c>
-      <c r="BW8" s="43"/>
-      <c r="BX8" s="43"/>
-      <c r="BY8" s="41"/>
+      <c r="BT8" s="65" t="s">
+        <v>44</v>
+      </c>
+      <c r="BU8" s="65" t="s">
+        <v>44</v>
+      </c>
+      <c r="BV8" s="89" t="s">
+        <v>44</v>
+      </c>
+      <c r="BW8" s="92"/>
+      <c r="BX8" s="92"/>
+      <c r="BY8" s="93"/>
       <c r="BZ8" s="16" t="s">
         <v>42</v>
       </c>
       <c r="CA8" s="16" t="s">
         <v>42</v>
       </c>
-      <c r="CB8" s="38" t="s">
+      <c r="CB8" s="65" t="s">
         <v>38</v>
       </c>
-      <c r="CC8" s="38" t="s">
-        <v>44</v>
-      </c>
-      <c r="CD8" s="38" t="s">
-        <v>44</v>
-      </c>
-      <c r="CE8" s="42" t="s">
-        <v>44</v>
-      </c>
-      <c r="CF8" s="43"/>
-      <c r="CG8" s="43"/>
-      <c r="CH8" s="41"/>
+      <c r="CC8" s="65" t="s">
+        <v>44</v>
+      </c>
+      <c r="CD8" s="65" t="s">
+        <v>44</v>
+      </c>
+      <c r="CE8" s="89" t="s">
+        <v>44</v>
+      </c>
+      <c r="CF8" s="92"/>
+      <c r="CG8" s="92"/>
+      <c r="CH8" s="93"/>
       <c r="CI8" s="17" t="s">
         <v>42</v>
       </c>
-      <c r="CJ8" s="38" t="s">
-        <v>44</v>
-      </c>
-      <c r="CK8" s="38" t="s">
-        <v>44</v>
-      </c>
-      <c r="CL8" s="38" t="s">
-        <v>44</v>
-      </c>
-      <c r="CM8" s="38" t="s">
-        <v>44</v>
-      </c>
-      <c r="CN8" s="38" t="s">
-        <v>44</v>
-      </c>
-      <c r="CO8" s="38" t="s">
-        <v>44</v>
-      </c>
-      <c r="CP8" s="38" t="s">
+      <c r="CJ8" s="65" t="s">
+        <v>44</v>
+      </c>
+      <c r="CK8" s="65" t="s">
+        <v>44</v>
+      </c>
+      <c r="CL8" s="65" t="s">
+        <v>44</v>
+      </c>
+      <c r="CM8" s="65" t="s">
+        <v>44</v>
+      </c>
+      <c r="CN8" s="65" t="s">
+        <v>44</v>
+      </c>
+      <c r="CO8" s="65" t="s">
+        <v>44</v>
+      </c>
+      <c r="CP8" s="65" t="s">
         <v>44</v>
       </c>
     </row>
     <row r="9" spans="1:94" s="2" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="59"/>
-      <c r="B9" s="50"/>
-      <c r="C9" s="55"/>
-      <c r="D9" s="92"/>
-      <c r="E9" s="38"/>
-      <c r="F9" s="38"/>
-      <c r="G9" s="38"/>
-      <c r="H9" s="38"/>
-      <c r="I9" s="38"/>
-      <c r="J9" s="38"/>
-      <c r="K9" s="38"/>
-      <c r="L9" s="38"/>
-      <c r="M9" s="38"/>
-      <c r="N9" s="38"/>
-      <c r="O9" s="57"/>
-      <c r="P9" s="38"/>
-      <c r="Q9" s="38"/>
-      <c r="R9" s="38"/>
-      <c r="S9" s="38"/>
-      <c r="T9" s="38"/>
-      <c r="U9" s="38"/>
-      <c r="V9" s="38"/>
-      <c r="W9" s="38"/>
-      <c r="X9" s="38"/>
-      <c r="Y9" s="38"/>
+      <c r="A9" s="48"/>
+      <c r="B9" s="51"/>
+      <c r="C9" s="59"/>
+      <c r="D9" s="63"/>
+      <c r="E9" s="65"/>
+      <c r="F9" s="65"/>
+      <c r="G9" s="65"/>
+      <c r="H9" s="65"/>
+      <c r="I9" s="65"/>
+      <c r="J9" s="65"/>
+      <c r="K9" s="65"/>
+      <c r="L9" s="65"/>
+      <c r="M9" s="65"/>
+      <c r="N9" s="65"/>
+      <c r="O9" s="100"/>
+      <c r="P9" s="65"/>
+      <c r="Q9" s="65"/>
+      <c r="R9" s="65"/>
+      <c r="S9" s="65"/>
+      <c r="T9" s="65"/>
+      <c r="U9" s="65"/>
+      <c r="V9" s="65"/>
+      <c r="W9" s="65"/>
+      <c r="X9" s="65"/>
+      <c r="Y9" s="65"/>
       <c r="Z9" s="18" t="s">
         <v>44</v>
       </c>
       <c r="AA9" s="18" t="s">
         <v>44</v>
       </c>
-      <c r="AB9" s="38"/>
-      <c r="AC9" s="38"/>
-      <c r="AD9" s="38"/>
-      <c r="AE9" s="38"/>
+      <c r="AB9" s="65"/>
+      <c r="AC9" s="65"/>
+      <c r="AD9" s="65"/>
+      <c r="AE9" s="65"/>
       <c r="AF9" s="18" t="s">
         <v>44</v>
       </c>
       <c r="AG9" s="18" t="s">
         <v>44</v>
       </c>
-      <c r="AH9" s="42" t="s">
-        <v>44</v>
-      </c>
-      <c r="AI9" s="55"/>
-      <c r="AJ9" s="38"/>
-      <c r="AK9" s="48"/>
-      <c r="AL9" s="55"/>
-      <c r="AM9" s="38"/>
-      <c r="AN9" s="48"/>
-      <c r="AO9" s="40"/>
-      <c r="AP9" s="38"/>
-      <c r="AQ9" s="50"/>
-      <c r="AR9" s="40"/>
-      <c r="AS9" s="38"/>
-      <c r="AT9" s="38"/>
-      <c r="AU9" s="38"/>
+      <c r="AH9" s="89" t="s">
+        <v>44</v>
+      </c>
+      <c r="AI9" s="59"/>
+      <c r="AJ9" s="65"/>
+      <c r="AK9" s="98"/>
+      <c r="AL9" s="59"/>
+      <c r="AM9" s="65"/>
+      <c r="AN9" s="98"/>
+      <c r="AO9" s="97"/>
+      <c r="AP9" s="65"/>
+      <c r="AQ9" s="51"/>
+      <c r="AR9" s="97"/>
+      <c r="AS9" s="65"/>
+      <c r="AT9" s="65"/>
+      <c r="AU9" s="65"/>
       <c r="AV9" s="18" t="s">
         <v>44</v>
       </c>
       <c r="AW9" s="18" t="s">
         <v>44</v>
       </c>
-      <c r="AX9" s="38"/>
-      <c r="AY9" s="38"/>
-      <c r="AZ9" s="38"/>
-      <c r="BA9" s="38"/>
+      <c r="AX9" s="65"/>
+      <c r="AY9" s="65"/>
+      <c r="AZ9" s="65"/>
+      <c r="BA9" s="65"/>
       <c r="BB9" s="18" t="s">
         <v>44</v>
       </c>
       <c r="BC9" s="18" t="s">
         <v>44</v>
       </c>
-      <c r="BD9" s="38"/>
-      <c r="BE9" s="38"/>
-      <c r="BF9" s="38"/>
-      <c r="BG9" s="51" t="s">
-        <v>44</v>
-      </c>
-      <c r="BH9" s="59"/>
-      <c r="BI9" s="38"/>
-      <c r="BJ9" s="38"/>
-      <c r="BK9" s="44"/>
-      <c r="BL9" s="45"/>
-      <c r="BM9" s="45"/>
-      <c r="BN9" s="46"/>
-      <c r="BO9" s="38"/>
+      <c r="BD9" s="65"/>
+      <c r="BE9" s="65"/>
+      <c r="BF9" s="65"/>
+      <c r="BG9" s="52" t="s">
+        <v>44</v>
+      </c>
+      <c r="BH9" s="48"/>
+      <c r="BI9" s="65"/>
+      <c r="BJ9" s="65"/>
+      <c r="BK9" s="90"/>
+      <c r="BL9" s="94"/>
+      <c r="BM9" s="94"/>
+      <c r="BN9" s="95"/>
+      <c r="BO9" s="65"/>
       <c r="BP9" s="18" t="s">
         <v>44</v>
       </c>
       <c r="BQ9" s="18" t="s">
         <v>44</v>
       </c>
-      <c r="BR9" s="38"/>
-      <c r="BS9" s="38"/>
-      <c r="BT9" s="38"/>
-      <c r="BU9" s="38"/>
-      <c r="BV9" s="44"/>
-      <c r="BW9" s="45"/>
-      <c r="BX9" s="45"/>
-      <c r="BY9" s="46"/>
+      <c r="BR9" s="65"/>
+      <c r="BS9" s="65"/>
+      <c r="BT9" s="65"/>
+      <c r="BU9" s="65"/>
+      <c r="BV9" s="90"/>
+      <c r="BW9" s="94"/>
+      <c r="BX9" s="94"/>
+      <c r="BY9" s="95"/>
       <c r="BZ9" s="18" t="s">
         <v>44</v>
       </c>
       <c r="CA9" s="18" t="s">
         <v>44</v>
       </c>
-      <c r="CB9" s="38"/>
-      <c r="CC9" s="38"/>
-      <c r="CD9" s="38"/>
-      <c r="CE9" s="44"/>
-      <c r="CF9" s="45"/>
-      <c r="CG9" s="45"/>
-      <c r="CH9" s="46"/>
-      <c r="CI9" s="51" t="s">
-        <v>44</v>
-      </c>
-      <c r="CJ9" s="38"/>
-      <c r="CK9" s="38"/>
-      <c r="CL9" s="38"/>
-      <c r="CM9" s="38"/>
-      <c r="CN9" s="38"/>
-      <c r="CO9" s="38"/>
-      <c r="CP9" s="38"/>
+      <c r="CB9" s="65"/>
+      <c r="CC9" s="65"/>
+      <c r="CD9" s="65"/>
+      <c r="CE9" s="90"/>
+      <c r="CF9" s="94"/>
+      <c r="CG9" s="94"/>
+      <c r="CH9" s="95"/>
+      <c r="CI9" s="52" t="s">
+        <v>44</v>
+      </c>
+      <c r="CJ9" s="65"/>
+      <c r="CK9" s="65"/>
+      <c r="CL9" s="65"/>
+      <c r="CM9" s="65"/>
+      <c r="CN9" s="65"/>
+      <c r="CO9" s="65"/>
+      <c r="CP9" s="65"/>
     </row>
     <row r="10" spans="1:94" s="2" customFormat="1" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="60"/>
-      <c r="B10" s="51"/>
-      <c r="C10" s="56"/>
-      <c r="D10" s="93"/>
-      <c r="E10" s="39"/>
-      <c r="F10" s="39"/>
-      <c r="G10" s="39"/>
-      <c r="H10" s="39"/>
-      <c r="I10" s="39"/>
-      <c r="J10" s="39"/>
-      <c r="K10" s="39"/>
-      <c r="L10" s="39"/>
-      <c r="M10" s="39"/>
-      <c r="N10" s="39"/>
-      <c r="O10" s="57"/>
-      <c r="P10" s="39"/>
-      <c r="Q10" s="39"/>
-      <c r="R10" s="39"/>
-      <c r="S10" s="39"/>
-      <c r="T10" s="39"/>
-      <c r="U10" s="39"/>
-      <c r="V10" s="39"/>
-      <c r="W10" s="39"/>
-      <c r="X10" s="39"/>
-      <c r="Y10" s="39"/>
+      <c r="A10" s="49"/>
+      <c r="B10" s="52"/>
+      <c r="C10" s="60"/>
+      <c r="D10" s="64"/>
+      <c r="E10" s="66"/>
+      <c r="F10" s="66"/>
+      <c r="G10" s="66"/>
+      <c r="H10" s="66"/>
+      <c r="I10" s="66"/>
+      <c r="J10" s="66"/>
+      <c r="K10" s="66"/>
+      <c r="L10" s="66"/>
+      <c r="M10" s="66"/>
+      <c r="N10" s="66"/>
+      <c r="O10" s="100"/>
+      <c r="P10" s="66"/>
+      <c r="Q10" s="66"/>
+      <c r="R10" s="66"/>
+      <c r="S10" s="66"/>
+      <c r="T10" s="66"/>
+      <c r="U10" s="66"/>
+      <c r="V10" s="66"/>
+      <c r="W10" s="66"/>
+      <c r="X10" s="66"/>
+      <c r="Y10" s="66"/>
       <c r="Z10" s="19" t="s">
         <v>44</v>
       </c>
       <c r="AA10" s="19" t="s">
         <v>38</v>
       </c>
-      <c r="AB10" s="39"/>
-      <c r="AC10" s="39"/>
-      <c r="AD10" s="39"/>
-      <c r="AE10" s="39"/>
+      <c r="AB10" s="66"/>
+      <c r="AC10" s="66"/>
+      <c r="AD10" s="66"/>
+      <c r="AE10" s="66"/>
       <c r="AF10" s="19" t="s">
         <v>44</v>
       </c>
       <c r="AG10" s="19" t="s">
         <v>38</v>
       </c>
-      <c r="AH10" s="44"/>
-      <c r="AI10" s="56"/>
-      <c r="AJ10" s="39"/>
-      <c r="AK10" s="49"/>
-      <c r="AL10" s="56"/>
-      <c r="AM10" s="39"/>
-      <c r="AN10" s="49"/>
-      <c r="AO10" s="41"/>
-      <c r="AP10" s="39"/>
-      <c r="AQ10" s="51"/>
-      <c r="AR10" s="41"/>
-      <c r="AS10" s="39"/>
-      <c r="AT10" s="39"/>
-      <c r="AU10" s="39"/>
+      <c r="AH10" s="90"/>
+      <c r="AI10" s="60"/>
+      <c r="AJ10" s="66"/>
+      <c r="AK10" s="99"/>
+      <c r="AL10" s="60"/>
+      <c r="AM10" s="66"/>
+      <c r="AN10" s="99"/>
+      <c r="AO10" s="93"/>
+      <c r="AP10" s="66"/>
+      <c r="AQ10" s="52"/>
+      <c r="AR10" s="93"/>
+      <c r="AS10" s="66"/>
+      <c r="AT10" s="66"/>
+      <c r="AU10" s="66"/>
       <c r="AV10" s="19" t="s">
         <v>44</v>
       </c>
       <c r="AW10" s="19" t="s">
         <v>38</v>
       </c>
-      <c r="AX10" s="39"/>
-      <c r="AY10" s="39"/>
-      <c r="AZ10" s="39"/>
-      <c r="BA10" s="39"/>
+      <c r="AX10" s="66"/>
+      <c r="AY10" s="66"/>
+      <c r="AZ10" s="66"/>
+      <c r="BA10" s="66"/>
       <c r="BB10" s="19" t="s">
         <v>44</v>
       </c>
       <c r="BC10" s="19" t="s">
         <v>38</v>
       </c>
-      <c r="BD10" s="39"/>
-      <c r="BE10" s="39"/>
-      <c r="BF10" s="39"/>
-      <c r="BG10" s="58"/>
-      <c r="BH10" s="60"/>
-      <c r="BI10" s="39"/>
-      <c r="BJ10" s="39"/>
-      <c r="BK10" s="44"/>
-      <c r="BL10" s="47"/>
-      <c r="BM10" s="47"/>
-      <c r="BN10" s="46"/>
-      <c r="BO10" s="39"/>
+      <c r="BD10" s="66"/>
+      <c r="BE10" s="66"/>
+      <c r="BF10" s="66"/>
+      <c r="BG10" s="91"/>
+      <c r="BH10" s="49"/>
+      <c r="BI10" s="66"/>
+      <c r="BJ10" s="66"/>
+      <c r="BK10" s="90"/>
+      <c r="BL10" s="96"/>
+      <c r="BM10" s="96"/>
+      <c r="BN10" s="95"/>
+      <c r="BO10" s="66"/>
       <c r="BP10" s="19" t="s">
         <v>44</v>
       </c>
       <c r="BQ10" s="19" t="s">
         <v>38</v>
       </c>
-      <c r="BR10" s="39"/>
-      <c r="BS10" s="39"/>
-      <c r="BT10" s="39"/>
-      <c r="BU10" s="39"/>
-      <c r="BV10" s="44"/>
-      <c r="BW10" s="47"/>
-      <c r="BX10" s="47"/>
-      <c r="BY10" s="46"/>
+      <c r="BR10" s="66"/>
+      <c r="BS10" s="66"/>
+      <c r="BT10" s="66"/>
+      <c r="BU10" s="66"/>
+      <c r="BV10" s="90"/>
+      <c r="BW10" s="96"/>
+      <c r="BX10" s="96"/>
+      <c r="BY10" s="95"/>
       <c r="BZ10" s="19" t="s">
         <v>44</v>
       </c>
       <c r="CA10" s="19" t="s">
         <v>38</v>
       </c>
-      <c r="CB10" s="39"/>
-      <c r="CC10" s="39"/>
-      <c r="CD10" s="39"/>
-      <c r="CE10" s="44"/>
-      <c r="CF10" s="47"/>
-      <c r="CG10" s="47"/>
-      <c r="CH10" s="46"/>
-      <c r="CI10" s="58"/>
-      <c r="CJ10" s="39"/>
-      <c r="CK10" s="39"/>
-      <c r="CL10" s="39"/>
-      <c r="CM10" s="39"/>
-      <c r="CN10" s="39"/>
-      <c r="CO10" s="39"/>
-      <c r="CP10" s="39"/>
+      <c r="CB10" s="66"/>
+      <c r="CC10" s="66"/>
+      <c r="CD10" s="66"/>
+      <c r="CE10" s="90"/>
+      <c r="CF10" s="96"/>
+      <c r="CG10" s="96"/>
+      <c r="CH10" s="95"/>
+      <c r="CI10" s="91"/>
+      <c r="CJ10" s="66"/>
+      <c r="CK10" s="66"/>
+      <c r="CL10" s="66"/>
+      <c r="CM10" s="66"/>
+      <c r="CN10" s="66"/>
+      <c r="CO10" s="66"/>
+      <c r="CP10" s="66"/>
     </row>
     <row r="11" spans="1:94" s="1" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A11" s="29" t="s">
@@ -3008,13 +3007,13 @@
       <c r="AB11" s="32" t="s">
         <v>66</v>
       </c>
-      <c r="AC11" s="94" t="s">
+      <c r="AC11" s="38" t="s">
         <v>67</v>
       </c>
-      <c r="AD11" s="94" t="s">
+      <c r="AD11" s="38" t="s">
         <v>68</v>
       </c>
-      <c r="AE11" s="94" t="s">
+      <c r="AE11" s="38" t="s">
         <v>69</v>
       </c>
       <c r="AF11" s="33" t="s">
@@ -3023,7 +3022,7 @@
       <c r="AG11" s="33" t="s">
         <v>120</v>
       </c>
-      <c r="AH11" s="95" t="s">
+      <c r="AH11" s="39" t="s">
         <v>121</v>
       </c>
       <c r="AI11" s="31" t="s">
@@ -3032,7 +3031,7 @@
       <c r="AJ11" s="32" t="s">
         <v>71</v>
       </c>
-      <c r="AK11" s="97" t="s">
+      <c r="AK11" s="41" t="s">
         <v>122</v>
       </c>
       <c r="AL11" s="35" t="s">
@@ -3041,7 +3040,7 @@
       <c r="AM11" s="35" t="s">
         <v>73</v>
       </c>
-      <c r="AN11" s="97" t="s">
+      <c r="AN11" s="41" t="s">
         <v>123</v>
       </c>
       <c r="AO11" s="36" t="s">
@@ -3050,7 +3049,7 @@
       <c r="AP11" s="32" t="s">
         <v>75</v>
       </c>
-      <c r="AQ11" s="97" t="s">
+      <c r="AQ11" s="41" t="s">
         <v>124</v>
       </c>
       <c r="AR11" s="34" t="s">
@@ -3185,7 +3184,7 @@
       <c r="CI11" s="37" t="s">
         <v>136</v>
       </c>
-      <c r="CJ11" s="99" t="s">
+      <c r="CJ11" s="43" t="s">
         <v>107</v>
       </c>
       <c r="CK11" s="33" t="s">
@@ -3307,7 +3306,7 @@
       <c r="AG12" s="24" t="s">
         <v>169</v>
       </c>
-      <c r="AH12" s="96" t="s">
+      <c r="AH12" s="40" t="s">
         <v>170</v>
       </c>
       <c r="AI12" s="22" t="s">
@@ -3316,7 +3315,7 @@
       <c r="AJ12" s="23" t="s">
         <v>172</v>
       </c>
-      <c r="AK12" s="98" t="s">
+      <c r="AK12" s="42" t="s">
         <v>173</v>
       </c>
       <c r="AL12" s="26" t="s">
@@ -3325,7 +3324,7 @@
       <c r="AM12" s="26" t="s">
         <v>175</v>
       </c>
-      <c r="AN12" s="98" t="s">
+      <c r="AN12" s="42" t="s">
         <v>176</v>
       </c>
       <c r="AO12" s="27" t="s">
@@ -3334,7 +3333,7 @@
       <c r="AP12" s="23" t="s">
         <v>178</v>
       </c>
-      <c r="AQ12" s="98" t="s">
+      <c r="AQ12" s="42" t="s">
         <v>179</v>
       </c>
       <c r="AR12" s="25" t="s">
@@ -3469,7 +3468,7 @@
       <c r="CI12" s="28" t="s">
         <v>222</v>
       </c>
-      <c r="CJ12" s="100" t="s">
+      <c r="CJ12" s="44" t="s">
         <v>223</v>
       </c>
       <c r="CK12" s="24" t="s">
@@ -3493,6 +3492,83 @@
     </row>
   </sheetData>
   <mergeCells count="101">
+    <mergeCell ref="CM8:CM10"/>
+    <mergeCell ref="CN8:CN10"/>
+    <mergeCell ref="CB8:CB10"/>
+    <mergeCell ref="BO8:BO10"/>
+    <mergeCell ref="CO8:CO10"/>
+    <mergeCell ref="AR8:AR10"/>
+    <mergeCell ref="AS8:AS10"/>
+    <mergeCell ref="AT8:AT10"/>
+    <mergeCell ref="AU8:AU10"/>
+    <mergeCell ref="AX8:AX10"/>
+    <mergeCell ref="AY8:AY10"/>
+    <mergeCell ref="AZ8:AZ10"/>
+    <mergeCell ref="BA8:BA10"/>
+    <mergeCell ref="BD8:BD10"/>
+    <mergeCell ref="BJ8:BJ10"/>
+    <mergeCell ref="BK8:BN10"/>
+    <mergeCell ref="AQ8:AQ10"/>
+    <mergeCell ref="AL7:AN7"/>
+    <mergeCell ref="AL8:AL10"/>
+    <mergeCell ref="AM8:AM10"/>
+    <mergeCell ref="AN8:AN10"/>
+    <mergeCell ref="O8:O10"/>
+    <mergeCell ref="P8:P10"/>
+    <mergeCell ref="Q8:Q10"/>
+    <mergeCell ref="R8:R10"/>
+    <mergeCell ref="S8:S10"/>
+    <mergeCell ref="T8:T10"/>
+    <mergeCell ref="V8:V10"/>
+    <mergeCell ref="W8:W10"/>
+    <mergeCell ref="X8:X10"/>
+    <mergeCell ref="Y8:Y10"/>
+    <mergeCell ref="AB8:AB10"/>
+    <mergeCell ref="AC8:AC10"/>
+    <mergeCell ref="AD8:AD10"/>
+    <mergeCell ref="AE8:AE10"/>
+    <mergeCell ref="CP8:CP10"/>
+    <mergeCell ref="AH9:AH10"/>
+    <mergeCell ref="BG9:BG10"/>
+    <mergeCell ref="CI9:CI10"/>
+    <mergeCell ref="CC8:CC10"/>
+    <mergeCell ref="CD8:CD10"/>
+    <mergeCell ref="CE8:CH10"/>
+    <mergeCell ref="CJ8:CJ10"/>
+    <mergeCell ref="CK8:CK10"/>
+    <mergeCell ref="CL8:CL10"/>
+    <mergeCell ref="BR8:BR10"/>
+    <mergeCell ref="BS8:BS10"/>
+    <mergeCell ref="BT8:BT10"/>
+    <mergeCell ref="BU8:BU10"/>
+    <mergeCell ref="BV8:BY10"/>
+    <mergeCell ref="BF8:BF10"/>
+    <mergeCell ref="BH8:BH10"/>
+    <mergeCell ref="BI8:BI10"/>
+    <mergeCell ref="AO8:AO10"/>
+    <mergeCell ref="AI8:AI10"/>
+    <mergeCell ref="AJ8:AJ10"/>
+    <mergeCell ref="AK8:AK10"/>
+    <mergeCell ref="BE8:BE10"/>
+    <mergeCell ref="AP8:AP10"/>
+    <mergeCell ref="AI5:AK5"/>
+    <mergeCell ref="AO5:AQ5"/>
+    <mergeCell ref="AR5:BG5"/>
+    <mergeCell ref="BH5:CI5"/>
+    <mergeCell ref="CJ5:CO5"/>
+    <mergeCell ref="AL5:AN5"/>
+    <mergeCell ref="CP5:CP7"/>
+    <mergeCell ref="AR6:AX6"/>
+    <mergeCell ref="AY6:BC6"/>
+    <mergeCell ref="BD6:BF6"/>
+    <mergeCell ref="BH6:BR6"/>
+    <mergeCell ref="CO6:CO7"/>
+    <mergeCell ref="CJ6:CJ7"/>
+    <mergeCell ref="CK6:CN6"/>
+    <mergeCell ref="AI7:AK7"/>
+    <mergeCell ref="AO7:AQ7"/>
+    <mergeCell ref="BS6:CA6"/>
+    <mergeCell ref="CB6:CI6"/>
     <mergeCell ref="B1:AA1"/>
     <mergeCell ref="B2:AA2"/>
     <mergeCell ref="M3:P3"/>
@@ -3517,83 +3593,6 @@
     <mergeCell ref="L8:L10"/>
     <mergeCell ref="M8:M10"/>
     <mergeCell ref="N8:N10"/>
-    <mergeCell ref="AI5:AK5"/>
-    <mergeCell ref="AO5:AQ5"/>
-    <mergeCell ref="AR5:BG5"/>
-    <mergeCell ref="BH5:CI5"/>
-    <mergeCell ref="CJ5:CO5"/>
-    <mergeCell ref="AL5:AN5"/>
-    <mergeCell ref="CP5:CP7"/>
-    <mergeCell ref="AR6:AX6"/>
-    <mergeCell ref="AY6:BC6"/>
-    <mergeCell ref="BD6:BF6"/>
-    <mergeCell ref="BH6:BR6"/>
-    <mergeCell ref="CO6:CO7"/>
-    <mergeCell ref="CJ6:CJ7"/>
-    <mergeCell ref="CK6:CN6"/>
-    <mergeCell ref="AI7:AK7"/>
-    <mergeCell ref="AO7:AQ7"/>
-    <mergeCell ref="BS6:CA6"/>
-    <mergeCell ref="CB6:CI6"/>
-    <mergeCell ref="CP8:CP10"/>
-    <mergeCell ref="AH9:AH10"/>
-    <mergeCell ref="BG9:BG10"/>
-    <mergeCell ref="CI9:CI10"/>
-    <mergeCell ref="CC8:CC10"/>
-    <mergeCell ref="CD8:CD10"/>
-    <mergeCell ref="CE8:CH10"/>
-    <mergeCell ref="CJ8:CJ10"/>
-    <mergeCell ref="CK8:CK10"/>
-    <mergeCell ref="CL8:CL10"/>
-    <mergeCell ref="BR8:BR10"/>
-    <mergeCell ref="BS8:BS10"/>
-    <mergeCell ref="BT8:BT10"/>
-    <mergeCell ref="BU8:BU10"/>
-    <mergeCell ref="BV8:BY10"/>
-    <mergeCell ref="BF8:BF10"/>
-    <mergeCell ref="BH8:BH10"/>
-    <mergeCell ref="BI8:BI10"/>
-    <mergeCell ref="AO8:AO10"/>
-    <mergeCell ref="AI8:AI10"/>
-    <mergeCell ref="AJ8:AJ10"/>
-    <mergeCell ref="AK8:AK10"/>
-    <mergeCell ref="BE8:BE10"/>
-    <mergeCell ref="AP8:AP10"/>
-    <mergeCell ref="AQ8:AQ10"/>
-    <mergeCell ref="AL7:AN7"/>
-    <mergeCell ref="AL8:AL10"/>
-    <mergeCell ref="AM8:AM10"/>
-    <mergeCell ref="AN8:AN10"/>
-    <mergeCell ref="O8:O10"/>
-    <mergeCell ref="P8:P10"/>
-    <mergeCell ref="Q8:Q10"/>
-    <mergeCell ref="R8:R10"/>
-    <mergeCell ref="S8:S10"/>
-    <mergeCell ref="T8:T10"/>
-    <mergeCell ref="V8:V10"/>
-    <mergeCell ref="W8:W10"/>
-    <mergeCell ref="X8:X10"/>
-    <mergeCell ref="Y8:Y10"/>
-    <mergeCell ref="AB8:AB10"/>
-    <mergeCell ref="AC8:AC10"/>
-    <mergeCell ref="AD8:AD10"/>
-    <mergeCell ref="AE8:AE10"/>
-    <mergeCell ref="CM8:CM10"/>
-    <mergeCell ref="CN8:CN10"/>
-    <mergeCell ref="CB8:CB10"/>
-    <mergeCell ref="BO8:BO10"/>
-    <mergeCell ref="CO8:CO10"/>
-    <mergeCell ref="AR8:AR10"/>
-    <mergeCell ref="AS8:AS10"/>
-    <mergeCell ref="AT8:AT10"/>
-    <mergeCell ref="AU8:AU10"/>
-    <mergeCell ref="AX8:AX10"/>
-    <mergeCell ref="AY8:AY10"/>
-    <mergeCell ref="AZ8:AZ10"/>
-    <mergeCell ref="BA8:BA10"/>
-    <mergeCell ref="BD8:BD10"/>
-    <mergeCell ref="BJ8:BJ10"/>
-    <mergeCell ref="BK8:BN10"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
fix 3 form template
</commit_message>
<xml_diff>
--- a/src/main/resources/templates/summaryReportForm3.xlsx
+++ b/src/main/resources/templates/summaryReportForm3.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="21231"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B1FC6157-4E66-41F1-A944-11ED7F5B2839}" xr6:coauthVersionLast="40" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{41264900-ED69-433C-BE6D-F5D0EA465CDE}" xr6:coauthVersionLast="40" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -220,15 +220,6 @@
     <t>$dist_value25</t>
   </si>
   <si>
-    <t>$dist_value26</t>
-  </si>
-  <si>
-    <t>$dist_value28</t>
-  </si>
-  <si>
-    <t>$dist_value29</t>
-  </si>
-  <si>
     <t>$dist_value31</t>
   </si>
   <si>
@@ -719,6 +710,15 @@
   </si>
   <si>
     <t>$cell_year</t>
+  </si>
+  <si>
+    <t>$dist_pdc_value14_value1</t>
+  </si>
+  <si>
+    <t>$dist_pdc_value16_value2</t>
+  </si>
+  <si>
+    <t>$dist_pdc_value17_value3</t>
   </si>
 </sst>
 </file>
@@ -1393,34 +1393,31 @@
     <xf numFmtId="2" fontId="4" fillId="0" borderId="32" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="3" fillId="0" borderId="35" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="3" fillId="0" borderId="34" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="4" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1429,13 +1426,22 @@
     <xf numFmtId="49" fontId="4" fillId="0" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="4" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1444,6 +1450,117 @@
     <xf numFmtId="49" fontId="4" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="49" fontId="4" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1452,123 +1569,6 @@
     </xf>
     <xf numFmtId="49" fontId="4" fillId="0" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="3" fillId="0" borderId="35" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="4" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="3" fillId="0" borderId="34" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1859,181 +1859,181 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:94" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B1" s="93" t="s">
+      <c r="B1" s="47" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="93"/>
-      <c r="D1" s="93"/>
-      <c r="E1" s="93"/>
-      <c r="F1" s="93"/>
-      <c r="G1" s="93"/>
-      <c r="H1" s="93"/>
-      <c r="I1" s="93"/>
-      <c r="J1" s="93"/>
-      <c r="K1" s="93"/>
-      <c r="L1" s="93"/>
-      <c r="M1" s="93"/>
-      <c r="N1" s="93"/>
-      <c r="O1" s="93"/>
-      <c r="P1" s="93"/>
-      <c r="Q1" s="93"/>
-      <c r="R1" s="93"/>
-      <c r="S1" s="93"/>
-      <c r="T1" s="93"/>
-      <c r="U1" s="93"/>
-      <c r="V1" s="93"/>
-      <c r="W1" s="93"/>
-      <c r="X1" s="93"/>
-      <c r="Y1" s="93"/>
-      <c r="Z1" s="93"/>
-      <c r="AA1" s="93"/>
+      <c r="C1" s="47"/>
+      <c r="D1" s="47"/>
+      <c r="E1" s="47"/>
+      <c r="F1" s="47"/>
+      <c r="G1" s="47"/>
+      <c r="H1" s="47"/>
+      <c r="I1" s="47"/>
+      <c r="J1" s="47"/>
+      <c r="K1" s="47"/>
+      <c r="L1" s="47"/>
+      <c r="M1" s="47"/>
+      <c r="N1" s="47"/>
+      <c r="O1" s="47"/>
+      <c r="P1" s="47"/>
+      <c r="Q1" s="47"/>
+      <c r="R1" s="47"/>
+      <c r="S1" s="47"/>
+      <c r="T1" s="47"/>
+      <c r="U1" s="47"/>
+      <c r="V1" s="47"/>
+      <c r="W1" s="47"/>
+      <c r="X1" s="47"/>
+      <c r="Y1" s="47"/>
+      <c r="Z1" s="47"/>
+      <c r="AA1" s="47"/>
     </row>
     <row r="2" spans="1:94" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B2" s="93" t="s">
+      <c r="B2" s="47" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="93"/>
-      <c r="D2" s="93"/>
-      <c r="E2" s="93"/>
-      <c r="F2" s="93"/>
-      <c r="G2" s="93"/>
-      <c r="H2" s="93"/>
-      <c r="I2" s="93"/>
-      <c r="J2" s="93"/>
-      <c r="K2" s="93"/>
-      <c r="L2" s="93"/>
-      <c r="M2" s="93"/>
-      <c r="N2" s="93"/>
-      <c r="O2" s="93"/>
-      <c r="P2" s="93"/>
-      <c r="Q2" s="93"/>
-      <c r="R2" s="93"/>
-      <c r="S2" s="93"/>
-      <c r="T2" s="93"/>
-      <c r="U2" s="93"/>
-      <c r="V2" s="93"/>
-      <c r="W2" s="93"/>
-      <c r="X2" s="93"/>
-      <c r="Y2" s="93"/>
-      <c r="Z2" s="93"/>
-      <c r="AA2" s="93"/>
+      <c r="C2" s="47"/>
+      <c r="D2" s="47"/>
+      <c r="E2" s="47"/>
+      <c r="F2" s="47"/>
+      <c r="G2" s="47"/>
+      <c r="H2" s="47"/>
+      <c r="I2" s="47"/>
+      <c r="J2" s="47"/>
+      <c r="K2" s="47"/>
+      <c r="L2" s="47"/>
+      <c r="M2" s="47"/>
+      <c r="N2" s="47"/>
+      <c r="O2" s="47"/>
+      <c r="P2" s="47"/>
+      <c r="Q2" s="47"/>
+      <c r="R2" s="47"/>
+      <c r="S2" s="47"/>
+      <c r="T2" s="47"/>
+      <c r="U2" s="47"/>
+      <c r="V2" s="47"/>
+      <c r="W2" s="47"/>
+      <c r="X2" s="47"/>
+      <c r="Y2" s="47"/>
+      <c r="Z2" s="47"/>
+      <c r="AA2" s="47"/>
       <c r="AB2" s="3"/>
     </row>
     <row r="3" spans="1:94" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="L3" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="M3" s="94" t="s">
-        <v>231</v>
-      </c>
-      <c r="N3" s="94"/>
-      <c r="O3" s="94"/>
-      <c r="P3" s="94"/>
+      <c r="M3" s="48" t="s">
+        <v>228</v>
+      </c>
+      <c r="N3" s="48"/>
+      <c r="O3" s="48"/>
+      <c r="P3" s="48"/>
     </row>
     <row r="4" spans="1:94" s="2" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="5" spans="1:94" s="2" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="95" t="s">
+      <c r="A5" s="49" t="s">
         <v>3</v>
       </c>
-      <c r="B5" s="96" t="s">
+      <c r="B5" s="52" t="s">
         <v>4</v>
       </c>
-      <c r="C5" s="74" t="s">
+      <c r="C5" s="55" t="s">
         <v>5</v>
       </c>
-      <c r="D5" s="73"/>
-      <c r="E5" s="73"/>
-      <c r="F5" s="73"/>
-      <c r="G5" s="73"/>
-      <c r="H5" s="73"/>
-      <c r="I5" s="73"/>
-      <c r="J5" s="73"/>
-      <c r="K5" s="73"/>
-      <c r="L5" s="73"/>
-      <c r="M5" s="73"/>
-      <c r="N5" s="73"/>
-      <c r="O5" s="73"/>
-      <c r="P5" s="73"/>
-      <c r="Q5" s="73"/>
-      <c r="R5" s="73"/>
-      <c r="S5" s="73"/>
-      <c r="T5" s="73"/>
-      <c r="U5" s="73"/>
-      <c r="V5" s="73"/>
-      <c r="W5" s="73"/>
-      <c r="X5" s="73"/>
-      <c r="Y5" s="73"/>
-      <c r="Z5" s="73"/>
-      <c r="AA5" s="73"/>
-      <c r="AB5" s="73"/>
-      <c r="AC5" s="73"/>
-      <c r="AD5" s="73"/>
-      <c r="AE5" s="73"/>
-      <c r="AF5" s="73"/>
-      <c r="AG5" s="73"/>
-      <c r="AH5" s="73"/>
-      <c r="AI5" s="67" t="s">
+      <c r="D5" s="56"/>
+      <c r="E5" s="56"/>
+      <c r="F5" s="56"/>
+      <c r="G5" s="56"/>
+      <c r="H5" s="56"/>
+      <c r="I5" s="56"/>
+      <c r="J5" s="56"/>
+      <c r="K5" s="56"/>
+      <c r="L5" s="56"/>
+      <c r="M5" s="56"/>
+      <c r="N5" s="56"/>
+      <c r="O5" s="56"/>
+      <c r="P5" s="56"/>
+      <c r="Q5" s="56"/>
+      <c r="R5" s="56"/>
+      <c r="S5" s="56"/>
+      <c r="T5" s="56"/>
+      <c r="U5" s="56"/>
+      <c r="V5" s="56"/>
+      <c r="W5" s="56"/>
+      <c r="X5" s="56"/>
+      <c r="Y5" s="56"/>
+      <c r="Z5" s="56"/>
+      <c r="AA5" s="56"/>
+      <c r="AB5" s="56"/>
+      <c r="AC5" s="56"/>
+      <c r="AD5" s="56"/>
+      <c r="AE5" s="56"/>
+      <c r="AF5" s="56"/>
+      <c r="AG5" s="56"/>
+      <c r="AH5" s="56"/>
+      <c r="AI5" s="69" t="s">
         <v>6</v>
       </c>
-      <c r="AJ5" s="68"/>
-      <c r="AK5" s="69"/>
-      <c r="AL5" s="67" t="s">
+      <c r="AJ5" s="70"/>
+      <c r="AK5" s="71"/>
+      <c r="AL5" s="69" t="s">
         <v>43</v>
       </c>
-      <c r="AM5" s="68"/>
-      <c r="AN5" s="69"/>
-      <c r="AO5" s="70" t="s">
+      <c r="AM5" s="70"/>
+      <c r="AN5" s="71"/>
+      <c r="AO5" s="72" t="s">
         <v>7</v>
       </c>
-      <c r="AP5" s="71"/>
-      <c r="AQ5" s="72"/>
-      <c r="AR5" s="73" t="s">
+      <c r="AP5" s="73"/>
+      <c r="AQ5" s="74"/>
+      <c r="AR5" s="56" t="s">
         <v>8</v>
       </c>
-      <c r="AS5" s="73"/>
-      <c r="AT5" s="73"/>
-      <c r="AU5" s="73"/>
-      <c r="AV5" s="73"/>
-      <c r="AW5" s="73"/>
-      <c r="AX5" s="73"/>
-      <c r="AY5" s="73"/>
-      <c r="AZ5" s="73"/>
-      <c r="BA5" s="73"/>
-      <c r="BB5" s="73"/>
-      <c r="BC5" s="73"/>
-      <c r="BD5" s="73"/>
-      <c r="BE5" s="73"/>
-      <c r="BF5" s="73"/>
-      <c r="BG5" s="73"/>
-      <c r="BH5" s="74" t="s">
+      <c r="AS5" s="56"/>
+      <c r="AT5" s="56"/>
+      <c r="AU5" s="56"/>
+      <c r="AV5" s="56"/>
+      <c r="AW5" s="56"/>
+      <c r="AX5" s="56"/>
+      <c r="AY5" s="56"/>
+      <c r="AZ5" s="56"/>
+      <c r="BA5" s="56"/>
+      <c r="BB5" s="56"/>
+      <c r="BC5" s="56"/>
+      <c r="BD5" s="56"/>
+      <c r="BE5" s="56"/>
+      <c r="BF5" s="56"/>
+      <c r="BG5" s="56"/>
+      <c r="BH5" s="55" t="s">
         <v>9</v>
       </c>
-      <c r="BI5" s="73"/>
-      <c r="BJ5" s="73"/>
-      <c r="BK5" s="73"/>
-      <c r="BL5" s="73"/>
-      <c r="BM5" s="73"/>
-      <c r="BN5" s="73"/>
-      <c r="BO5" s="73"/>
-      <c r="BP5" s="73"/>
-      <c r="BQ5" s="73"/>
-      <c r="BR5" s="73"/>
-      <c r="BS5" s="73"/>
-      <c r="BT5" s="73"/>
-      <c r="BU5" s="73"/>
-      <c r="BV5" s="73"/>
-      <c r="BW5" s="73"/>
-      <c r="BX5" s="73"/>
-      <c r="BY5" s="73"/>
-      <c r="BZ5" s="73"/>
-      <c r="CA5" s="73"/>
-      <c r="CB5" s="73"/>
-      <c r="CC5" s="73"/>
-      <c r="CD5" s="73"/>
-      <c r="CE5" s="73"/>
-      <c r="CF5" s="73"/>
-      <c r="CG5" s="73"/>
-      <c r="CH5" s="73"/>
+      <c r="BI5" s="56"/>
+      <c r="BJ5" s="56"/>
+      <c r="BK5" s="56"/>
+      <c r="BL5" s="56"/>
+      <c r="BM5" s="56"/>
+      <c r="BN5" s="56"/>
+      <c r="BO5" s="56"/>
+      <c r="BP5" s="56"/>
+      <c r="BQ5" s="56"/>
+      <c r="BR5" s="56"/>
+      <c r="BS5" s="56"/>
+      <c r="BT5" s="56"/>
+      <c r="BU5" s="56"/>
+      <c r="BV5" s="56"/>
+      <c r="BW5" s="56"/>
+      <c r="BX5" s="56"/>
+      <c r="BY5" s="56"/>
+      <c r="BZ5" s="56"/>
+      <c r="CA5" s="56"/>
+      <c r="CB5" s="56"/>
+      <c r="CC5" s="56"/>
+      <c r="CD5" s="56"/>
+      <c r="CE5" s="56"/>
+      <c r="CF5" s="56"/>
+      <c r="CG5" s="56"/>
+      <c r="CH5" s="56"/>
       <c r="CI5" s="75"/>
       <c r="CJ5" s="76" t="s">
         <v>10</v>
@@ -2048,46 +2048,46 @@
       </c>
     </row>
     <row r="6" spans="1:94" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="65"/>
-      <c r="B6" s="54"/>
-      <c r="C6" s="97" t="s">
+      <c r="A6" s="50"/>
+      <c r="B6" s="53"/>
+      <c r="C6" s="57" t="s">
         <v>12</v>
       </c>
-      <c r="D6" s="80"/>
-      <c r="E6" s="80"/>
-      <c r="F6" s="80"/>
-      <c r="G6" s="80"/>
-      <c r="H6" s="80"/>
-      <c r="I6" s="80"/>
-      <c r="J6" s="80"/>
-      <c r="K6" s="80"/>
-      <c r="L6" s="80"/>
-      <c r="M6" s="80"/>
-      <c r="N6" s="80"/>
-      <c r="O6" s="80"/>
-      <c r="P6" s="80"/>
-      <c r="Q6" s="86" t="s">
+      <c r="D6" s="58"/>
+      <c r="E6" s="58"/>
+      <c r="F6" s="58"/>
+      <c r="G6" s="58"/>
+      <c r="H6" s="58"/>
+      <c r="I6" s="58"/>
+      <c r="J6" s="58"/>
+      <c r="K6" s="58"/>
+      <c r="L6" s="58"/>
+      <c r="M6" s="58"/>
+      <c r="N6" s="58"/>
+      <c r="O6" s="58"/>
+      <c r="P6" s="58"/>
+      <c r="Q6" s="59" t="s">
         <v>13</v>
       </c>
-      <c r="R6" s="86"/>
-      <c r="S6" s="86"/>
-      <c r="T6" s="86"/>
-      <c r="U6" s="86"/>
-      <c r="V6" s="86"/>
-      <c r="W6" s="86"/>
-      <c r="X6" s="86"/>
-      <c r="Y6" s="86"/>
-      <c r="Z6" s="86"/>
-      <c r="AA6" s="86"/>
-      <c r="AB6" s="86"/>
-      <c r="AC6" s="86" t="s">
+      <c r="R6" s="59"/>
+      <c r="S6" s="59"/>
+      <c r="T6" s="59"/>
+      <c r="U6" s="59"/>
+      <c r="V6" s="59"/>
+      <c r="W6" s="59"/>
+      <c r="X6" s="59"/>
+      <c r="Y6" s="59"/>
+      <c r="Z6" s="59"/>
+      <c r="AA6" s="59"/>
+      <c r="AB6" s="59"/>
+      <c r="AC6" s="59" t="s">
         <v>14</v>
       </c>
-      <c r="AD6" s="86"/>
-      <c r="AE6" s="86"/>
-      <c r="AF6" s="86"/>
-      <c r="AG6" s="86"/>
-      <c r="AH6" s="82"/>
+      <c r="AD6" s="59"/>
+      <c r="AE6" s="59"/>
+      <c r="AF6" s="59"/>
+      <c r="AG6" s="59"/>
+      <c r="AH6" s="60"/>
       <c r="AI6" s="5" t="s">
         <v>12</v>
       </c>
@@ -2115,94 +2115,94 @@
       <c r="AQ6" s="14" t="s">
         <v>15</v>
       </c>
-      <c r="AR6" s="80" t="s">
+      <c r="AR6" s="58" t="s">
         <v>12</v>
       </c>
-      <c r="AS6" s="80"/>
-      <c r="AT6" s="80"/>
-      <c r="AU6" s="80"/>
-      <c r="AV6" s="80"/>
-      <c r="AW6" s="80"/>
-      <c r="AX6" s="81"/>
-      <c r="AY6" s="82" t="s">
+      <c r="AS6" s="58"/>
+      <c r="AT6" s="58"/>
+      <c r="AU6" s="58"/>
+      <c r="AV6" s="58"/>
+      <c r="AW6" s="58"/>
+      <c r="AX6" s="80"/>
+      <c r="AY6" s="60" t="s">
         <v>13</v>
       </c>
-      <c r="AZ6" s="83"/>
-      <c r="BA6" s="83"/>
-      <c r="BB6" s="83"/>
-      <c r="BC6" s="84"/>
-      <c r="BD6" s="82" t="s">
+      <c r="AZ6" s="63"/>
+      <c r="BA6" s="63"/>
+      <c r="BB6" s="63"/>
+      <c r="BC6" s="64"/>
+      <c r="BD6" s="60" t="s">
         <v>14</v>
       </c>
-      <c r="BE6" s="83"/>
-      <c r="BF6" s="83"/>
+      <c r="BE6" s="63"/>
+      <c r="BF6" s="63"/>
       <c r="BG6" s="6"/>
-      <c r="BH6" s="85" t="s">
+      <c r="BH6" s="81" t="s">
         <v>12</v>
       </c>
-      <c r="BI6" s="83"/>
-      <c r="BJ6" s="83"/>
-      <c r="BK6" s="83"/>
-      <c r="BL6" s="83"/>
-      <c r="BM6" s="83"/>
-      <c r="BN6" s="83"/>
-      <c r="BO6" s="83"/>
-      <c r="BP6" s="83"/>
-      <c r="BQ6" s="83"/>
-      <c r="BR6" s="84"/>
-      <c r="BS6" s="86" t="s">
+      <c r="BI6" s="63"/>
+      <c r="BJ6" s="63"/>
+      <c r="BK6" s="63"/>
+      <c r="BL6" s="63"/>
+      <c r="BM6" s="63"/>
+      <c r="BN6" s="63"/>
+      <c r="BO6" s="63"/>
+      <c r="BP6" s="63"/>
+      <c r="BQ6" s="63"/>
+      <c r="BR6" s="64"/>
+      <c r="BS6" s="59" t="s">
         <v>13</v>
       </c>
-      <c r="BT6" s="86"/>
-      <c r="BU6" s="86"/>
-      <c r="BV6" s="86"/>
-      <c r="BW6" s="86"/>
-      <c r="BX6" s="86"/>
-      <c r="BY6" s="86"/>
-      <c r="BZ6" s="86"/>
-      <c r="CA6" s="86"/>
-      <c r="CB6" s="86" t="s">
+      <c r="BT6" s="59"/>
+      <c r="BU6" s="59"/>
+      <c r="BV6" s="59"/>
+      <c r="BW6" s="59"/>
+      <c r="BX6" s="59"/>
+      <c r="BY6" s="59"/>
+      <c r="BZ6" s="59"/>
+      <c r="CA6" s="59"/>
+      <c r="CB6" s="59" t="s">
         <v>14</v>
       </c>
-      <c r="CC6" s="86"/>
-      <c r="CD6" s="86"/>
-      <c r="CE6" s="82"/>
-      <c r="CF6" s="82"/>
-      <c r="CG6" s="82"/>
-      <c r="CH6" s="82"/>
-      <c r="CI6" s="92"/>
-      <c r="CJ6" s="87" t="s">
+      <c r="CC6" s="59"/>
+      <c r="CD6" s="59"/>
+      <c r="CE6" s="60"/>
+      <c r="CF6" s="60"/>
+      <c r="CG6" s="60"/>
+      <c r="CH6" s="60"/>
+      <c r="CI6" s="90"/>
+      <c r="CJ6" s="82" t="s">
         <v>16</v>
       </c>
-      <c r="CK6" s="89" t="s">
+      <c r="CK6" s="84" t="s">
         <v>17</v>
       </c>
-      <c r="CL6" s="90"/>
-      <c r="CM6" s="90"/>
-      <c r="CN6" s="91"/>
-      <c r="CO6" s="86" t="s">
+      <c r="CL6" s="85"/>
+      <c r="CM6" s="85"/>
+      <c r="CN6" s="86"/>
+      <c r="CO6" s="59" t="s">
         <v>18</v>
       </c>
       <c r="CP6" s="78"/>
     </row>
     <row r="7" spans="1:94" s="2" customFormat="1" ht="56.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="65"/>
-      <c r="B7" s="54"/>
+      <c r="A7" s="50"/>
+      <c r="B7" s="53"/>
       <c r="C7" s="9" t="s">
         <v>19</v>
       </c>
       <c r="D7" s="8" t="s">
         <v>20</v>
       </c>
-      <c r="E7" s="82" t="s">
+      <c r="E7" s="60" t="s">
         <v>21</v>
       </c>
-      <c r="F7" s="83"/>
-      <c r="G7" s="83"/>
-      <c r="H7" s="83"/>
-      <c r="I7" s="83"/>
-      <c r="J7" s="83"/>
-      <c r="K7" s="84"/>
+      <c r="F7" s="63"/>
+      <c r="G7" s="63"/>
+      <c r="H7" s="63"/>
+      <c r="I7" s="63"/>
+      <c r="J7" s="63"/>
+      <c r="K7" s="64"/>
       <c r="L7" s="8" t="s">
         <v>22</v>
       </c>
@@ -2224,15 +2224,15 @@
       <c r="R7" s="8" t="s">
         <v>20</v>
       </c>
-      <c r="S7" s="82" t="s">
+      <c r="S7" s="60" t="s">
         <v>27</v>
       </c>
-      <c r="T7" s="83"/>
-      <c r="U7" s="83"/>
-      <c r="V7" s="83"/>
-      <c r="W7" s="83"/>
-      <c r="X7" s="83"/>
-      <c r="Y7" s="84"/>
+      <c r="T7" s="63"/>
+      <c r="U7" s="63"/>
+      <c r="V7" s="63"/>
+      <c r="W7" s="63"/>
+      <c r="X7" s="63"/>
+      <c r="Y7" s="64"/>
       <c r="Z7" s="10" t="s">
         <v>24</v>
       </c>
@@ -2260,21 +2260,21 @@
       <c r="AH7" s="15" t="s">
         <v>29</v>
       </c>
-      <c r="AI7" s="56" t="s">
+      <c r="AI7" s="87" t="s">
         <v>27</v>
       </c>
-      <c r="AJ7" s="57"/>
-      <c r="AK7" s="58"/>
-      <c r="AL7" s="56" t="s">
+      <c r="AJ7" s="88"/>
+      <c r="AK7" s="89"/>
+      <c r="AL7" s="87" t="s">
         <v>27</v>
       </c>
-      <c r="AM7" s="57"/>
-      <c r="AN7" s="58"/>
-      <c r="AO7" s="84" t="s">
+      <c r="AM7" s="88"/>
+      <c r="AN7" s="89"/>
+      <c r="AO7" s="64" t="s">
         <v>27</v>
       </c>
-      <c r="AP7" s="86"/>
-      <c r="AQ7" s="92"/>
+      <c r="AP7" s="59"/>
+      <c r="AQ7" s="90"/>
       <c r="AR7" s="7" t="s">
         <v>19</v>
       </c>
@@ -2407,7 +2407,7 @@
       <c r="CI7" s="12" t="s">
         <v>29</v>
       </c>
-      <c r="CJ7" s="88"/>
+      <c r="CJ7" s="83"/>
       <c r="CK7" s="8" t="s">
         <v>34</v>
       </c>
@@ -2420,79 +2420,79 @@
       <c r="CN7" s="8" t="s">
         <v>37</v>
       </c>
-      <c r="CO7" s="86"/>
+      <c r="CO7" s="59"/>
       <c r="CP7" s="79"/>
     </row>
     <row r="8" spans="1:94" s="2" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="65"/>
-      <c r="B8" s="54"/>
-      <c r="C8" s="59" t="s">
+      <c r="A8" s="50"/>
+      <c r="B8" s="53"/>
+      <c r="C8" s="61" t="s">
         <v>38</v>
       </c>
-      <c r="D8" s="98" t="s">
-        <v>232</v>
-      </c>
-      <c r="E8" s="44" t="s">
-        <v>232</v>
-      </c>
-      <c r="F8" s="44" t="s">
+      <c r="D8" s="65" t="s">
+        <v>229</v>
+      </c>
+      <c r="E8" s="67" t="s">
+        <v>229</v>
+      </c>
+      <c r="F8" s="67" t="s">
         <v>35</v>
       </c>
-      <c r="G8" s="44" t="s">
+      <c r="G8" s="67" t="s">
         <v>36</v>
       </c>
-      <c r="H8" s="44" t="s">
+      <c r="H8" s="67" t="s">
         <v>39</v>
       </c>
-      <c r="I8" s="44" t="s">
+      <c r="I8" s="67" t="s">
         <v>40</v>
       </c>
-      <c r="J8" s="44" t="s">
+      <c r="J8" s="67" t="s">
         <v>34</v>
       </c>
-      <c r="K8" s="44" t="s">
+      <c r="K8" s="67" t="s">
         <v>41</v>
       </c>
-      <c r="L8" s="44" t="s">
-        <v>232</v>
-      </c>
-      <c r="M8" s="44" t="s">
-        <v>232</v>
-      </c>
-      <c r="N8" s="44" t="s">
-        <v>232</v>
-      </c>
-      <c r="O8" s="45" t="s">
+      <c r="L8" s="67" t="s">
+        <v>229</v>
+      </c>
+      <c r="M8" s="67" t="s">
+        <v>229</v>
+      </c>
+      <c r="N8" s="67" t="s">
+        <v>229</v>
+      </c>
+      <c r="O8" s="68" t="s">
         <v>42</v>
       </c>
-      <c r="P8" s="44" t="s">
-        <v>232</v>
-      </c>
-      <c r="Q8" s="44" t="s">
+      <c r="P8" s="67" t="s">
+        <v>229</v>
+      </c>
+      <c r="Q8" s="67" t="s">
         <v>38</v>
       </c>
-      <c r="R8" s="44" t="s">
-        <v>232</v>
-      </c>
-      <c r="S8" s="44" t="s">
-        <v>232</v>
-      </c>
-      <c r="T8" s="44" t="s">
+      <c r="R8" s="67" t="s">
+        <v>229</v>
+      </c>
+      <c r="S8" s="67" t="s">
+        <v>229</v>
+      </c>
+      <c r="T8" s="67" t="s">
         <v>35</v>
       </c>
-      <c r="U8" s="44" t="s">
+      <c r="U8" s="67" t="s">
         <v>36</v>
       </c>
-      <c r="V8" s="44" t="s">
+      <c r="V8" s="67" t="s">
         <v>39</v>
       </c>
-      <c r="W8" s="44" t="s">
+      <c r="W8" s="67" t="s">
         <v>40</v>
       </c>
-      <c r="X8" s="44" t="s">
+      <c r="X8" s="67" t="s">
         <v>34</v>
       </c>
-      <c r="Y8" s="44" t="s">
+      <c r="Y8" s="67" t="s">
         <v>41</v>
       </c>
       <c r="Z8" s="16" t="s">
@@ -2501,17 +2501,17 @@
       <c r="AA8" s="16" t="s">
         <v>42</v>
       </c>
-      <c r="AB8" s="44" t="s">
-        <v>232</v>
-      </c>
-      <c r="AC8" s="44" t="s">
+      <c r="AB8" s="67" t="s">
+        <v>229</v>
+      </c>
+      <c r="AC8" s="67" t="s">
         <v>38</v>
       </c>
-      <c r="AD8" s="44" t="s">
-        <v>232</v>
-      </c>
-      <c r="AE8" s="44" t="s">
-        <v>232</v>
+      <c r="AD8" s="67" t="s">
+        <v>229</v>
+      </c>
+      <c r="AE8" s="67" t="s">
+        <v>229</v>
       </c>
       <c r="AF8" s="16" t="s">
         <v>42</v>
@@ -2522,44 +2522,44 @@
       <c r="AH8" s="15" t="s">
         <v>42</v>
       </c>
-      <c r="AI8" s="59" t="s">
-        <v>232</v>
-      </c>
-      <c r="AJ8" s="44" t="s">
-        <v>232</v>
-      </c>
-      <c r="AK8" s="61" t="s">
-        <v>232</v>
-      </c>
-      <c r="AL8" s="59" t="s">
-        <v>232</v>
-      </c>
-      <c r="AM8" s="44" t="s">
-        <v>232</v>
-      </c>
-      <c r="AN8" s="61" t="s">
-        <v>232</v>
-      </c>
-      <c r="AO8" s="46" t="s">
-        <v>232</v>
-      </c>
-      <c r="AP8" s="44" t="s">
-        <v>232</v>
-      </c>
-      <c r="AQ8" s="54" t="s">
-        <v>232</v>
-      </c>
-      <c r="AR8" s="46" t="s">
+      <c r="AI8" s="61" t="s">
+        <v>229</v>
+      </c>
+      <c r="AJ8" s="67" t="s">
+        <v>229</v>
+      </c>
+      <c r="AK8" s="100" t="s">
+        <v>229</v>
+      </c>
+      <c r="AL8" s="61" t="s">
+        <v>229</v>
+      </c>
+      <c r="AM8" s="67" t="s">
+        <v>229</v>
+      </c>
+      <c r="AN8" s="100" t="s">
+        <v>229</v>
+      </c>
+      <c r="AO8" s="99" t="s">
+        <v>229</v>
+      </c>
+      <c r="AP8" s="67" t="s">
+        <v>229</v>
+      </c>
+      <c r="AQ8" s="53" t="s">
+        <v>229</v>
+      </c>
+      <c r="AR8" s="99" t="s">
         <v>38</v>
       </c>
-      <c r="AS8" s="44" t="s">
-        <v>232</v>
-      </c>
-      <c r="AT8" s="44" t="s">
-        <v>232</v>
-      </c>
-      <c r="AU8" s="44" t="s">
-        <v>232</v>
+      <c r="AS8" s="67" t="s">
+        <v>229</v>
+      </c>
+      <c r="AT8" s="67" t="s">
+        <v>229</v>
+      </c>
+      <c r="AU8" s="67" t="s">
+        <v>229</v>
       </c>
       <c r="AV8" s="16" t="s">
         <v>42</v>
@@ -2567,17 +2567,17 @@
       <c r="AW8" s="16" t="s">
         <v>42</v>
       </c>
-      <c r="AX8" s="44" t="s">
-        <v>232</v>
-      </c>
-      <c r="AY8" s="44" t="s">
+      <c r="AX8" s="67" t="s">
+        <v>229</v>
+      </c>
+      <c r="AY8" s="67" t="s">
         <v>38</v>
       </c>
-      <c r="AZ8" s="44" t="s">
-        <v>232</v>
-      </c>
-      <c r="BA8" s="44" t="s">
-        <v>232</v>
+      <c r="AZ8" s="67" t="s">
+        <v>229</v>
+      </c>
+      <c r="BA8" s="67" t="s">
+        <v>229</v>
       </c>
       <c r="BB8" s="16" t="s">
         <v>42</v>
@@ -2585,35 +2585,35 @@
       <c r="BC8" s="16" t="s">
         <v>42</v>
       </c>
-      <c r="BD8" s="44" t="s">
+      <c r="BD8" s="67" t="s">
         <v>38</v>
       </c>
-      <c r="BE8" s="44" t="s">
-        <v>232</v>
-      </c>
-      <c r="BF8" s="44" t="s">
-        <v>232</v>
+      <c r="BE8" s="67" t="s">
+        <v>229</v>
+      </c>
+      <c r="BF8" s="67" t="s">
+        <v>229</v>
       </c>
       <c r="BG8" s="15" t="s">
         <v>42</v>
       </c>
-      <c r="BH8" s="65" t="s">
+      <c r="BH8" s="50" t="s">
         <v>38</v>
       </c>
-      <c r="BI8" s="44" t="s">
-        <v>232</v>
-      </c>
-      <c r="BJ8" s="44" t="s">
-        <v>232</v>
-      </c>
-      <c r="BK8" s="48" t="s">
-        <v>232</v>
-      </c>
-      <c r="BL8" s="49"/>
-      <c r="BM8" s="49"/>
-      <c r="BN8" s="47"/>
-      <c r="BO8" s="44" t="s">
-        <v>232</v>
+      <c r="BI8" s="67" t="s">
+        <v>229</v>
+      </c>
+      <c r="BJ8" s="67" t="s">
+        <v>229</v>
+      </c>
+      <c r="BK8" s="91" t="s">
+        <v>229</v>
+      </c>
+      <c r="BL8" s="94"/>
+      <c r="BM8" s="94"/>
+      <c r="BN8" s="95"/>
+      <c r="BO8" s="67" t="s">
+        <v>229</v>
       </c>
       <c r="BP8" s="16" t="s">
         <v>42</v>
@@ -2621,315 +2621,315 @@
       <c r="BQ8" s="15" t="s">
         <v>42</v>
       </c>
-      <c r="BR8" s="44" t="s">
-        <v>232</v>
-      </c>
-      <c r="BS8" s="44" t="s">
+      <c r="BR8" s="67" t="s">
+        <v>229</v>
+      </c>
+      <c r="BS8" s="67" t="s">
         <v>38</v>
       </c>
-      <c r="BT8" s="44" t="s">
-        <v>232</v>
-      </c>
-      <c r="BU8" s="44" t="s">
-        <v>232</v>
-      </c>
-      <c r="BV8" s="48" t="s">
-        <v>232</v>
-      </c>
-      <c r="BW8" s="49"/>
-      <c r="BX8" s="49"/>
-      <c r="BY8" s="47"/>
+      <c r="BT8" s="67" t="s">
+        <v>229</v>
+      </c>
+      <c r="BU8" s="67" t="s">
+        <v>229</v>
+      </c>
+      <c r="BV8" s="91" t="s">
+        <v>229</v>
+      </c>
+      <c r="BW8" s="94"/>
+      <c r="BX8" s="94"/>
+      <c r="BY8" s="95"/>
       <c r="BZ8" s="16" t="s">
         <v>42</v>
       </c>
       <c r="CA8" s="16" t="s">
         <v>42</v>
       </c>
-      <c r="CB8" s="44" t="s">
+      <c r="CB8" s="67" t="s">
         <v>38</v>
       </c>
-      <c r="CC8" s="44" t="s">
-        <v>232</v>
-      </c>
-      <c r="CD8" s="44" t="s">
-        <v>232</v>
-      </c>
-      <c r="CE8" s="48" t="s">
-        <v>232</v>
-      </c>
-      <c r="CF8" s="49"/>
-      <c r="CG8" s="49"/>
-      <c r="CH8" s="47"/>
+      <c r="CC8" s="67" t="s">
+        <v>229</v>
+      </c>
+      <c r="CD8" s="67" t="s">
+        <v>229</v>
+      </c>
+      <c r="CE8" s="91" t="s">
+        <v>229</v>
+      </c>
+      <c r="CF8" s="94"/>
+      <c r="CG8" s="94"/>
+      <c r="CH8" s="95"/>
       <c r="CI8" s="17" t="s">
         <v>42</v>
       </c>
-      <c r="CJ8" s="44" t="s">
-        <v>232</v>
-      </c>
-      <c r="CK8" s="44" t="s">
-        <v>232</v>
-      </c>
-      <c r="CL8" s="44" t="s">
-        <v>232</v>
-      </c>
-      <c r="CM8" s="44" t="s">
-        <v>232</v>
-      </c>
-      <c r="CN8" s="44" t="s">
-        <v>232</v>
-      </c>
-      <c r="CO8" s="44" t="s">
-        <v>232</v>
-      </c>
-      <c r="CP8" s="44" t="s">
-        <v>232</v>
+      <c r="CJ8" s="67" t="s">
+        <v>229</v>
+      </c>
+      <c r="CK8" s="67" t="s">
+        <v>229</v>
+      </c>
+      <c r="CL8" s="67" t="s">
+        <v>229</v>
+      </c>
+      <c r="CM8" s="67" t="s">
+        <v>229</v>
+      </c>
+      <c r="CN8" s="67" t="s">
+        <v>229</v>
+      </c>
+      <c r="CO8" s="67" t="s">
+        <v>229</v>
+      </c>
+      <c r="CP8" s="67" t="s">
+        <v>229</v>
       </c>
     </row>
     <row r="9" spans="1:94" s="2" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="65"/>
-      <c r="B9" s="54"/>
-      <c r="C9" s="59"/>
-      <c r="D9" s="98"/>
-      <c r="E9" s="44"/>
-      <c r="F9" s="44"/>
-      <c r="G9" s="44"/>
-      <c r="H9" s="44"/>
-      <c r="I9" s="44"/>
-      <c r="J9" s="44"/>
-      <c r="K9" s="44"/>
-      <c r="L9" s="44"/>
-      <c r="M9" s="44"/>
-      <c r="N9" s="44"/>
-      <c r="O9" s="63"/>
-      <c r="P9" s="44"/>
-      <c r="Q9" s="44"/>
-      <c r="R9" s="44"/>
-      <c r="S9" s="44"/>
-      <c r="T9" s="44"/>
-      <c r="U9" s="44"/>
-      <c r="V9" s="44"/>
-      <c r="W9" s="44"/>
-      <c r="X9" s="44"/>
-      <c r="Y9" s="44"/>
+      <c r="A9" s="50"/>
+      <c r="B9" s="53"/>
+      <c r="C9" s="61"/>
+      <c r="D9" s="65"/>
+      <c r="E9" s="67"/>
+      <c r="F9" s="67"/>
+      <c r="G9" s="67"/>
+      <c r="H9" s="67"/>
+      <c r="I9" s="67"/>
+      <c r="J9" s="67"/>
+      <c r="K9" s="67"/>
+      <c r="L9" s="67"/>
+      <c r="M9" s="67"/>
+      <c r="N9" s="67"/>
+      <c r="O9" s="102"/>
+      <c r="P9" s="67"/>
+      <c r="Q9" s="67"/>
+      <c r="R9" s="67"/>
+      <c r="S9" s="67"/>
+      <c r="T9" s="67"/>
+      <c r="U9" s="67"/>
+      <c r="V9" s="67"/>
+      <c r="W9" s="67"/>
+      <c r="X9" s="67"/>
+      <c r="Y9" s="67"/>
       <c r="Z9" s="18" t="s">
-        <v>232</v>
+        <v>229</v>
       </c>
       <c r="AA9" s="18" t="s">
-        <v>232</v>
-      </c>
-      <c r="AB9" s="44"/>
-      <c r="AC9" s="44"/>
-      <c r="AD9" s="44"/>
-      <c r="AE9" s="44"/>
+        <v>229</v>
+      </c>
+      <c r="AB9" s="67"/>
+      <c r="AC9" s="67"/>
+      <c r="AD9" s="67"/>
+      <c r="AE9" s="67"/>
       <c r="AF9" s="18" t="s">
-        <v>232</v>
+        <v>229</v>
       </c>
       <c r="AG9" s="18" t="s">
-        <v>232</v>
-      </c>
-      <c r="AH9" s="48" t="s">
-        <v>232</v>
-      </c>
-      <c r="AI9" s="59"/>
-      <c r="AJ9" s="44"/>
-      <c r="AK9" s="61"/>
-      <c r="AL9" s="59"/>
-      <c r="AM9" s="44"/>
-      <c r="AN9" s="61"/>
-      <c r="AO9" s="46"/>
-      <c r="AP9" s="44"/>
-      <c r="AQ9" s="54"/>
-      <c r="AR9" s="46"/>
-      <c r="AS9" s="44"/>
-      <c r="AT9" s="44"/>
-      <c r="AU9" s="44"/>
+        <v>229</v>
+      </c>
+      <c r="AH9" s="91" t="s">
+        <v>229</v>
+      </c>
+      <c r="AI9" s="61"/>
+      <c r="AJ9" s="67"/>
+      <c r="AK9" s="100"/>
+      <c r="AL9" s="61"/>
+      <c r="AM9" s="67"/>
+      <c r="AN9" s="100"/>
+      <c r="AO9" s="99"/>
+      <c r="AP9" s="67"/>
+      <c r="AQ9" s="53"/>
+      <c r="AR9" s="99"/>
+      <c r="AS9" s="67"/>
+      <c r="AT9" s="67"/>
+      <c r="AU9" s="67"/>
       <c r="AV9" s="18" t="s">
-        <v>232</v>
+        <v>229</v>
       </c>
       <c r="AW9" s="18" t="s">
-        <v>232</v>
-      </c>
-      <c r="AX9" s="44"/>
-      <c r="AY9" s="44"/>
-      <c r="AZ9" s="44"/>
-      <c r="BA9" s="44"/>
+        <v>229</v>
+      </c>
+      <c r="AX9" s="67"/>
+      <c r="AY9" s="67"/>
+      <c r="AZ9" s="67"/>
+      <c r="BA9" s="67"/>
       <c r="BB9" s="18" t="s">
-        <v>232</v>
+        <v>229</v>
       </c>
       <c r="BC9" s="18" t="s">
-        <v>232</v>
-      </c>
-      <c r="BD9" s="44"/>
-      <c r="BE9" s="44"/>
-      <c r="BF9" s="44"/>
-      <c r="BG9" s="55" t="s">
-        <v>232</v>
-      </c>
-      <c r="BH9" s="65"/>
-      <c r="BI9" s="44"/>
-      <c r="BJ9" s="44"/>
-      <c r="BK9" s="50"/>
-      <c r="BL9" s="51"/>
-      <c r="BM9" s="51"/>
-      <c r="BN9" s="52"/>
-      <c r="BO9" s="44"/>
+        <v>229</v>
+      </c>
+      <c r="BD9" s="67"/>
+      <c r="BE9" s="67"/>
+      <c r="BF9" s="67"/>
+      <c r="BG9" s="54" t="s">
+        <v>229</v>
+      </c>
+      <c r="BH9" s="50"/>
+      <c r="BI9" s="67"/>
+      <c r="BJ9" s="67"/>
+      <c r="BK9" s="92"/>
+      <c r="BL9" s="96"/>
+      <c r="BM9" s="96"/>
+      <c r="BN9" s="97"/>
+      <c r="BO9" s="67"/>
       <c r="BP9" s="18" t="s">
-        <v>232</v>
+        <v>229</v>
       </c>
       <c r="BQ9" s="18" t="s">
-        <v>232</v>
-      </c>
-      <c r="BR9" s="44"/>
-      <c r="BS9" s="44"/>
-      <c r="BT9" s="44"/>
-      <c r="BU9" s="44"/>
-      <c r="BV9" s="50"/>
-      <c r="BW9" s="51"/>
-      <c r="BX9" s="51"/>
-      <c r="BY9" s="52"/>
+        <v>229</v>
+      </c>
+      <c r="BR9" s="67"/>
+      <c r="BS9" s="67"/>
+      <c r="BT9" s="67"/>
+      <c r="BU9" s="67"/>
+      <c r="BV9" s="92"/>
+      <c r="BW9" s="96"/>
+      <c r="BX9" s="96"/>
+      <c r="BY9" s="97"/>
       <c r="BZ9" s="18" t="s">
-        <v>232</v>
+        <v>229</v>
       </c>
       <c r="CA9" s="18" t="s">
-        <v>232</v>
-      </c>
-      <c r="CB9" s="44"/>
-      <c r="CC9" s="44"/>
-      <c r="CD9" s="44"/>
-      <c r="CE9" s="50"/>
-      <c r="CF9" s="51"/>
-      <c r="CG9" s="51"/>
-      <c r="CH9" s="52"/>
-      <c r="CI9" s="55" t="s">
-        <v>232</v>
-      </c>
-      <c r="CJ9" s="44"/>
-      <c r="CK9" s="44"/>
-      <c r="CL9" s="44"/>
-      <c r="CM9" s="44"/>
-      <c r="CN9" s="44"/>
-      <c r="CO9" s="44"/>
-      <c r="CP9" s="44"/>
+        <v>229</v>
+      </c>
+      <c r="CB9" s="67"/>
+      <c r="CC9" s="67"/>
+      <c r="CD9" s="67"/>
+      <c r="CE9" s="92"/>
+      <c r="CF9" s="96"/>
+      <c r="CG9" s="96"/>
+      <c r="CH9" s="97"/>
+      <c r="CI9" s="54" t="s">
+        <v>229</v>
+      </c>
+      <c r="CJ9" s="67"/>
+      <c r="CK9" s="67"/>
+      <c r="CL9" s="67"/>
+      <c r="CM9" s="67"/>
+      <c r="CN9" s="67"/>
+      <c r="CO9" s="67"/>
+      <c r="CP9" s="67"/>
     </row>
     <row r="10" spans="1:94" s="2" customFormat="1" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="66"/>
-      <c r="B10" s="55"/>
-      <c r="C10" s="60"/>
-      <c r="D10" s="99"/>
-      <c r="E10" s="45"/>
-      <c r="F10" s="45"/>
-      <c r="G10" s="45"/>
-      <c r="H10" s="45"/>
-      <c r="I10" s="45"/>
-      <c r="J10" s="45"/>
-      <c r="K10" s="45"/>
-      <c r="L10" s="45"/>
-      <c r="M10" s="45"/>
-      <c r="N10" s="45"/>
-      <c r="O10" s="63"/>
-      <c r="P10" s="45"/>
-      <c r="Q10" s="45"/>
-      <c r="R10" s="45"/>
-      <c r="S10" s="45"/>
-      <c r="T10" s="45"/>
-      <c r="U10" s="45"/>
-      <c r="V10" s="45"/>
-      <c r="W10" s="45"/>
-      <c r="X10" s="45"/>
-      <c r="Y10" s="45"/>
+      <c r="A10" s="51"/>
+      <c r="B10" s="54"/>
+      <c r="C10" s="62"/>
+      <c r="D10" s="66"/>
+      <c r="E10" s="68"/>
+      <c r="F10" s="68"/>
+      <c r="G10" s="68"/>
+      <c r="H10" s="68"/>
+      <c r="I10" s="68"/>
+      <c r="J10" s="68"/>
+      <c r="K10" s="68"/>
+      <c r="L10" s="68"/>
+      <c r="M10" s="68"/>
+      <c r="N10" s="68"/>
+      <c r="O10" s="102"/>
+      <c r="P10" s="68"/>
+      <c r="Q10" s="68"/>
+      <c r="R10" s="68"/>
+      <c r="S10" s="68"/>
+      <c r="T10" s="68"/>
+      <c r="U10" s="68"/>
+      <c r="V10" s="68"/>
+      <c r="W10" s="68"/>
+      <c r="X10" s="68"/>
+      <c r="Y10" s="68"/>
       <c r="Z10" s="19" t="s">
-        <v>232</v>
+        <v>229</v>
       </c>
       <c r="AA10" s="19" t="s">
         <v>38</v>
       </c>
-      <c r="AB10" s="45"/>
-      <c r="AC10" s="45"/>
-      <c r="AD10" s="45"/>
-      <c r="AE10" s="45"/>
+      <c r="AB10" s="68"/>
+      <c r="AC10" s="68"/>
+      <c r="AD10" s="68"/>
+      <c r="AE10" s="68"/>
       <c r="AF10" s="19" t="s">
-        <v>232</v>
+        <v>229</v>
       </c>
       <c r="AG10" s="19" t="s">
         <v>38</v>
       </c>
-      <c r="AH10" s="50"/>
-      <c r="AI10" s="60"/>
-      <c r="AJ10" s="45"/>
-      <c r="AK10" s="62"/>
-      <c r="AL10" s="60"/>
-      <c r="AM10" s="45"/>
-      <c r="AN10" s="62"/>
-      <c r="AO10" s="47"/>
-      <c r="AP10" s="45"/>
-      <c r="AQ10" s="55"/>
-      <c r="AR10" s="47"/>
-      <c r="AS10" s="45"/>
-      <c r="AT10" s="45"/>
-      <c r="AU10" s="45"/>
+      <c r="AH10" s="92"/>
+      <c r="AI10" s="62"/>
+      <c r="AJ10" s="68"/>
+      <c r="AK10" s="101"/>
+      <c r="AL10" s="62"/>
+      <c r="AM10" s="68"/>
+      <c r="AN10" s="101"/>
+      <c r="AO10" s="95"/>
+      <c r="AP10" s="68"/>
+      <c r="AQ10" s="54"/>
+      <c r="AR10" s="95"/>
+      <c r="AS10" s="68"/>
+      <c r="AT10" s="68"/>
+      <c r="AU10" s="68"/>
       <c r="AV10" s="19" t="s">
-        <v>232</v>
+        <v>229</v>
       </c>
       <c r="AW10" s="19" t="s">
         <v>38</v>
       </c>
-      <c r="AX10" s="45"/>
-      <c r="AY10" s="45"/>
-      <c r="AZ10" s="45"/>
-      <c r="BA10" s="45"/>
+      <c r="AX10" s="68"/>
+      <c r="AY10" s="68"/>
+      <c r="AZ10" s="68"/>
+      <c r="BA10" s="68"/>
       <c r="BB10" s="19" t="s">
-        <v>232</v>
+        <v>229</v>
       </c>
       <c r="BC10" s="19" t="s">
         <v>38</v>
       </c>
-      <c r="BD10" s="45"/>
-      <c r="BE10" s="45"/>
-      <c r="BF10" s="45"/>
-      <c r="BG10" s="64"/>
-      <c r="BH10" s="66"/>
-      <c r="BI10" s="45"/>
-      <c r="BJ10" s="45"/>
-      <c r="BK10" s="50"/>
-      <c r="BL10" s="53"/>
-      <c r="BM10" s="53"/>
-      <c r="BN10" s="52"/>
-      <c r="BO10" s="45"/>
+      <c r="BD10" s="68"/>
+      <c r="BE10" s="68"/>
+      <c r="BF10" s="68"/>
+      <c r="BG10" s="93"/>
+      <c r="BH10" s="51"/>
+      <c r="BI10" s="68"/>
+      <c r="BJ10" s="68"/>
+      <c r="BK10" s="92"/>
+      <c r="BL10" s="98"/>
+      <c r="BM10" s="98"/>
+      <c r="BN10" s="97"/>
+      <c r="BO10" s="68"/>
       <c r="BP10" s="19" t="s">
-        <v>232</v>
+        <v>229</v>
       </c>
       <c r="BQ10" s="19" t="s">
         <v>38</v>
       </c>
-      <c r="BR10" s="45"/>
-      <c r="BS10" s="45"/>
-      <c r="BT10" s="45"/>
-      <c r="BU10" s="45"/>
-      <c r="BV10" s="50"/>
-      <c r="BW10" s="53"/>
-      <c r="BX10" s="53"/>
-      <c r="BY10" s="52"/>
+      <c r="BR10" s="68"/>
+      <c r="BS10" s="68"/>
+      <c r="BT10" s="68"/>
+      <c r="BU10" s="68"/>
+      <c r="BV10" s="92"/>
+      <c r="BW10" s="98"/>
+      <c r="BX10" s="98"/>
+      <c r="BY10" s="97"/>
       <c r="BZ10" s="19" t="s">
-        <v>232</v>
+        <v>229</v>
       </c>
       <c r="CA10" s="19" t="s">
         <v>38</v>
       </c>
-      <c r="CB10" s="45"/>
-      <c r="CC10" s="45"/>
-      <c r="CD10" s="45"/>
-      <c r="CE10" s="50"/>
-      <c r="CF10" s="53"/>
-      <c r="CG10" s="53"/>
-      <c r="CH10" s="52"/>
-      <c r="CI10" s="64"/>
-      <c r="CJ10" s="45"/>
-      <c r="CK10" s="45"/>
-      <c r="CL10" s="45"/>
-      <c r="CM10" s="45"/>
-      <c r="CN10" s="45"/>
-      <c r="CO10" s="45"/>
-      <c r="CP10" s="45"/>
+      <c r="CB10" s="68"/>
+      <c r="CC10" s="68"/>
+      <c r="CD10" s="68"/>
+      <c r="CE10" s="92"/>
+      <c r="CF10" s="98"/>
+      <c r="CG10" s="98"/>
+      <c r="CH10" s="97"/>
+      <c r="CI10" s="93"/>
+      <c r="CJ10" s="68"/>
+      <c r="CK10" s="68"/>
+      <c r="CL10" s="68"/>
+      <c r="CM10" s="68"/>
+      <c r="CN10" s="68"/>
+      <c r="CO10" s="68"/>
+      <c r="CP10" s="68"/>
     </row>
     <row r="11" spans="1:94" s="1" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A11" s="29" t="s">
@@ -2970,13 +2970,13 @@
         <v>55</v>
       </c>
       <c r="N11" s="33" t="s">
-        <v>113</v>
+        <v>110</v>
       </c>
       <c r="O11" s="33" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
       <c r="P11" s="32" t="s">
-        <v>115</v>
+        <v>112</v>
       </c>
       <c r="Q11" s="32" t="s">
         <v>56</v>
@@ -3006,499 +3006,576 @@
         <v>64</v>
       </c>
       <c r="Z11" s="33" t="s">
-        <v>116</v>
+        <v>113</v>
       </c>
       <c r="AA11" s="33" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="AB11" s="32" t="s">
         <v>65</v>
       </c>
-      <c r="AC11" s="100" t="s">
+      <c r="AC11" s="44" t="s">
+        <v>230</v>
+      </c>
+      <c r="AD11" s="33" t="s">
+        <v>231</v>
+      </c>
+      <c r="AE11" s="33" t="s">
+        <v>232</v>
+      </c>
+      <c r="AF11" s="33" t="s">
+        <v>115</v>
+      </c>
+      <c r="AG11" s="33" t="s">
+        <v>116</v>
+      </c>
+      <c r="AH11" s="38" t="s">
+        <v>117</v>
+      </c>
+      <c r="AI11" s="31" t="s">
         <v>66</v>
       </c>
-      <c r="AD11" s="33" t="s">
+      <c r="AJ11" s="32" t="s">
         <v>67</v>
       </c>
-      <c r="AE11" s="33" t="s">
+      <c r="AK11" s="40" t="s">
+        <v>222</v>
+      </c>
+      <c r="AL11" s="35" t="s">
         <v>68</v>
       </c>
-      <c r="AF11" s="33" t="s">
+      <c r="AM11" s="35" t="s">
+        <v>69</v>
+      </c>
+      <c r="AN11" s="40" t="s">
+        <v>223</v>
+      </c>
+      <c r="AO11" s="36" t="s">
+        <v>70</v>
+      </c>
+      <c r="AP11" s="32" t="s">
+        <v>71</v>
+      </c>
+      <c r="AQ11" s="40" t="s">
+        <v>224</v>
+      </c>
+      <c r="AR11" s="34" t="s">
+        <v>72</v>
+      </c>
+      <c r="AS11" s="32" t="s">
+        <v>73</v>
+      </c>
+      <c r="AT11" s="32" t="s">
+        <v>74</v>
+      </c>
+      <c r="AU11" s="32" t="s">
+        <v>75</v>
+      </c>
+      <c r="AV11" s="33" t="s">
         <v>118</v>
       </c>
-      <c r="AG11" s="33" t="s">
+      <c r="AW11" s="33" t="s">
         <v>119</v>
       </c>
-      <c r="AH11" s="38" t="s">
+      <c r="AX11" s="32" t="s">
         <v>120</v>
       </c>
-      <c r="AI11" s="31" t="s">
-        <v>69</v>
-      </c>
-      <c r="AJ11" s="32" t="s">
-        <v>70</v>
-      </c>
-      <c r="AK11" s="40" t="s">
-        <v>225</v>
-      </c>
-      <c r="AL11" s="35" t="s">
-        <v>71</v>
-      </c>
-      <c r="AM11" s="35" t="s">
-        <v>72</v>
-      </c>
-      <c r="AN11" s="40" t="s">
-        <v>226</v>
-      </c>
-      <c r="AO11" s="36" t="s">
-        <v>73</v>
-      </c>
-      <c r="AP11" s="32" t="s">
-        <v>74</v>
-      </c>
-      <c r="AQ11" s="40" t="s">
-        <v>227</v>
-      </c>
-      <c r="AR11" s="34" t="s">
-        <v>75</v>
-      </c>
-      <c r="AS11" s="32" t="s">
+      <c r="AY11" s="32" t="s">
         <v>76</v>
       </c>
-      <c r="AT11" s="32" t="s">
+      <c r="AZ11" s="32" t="s">
         <v>77</v>
       </c>
-      <c r="AU11" s="32" t="s">
+      <c r="BA11" s="32" t="s">
         <v>78</v>
       </c>
-      <c r="AV11" s="33" t="s">
+      <c r="BB11" s="33" t="s">
         <v>121</v>
       </c>
-      <c r="AW11" s="33" t="s">
+      <c r="BC11" s="33" t="s">
         <v>122</v>
       </c>
-      <c r="AX11" s="32" t="s">
+      <c r="BD11" s="32" t="s">
+        <v>79</v>
+      </c>
+      <c r="BE11" s="32" t="s">
+        <v>80</v>
+      </c>
+      <c r="BF11" s="32" t="s">
+        <v>81</v>
+      </c>
+      <c r="BG11" s="35" t="s">
         <v>123</v>
       </c>
-      <c r="AY11" s="32" t="s">
-        <v>79</v>
-      </c>
-      <c r="AZ11" s="32" t="s">
-        <v>80</v>
-      </c>
-      <c r="BA11" s="32" t="s">
-        <v>81</v>
-      </c>
-      <c r="BB11" s="33" t="s">
+      <c r="BH11" s="31" t="s">
+        <v>220</v>
+      </c>
+      <c r="BI11" s="32" t="s">
+        <v>82</v>
+      </c>
+      <c r="BJ11" s="32" t="s">
+        <v>83</v>
+      </c>
+      <c r="BK11" s="32" t="s">
+        <v>84</v>
+      </c>
+      <c r="BL11" s="32" t="s">
+        <v>85</v>
+      </c>
+      <c r="BM11" s="32" t="s">
+        <v>86</v>
+      </c>
+      <c r="BN11" s="32" t="s">
+        <v>87</v>
+      </c>
+      <c r="BO11" s="32" t="s">
+        <v>88</v>
+      </c>
+      <c r="BP11" s="33" t="s">
         <v>124</v>
       </c>
-      <c r="BC11" s="33" t="s">
+      <c r="BQ11" s="33" t="s">
         <v>125</v>
       </c>
-      <c r="BD11" s="32" t="s">
-        <v>82</v>
-      </c>
-      <c r="BE11" s="32" t="s">
-        <v>83</v>
-      </c>
-      <c r="BF11" s="32" t="s">
-        <v>84</v>
-      </c>
-      <c r="BG11" s="35" t="s">
+      <c r="BR11" s="32" t="s">
         <v>126</v>
       </c>
-      <c r="BH11" s="31" t="s">
-        <v>223</v>
-      </c>
-      <c r="BI11" s="32" t="s">
-        <v>85</v>
-      </c>
-      <c r="BJ11" s="32" t="s">
-        <v>86</v>
-      </c>
-      <c r="BK11" s="32" t="s">
-        <v>87</v>
-      </c>
-      <c r="BL11" s="32" t="s">
-        <v>88</v>
-      </c>
-      <c r="BM11" s="32" t="s">
+      <c r="BS11" s="32" t="s">
         <v>89</v>
       </c>
-      <c r="BN11" s="32" t="s">
+      <c r="BT11" s="32" t="s">
         <v>90</v>
       </c>
-      <c r="BO11" s="32" t="s">
+      <c r="BU11" s="32" t="s">
         <v>91</v>
       </c>
-      <c r="BP11" s="33" t="s">
+      <c r="BV11" s="32" t="s">
+        <v>92</v>
+      </c>
+      <c r="BW11" s="32" t="s">
+        <v>93</v>
+      </c>
+      <c r="BX11" s="32" t="s">
+        <v>94</v>
+      </c>
+      <c r="BY11" s="32" t="s">
+        <v>95</v>
+      </c>
+      <c r="BZ11" s="33" t="s">
         <v>127</v>
       </c>
-      <c r="BQ11" s="33" t="s">
+      <c r="CA11" s="33" t="s">
         <v>128</v>
       </c>
-      <c r="BR11" s="32" t="s">
+      <c r="CB11" s="32" t="s">
+        <v>96</v>
+      </c>
+      <c r="CC11" s="32" t="s">
+        <v>97</v>
+      </c>
+      <c r="CD11" s="32" t="s">
+        <v>98</v>
+      </c>
+      <c r="CE11" s="32" t="s">
+        <v>99</v>
+      </c>
+      <c r="CF11" s="32" t="s">
+        <v>100</v>
+      </c>
+      <c r="CG11" s="32" t="s">
+        <v>101</v>
+      </c>
+      <c r="CH11" s="32" t="s">
+        <v>102</v>
+      </c>
+      <c r="CI11" s="37" t="s">
         <v>129</v>
       </c>
-      <c r="BS11" s="32" t="s">
-        <v>92</v>
-      </c>
-      <c r="BT11" s="32" t="s">
-        <v>93</v>
-      </c>
-      <c r="BU11" s="32" t="s">
-        <v>94</v>
-      </c>
-      <c r="BV11" s="32" t="s">
-        <v>95</v>
-      </c>
-      <c r="BW11" s="32" t="s">
-        <v>96</v>
-      </c>
-      <c r="BX11" s="32" t="s">
-        <v>97</v>
-      </c>
-      <c r="BY11" s="32" t="s">
-        <v>98</v>
-      </c>
-      <c r="BZ11" s="33" t="s">
-        <v>130</v>
-      </c>
-      <c r="CA11" s="33" t="s">
-        <v>131</v>
-      </c>
-      <c r="CB11" s="32" t="s">
-        <v>99</v>
-      </c>
-      <c r="CC11" s="32" t="s">
-        <v>100</v>
-      </c>
-      <c r="CD11" s="32" t="s">
-        <v>101</v>
-      </c>
-      <c r="CE11" s="32" t="s">
-        <v>102</v>
-      </c>
-      <c r="CF11" s="32" t="s">
+      <c r="CJ11" s="42" t="s">
         <v>103</v>
       </c>
-      <c r="CG11" s="32" t="s">
+      <c r="CK11" s="33" t="s">
         <v>104</v>
       </c>
-      <c r="CH11" s="32" t="s">
+      <c r="CL11" s="33" t="s">
         <v>105</v>
       </c>
-      <c r="CI11" s="37" t="s">
-        <v>132</v>
-      </c>
-      <c r="CJ11" s="42" t="s">
+      <c r="CM11" s="33" t="s">
         <v>106</v>
       </c>
-      <c r="CK11" s="33" t="s">
+      <c r="CN11" s="33" t="s">
         <v>107</v>
       </c>
-      <c r="CL11" s="33" t="s">
+      <c r="CO11" s="33" t="s">
         <v>108</v>
       </c>
-      <c r="CM11" s="33" t="s">
+      <c r="CP11" s="46" t="s">
         <v>109</v>
-      </c>
-      <c r="CN11" s="33" t="s">
-        <v>110</v>
-      </c>
-      <c r="CO11" s="33" t="s">
-        <v>111</v>
-      </c>
-      <c r="CP11" s="102" t="s">
-        <v>112</v>
       </c>
     </row>
     <row r="12" spans="1:94" s="13" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A12" s="20" t="s">
+        <v>131</v>
+      </c>
+      <c r="B12" s="21" t="s">
+        <v>130</v>
+      </c>
+      <c r="C12" s="22" t="s">
+        <v>132</v>
+      </c>
+      <c r="D12" s="23" t="s">
+        <v>133</v>
+      </c>
+      <c r="E12" s="23" t="s">
         <v>134</v>
       </c>
-      <c r="B12" s="21" t="s">
-        <v>133</v>
-      </c>
-      <c r="C12" s="22" t="s">
+      <c r="F12" s="23" t="s">
         <v>135</v>
       </c>
-      <c r="D12" s="23" t="s">
+      <c r="G12" s="23" t="s">
         <v>136</v>
       </c>
-      <c r="E12" s="23" t="s">
+      <c r="H12" s="23" t="s">
         <v>137</v>
       </c>
-      <c r="F12" s="23" t="s">
+      <c r="I12" s="23" t="s">
         <v>138</v>
       </c>
-      <c r="G12" s="23" t="s">
+      <c r="J12" s="23" t="s">
         <v>139</v>
       </c>
-      <c r="H12" s="23" t="s">
+      <c r="K12" s="23" t="s">
         <v>140</v>
       </c>
-      <c r="I12" s="23" t="s">
+      <c r="L12" s="23" t="s">
         <v>141</v>
       </c>
-      <c r="J12" s="23" t="s">
+      <c r="M12" s="23" t="s">
         <v>142</v>
       </c>
-      <c r="K12" s="23" t="s">
+      <c r="N12" s="24" t="s">
         <v>143</v>
       </c>
-      <c r="L12" s="23" t="s">
+      <c r="O12" s="24" t="s">
         <v>144</v>
       </c>
-      <c r="M12" s="23" t="s">
+      <c r="P12" s="23" t="s">
         <v>145</v>
       </c>
-      <c r="N12" s="24" t="s">
+      <c r="Q12" s="23" t="s">
         <v>146</v>
       </c>
-      <c r="O12" s="24" t="s">
+      <c r="R12" s="25" t="s">
         <v>147</v>
       </c>
-      <c r="P12" s="23" t="s">
+      <c r="S12" s="23" t="s">
         <v>148</v>
       </c>
-      <c r="Q12" s="23" t="s">
+      <c r="T12" s="23" t="s">
         <v>149</v>
       </c>
-      <c r="R12" s="25" t="s">
+      <c r="U12" s="23" t="s">
         <v>150</v>
       </c>
-      <c r="S12" s="23" t="s">
+      <c r="V12" s="23" t="s">
         <v>151</v>
       </c>
-      <c r="T12" s="23" t="s">
+      <c r="W12" s="23" t="s">
         <v>152</v>
       </c>
-      <c r="U12" s="23" t="s">
+      <c r="X12" s="23" t="s">
         <v>153</v>
       </c>
-      <c r="V12" s="23" t="s">
+      <c r="Y12" s="23" t="s">
         <v>154</v>
       </c>
-      <c r="W12" s="23" t="s">
+      <c r="Z12" s="24" t="s">
         <v>155</v>
       </c>
-      <c r="X12" s="23" t="s">
+      <c r="AA12" s="24" t="s">
         <v>156</v>
       </c>
-      <c r="Y12" s="23" t="s">
+      <c r="AB12" s="23" t="s">
         <v>157</v>
       </c>
-      <c r="Z12" s="24" t="s">
+      <c r="AC12" s="45" t="s">
         <v>158</v>
       </c>
-      <c r="AA12" s="24" t="s">
+      <c r="AD12" s="24" t="s">
         <v>159</v>
       </c>
-      <c r="AB12" s="23" t="s">
+      <c r="AE12" s="24" t="s">
         <v>160</v>
       </c>
-      <c r="AC12" s="101" t="s">
+      <c r="AF12" s="24" t="s">
         <v>161</v>
       </c>
-      <c r="AD12" s="24" t="s">
+      <c r="AG12" s="24" t="s">
         <v>162</v>
       </c>
-      <c r="AE12" s="24" t="s">
+      <c r="AH12" s="39" t="s">
         <v>163</v>
       </c>
-      <c r="AF12" s="24" t="s">
+      <c r="AI12" s="22" t="s">
         <v>164</v>
       </c>
-      <c r="AG12" s="24" t="s">
+      <c r="AJ12" s="23" t="s">
         <v>165</v>
       </c>
-      <c r="AH12" s="39" t="s">
+      <c r="AK12" s="41" t="s">
+        <v>225</v>
+      </c>
+      <c r="AL12" s="26" t="s">
         <v>166</v>
       </c>
-      <c r="AI12" s="22" t="s">
+      <c r="AM12" s="26" t="s">
         <v>167</v>
       </c>
-      <c r="AJ12" s="23" t="s">
+      <c r="AN12" s="41" t="s">
+        <v>226</v>
+      </c>
+      <c r="AO12" s="27" t="s">
         <v>168</v>
       </c>
-      <c r="AK12" s="41" t="s">
-        <v>228</v>
-      </c>
-      <c r="AL12" s="26" t="s">
+      <c r="AP12" s="23" t="s">
         <v>169</v>
       </c>
-      <c r="AM12" s="26" t="s">
+      <c r="AQ12" s="41" t="s">
+        <v>227</v>
+      </c>
+      <c r="AR12" s="25" t="s">
         <v>170</v>
       </c>
-      <c r="AN12" s="41" t="s">
-        <v>229</v>
-      </c>
-      <c r="AO12" s="27" t="s">
+      <c r="AS12" s="23" t="s">
         <v>171</v>
       </c>
-      <c r="AP12" s="23" t="s">
+      <c r="AT12" s="23" t="s">
         <v>172</v>
       </c>
-      <c r="AQ12" s="41" t="s">
-        <v>230</v>
-      </c>
-      <c r="AR12" s="25" t="s">
+      <c r="AU12" s="23" t="s">
         <v>173</v>
       </c>
-      <c r="AS12" s="23" t="s">
+      <c r="AV12" s="24" t="s">
         <v>174</v>
       </c>
-      <c r="AT12" s="23" t="s">
+      <c r="AW12" s="24" t="s">
         <v>175</v>
       </c>
-      <c r="AU12" s="23" t="s">
+      <c r="AX12" s="23" t="s">
         <v>176</v>
       </c>
-      <c r="AV12" s="24" t="s">
+      <c r="AY12" s="23" t="s">
         <v>177</v>
       </c>
-      <c r="AW12" s="24" t="s">
+      <c r="AZ12" s="23" t="s">
         <v>178</v>
       </c>
-      <c r="AX12" s="23" t="s">
+      <c r="BA12" s="23" t="s">
         <v>179</v>
       </c>
-      <c r="AY12" s="23" t="s">
+      <c r="BB12" s="24" t="s">
         <v>180</v>
       </c>
-      <c r="AZ12" s="23" t="s">
+      <c r="BC12" s="24" t="s">
         <v>181</v>
       </c>
-      <c r="BA12" s="23" t="s">
+      <c r="BD12" s="23" t="s">
         <v>182</v>
       </c>
-      <c r="BB12" s="24" t="s">
+      <c r="BE12" s="23" t="s">
         <v>183</v>
       </c>
-      <c r="BC12" s="24" t="s">
+      <c r="BF12" s="23" t="s">
         <v>184</v>
       </c>
-      <c r="BD12" s="23" t="s">
+      <c r="BG12" s="26" t="s">
         <v>185</v>
       </c>
-      <c r="BE12" s="23" t="s">
+      <c r="BH12" s="22" t="s">
+        <v>221</v>
+      </c>
+      <c r="BI12" s="23" t="s">
         <v>186</v>
       </c>
-      <c r="BF12" s="23" t="s">
+      <c r="BJ12" s="23" t="s">
         <v>187</v>
       </c>
-      <c r="BG12" s="26" t="s">
+      <c r="BK12" s="23" t="s">
         <v>188</v>
       </c>
-      <c r="BH12" s="22" t="s">
-        <v>224</v>
-      </c>
-      <c r="BI12" s="23" t="s">
+      <c r="BL12" s="23" t="s">
         <v>189</v>
       </c>
-      <c r="BJ12" s="23" t="s">
+      <c r="BM12" s="23" t="s">
         <v>190</v>
       </c>
-      <c r="BK12" s="23" t="s">
+      <c r="BN12" s="23" t="s">
         <v>191</v>
       </c>
-      <c r="BL12" s="23" t="s">
+      <c r="BO12" s="23" t="s">
         <v>192</v>
       </c>
-      <c r="BM12" s="23" t="s">
+      <c r="BP12" s="24" t="s">
         <v>193</v>
       </c>
-      <c r="BN12" s="23" t="s">
+      <c r="BQ12" s="24" t="s">
         <v>194</v>
       </c>
-      <c r="BO12" s="23" t="s">
+      <c r="BR12" s="23" t="s">
         <v>195</v>
       </c>
-      <c r="BP12" s="24" t="s">
+      <c r="BS12" s="23" t="s">
         <v>196</v>
       </c>
-      <c r="BQ12" s="24" t="s">
+      <c r="BT12" s="23" t="s">
         <v>197</v>
       </c>
-      <c r="BR12" s="23" t="s">
+      <c r="BU12" s="23" t="s">
         <v>198</v>
       </c>
-      <c r="BS12" s="23" t="s">
+      <c r="BV12" s="23" t="s">
         <v>199</v>
       </c>
-      <c r="BT12" s="23" t="s">
+      <c r="BW12" s="23" t="s">
         <v>200</v>
       </c>
-      <c r="BU12" s="23" t="s">
+      <c r="BX12" s="23" t="s">
         <v>201</v>
       </c>
-      <c r="BV12" s="23" t="s">
+      <c r="BY12" s="23" t="s">
         <v>202</v>
       </c>
-      <c r="BW12" s="23" t="s">
+      <c r="BZ12" s="24" t="s">
         <v>203</v>
       </c>
-      <c r="BX12" s="23" t="s">
+      <c r="CA12" s="24" t="s">
         <v>204</v>
       </c>
-      <c r="BY12" s="23" t="s">
+      <c r="CB12" s="23" t="s">
         <v>205</v>
       </c>
-      <c r="BZ12" s="24" t="s">
+      <c r="CC12" s="23" t="s">
         <v>206</v>
       </c>
-      <c r="CA12" s="24" t="s">
+      <c r="CD12" s="23" t="s">
         <v>207</v>
       </c>
-      <c r="CB12" s="23" t="s">
+      <c r="CE12" s="23" t="s">
         <v>208</v>
       </c>
-      <c r="CC12" s="23" t="s">
+      <c r="CF12" s="23" t="s">
         <v>209</v>
       </c>
-      <c r="CD12" s="23" t="s">
+      <c r="CG12" s="23" t="s">
         <v>210</v>
       </c>
-      <c r="CE12" s="23" t="s">
+      <c r="CH12" s="23" t="s">
         <v>211</v>
       </c>
-      <c r="CF12" s="23" t="s">
+      <c r="CI12" s="28" t="s">
         <v>212</v>
       </c>
-      <c r="CG12" s="23" t="s">
+      <c r="CJ12" s="43" t="s">
         <v>213</v>
       </c>
-      <c r="CH12" s="23" t="s">
+      <c r="CK12" s="24" t="s">
         <v>214</v>
       </c>
-      <c r="CI12" s="28" t="s">
+      <c r="CL12" s="24" t="s">
         <v>215</v>
       </c>
-      <c r="CJ12" s="43" t="s">
+      <c r="CM12" s="24" t="s">
         <v>216</v>
       </c>
-      <c r="CK12" s="24" t="s">
+      <c r="CN12" s="24" t="s">
         <v>217</v>
       </c>
-      <c r="CL12" s="24" t="s">
+      <c r="CO12" s="24" t="s">
         <v>218</v>
       </c>
-      <c r="CM12" s="24" t="s">
+      <c r="CP12" s="24" t="s">
         <v>219</v>
-      </c>
-      <c r="CN12" s="24" t="s">
-        <v>220</v>
-      </c>
-      <c r="CO12" s="24" t="s">
-        <v>221</v>
-      </c>
-      <c r="CP12" s="24" t="s">
-        <v>222</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="101">
+    <mergeCell ref="CM8:CM10"/>
+    <mergeCell ref="CN8:CN10"/>
+    <mergeCell ref="CB8:CB10"/>
+    <mergeCell ref="BO8:BO10"/>
+    <mergeCell ref="CO8:CO10"/>
+    <mergeCell ref="AR8:AR10"/>
+    <mergeCell ref="AS8:AS10"/>
+    <mergeCell ref="AT8:AT10"/>
+    <mergeCell ref="AU8:AU10"/>
+    <mergeCell ref="AX8:AX10"/>
+    <mergeCell ref="AY8:AY10"/>
+    <mergeCell ref="AZ8:AZ10"/>
+    <mergeCell ref="BA8:BA10"/>
+    <mergeCell ref="BD8:BD10"/>
+    <mergeCell ref="BJ8:BJ10"/>
+    <mergeCell ref="BK8:BN10"/>
+    <mergeCell ref="AQ8:AQ10"/>
+    <mergeCell ref="AL7:AN7"/>
+    <mergeCell ref="AL8:AL10"/>
+    <mergeCell ref="AM8:AM10"/>
+    <mergeCell ref="AN8:AN10"/>
+    <mergeCell ref="O8:O10"/>
+    <mergeCell ref="P8:P10"/>
+    <mergeCell ref="Q8:Q10"/>
+    <mergeCell ref="R8:R10"/>
+    <mergeCell ref="S8:S10"/>
+    <mergeCell ref="T8:T10"/>
+    <mergeCell ref="V8:V10"/>
+    <mergeCell ref="W8:W10"/>
+    <mergeCell ref="X8:X10"/>
+    <mergeCell ref="Y8:Y10"/>
+    <mergeCell ref="AB8:AB10"/>
+    <mergeCell ref="AC8:AC10"/>
+    <mergeCell ref="AD8:AD10"/>
+    <mergeCell ref="AE8:AE10"/>
+    <mergeCell ref="CP8:CP10"/>
+    <mergeCell ref="AH9:AH10"/>
+    <mergeCell ref="BG9:BG10"/>
+    <mergeCell ref="CI9:CI10"/>
+    <mergeCell ref="CC8:CC10"/>
+    <mergeCell ref="CD8:CD10"/>
+    <mergeCell ref="CE8:CH10"/>
+    <mergeCell ref="CJ8:CJ10"/>
+    <mergeCell ref="CK8:CK10"/>
+    <mergeCell ref="CL8:CL10"/>
+    <mergeCell ref="BR8:BR10"/>
+    <mergeCell ref="BS8:BS10"/>
+    <mergeCell ref="BT8:BT10"/>
+    <mergeCell ref="BU8:BU10"/>
+    <mergeCell ref="BV8:BY10"/>
+    <mergeCell ref="BF8:BF10"/>
+    <mergeCell ref="BH8:BH10"/>
+    <mergeCell ref="BI8:BI10"/>
+    <mergeCell ref="AO8:AO10"/>
+    <mergeCell ref="AI8:AI10"/>
+    <mergeCell ref="AJ8:AJ10"/>
+    <mergeCell ref="AK8:AK10"/>
+    <mergeCell ref="BE8:BE10"/>
+    <mergeCell ref="AP8:AP10"/>
+    <mergeCell ref="AI5:AK5"/>
+    <mergeCell ref="AO5:AQ5"/>
+    <mergeCell ref="AR5:BG5"/>
+    <mergeCell ref="BH5:CI5"/>
+    <mergeCell ref="CJ5:CO5"/>
+    <mergeCell ref="AL5:AN5"/>
+    <mergeCell ref="CP5:CP7"/>
+    <mergeCell ref="AR6:AX6"/>
+    <mergeCell ref="AY6:BC6"/>
+    <mergeCell ref="BD6:BF6"/>
+    <mergeCell ref="BH6:BR6"/>
+    <mergeCell ref="CO6:CO7"/>
+    <mergeCell ref="CJ6:CJ7"/>
+    <mergeCell ref="CK6:CN6"/>
+    <mergeCell ref="AI7:AK7"/>
+    <mergeCell ref="AO7:AQ7"/>
+    <mergeCell ref="BS6:CA6"/>
+    <mergeCell ref="CB6:CI6"/>
     <mergeCell ref="B1:AA1"/>
     <mergeCell ref="B2:AA2"/>
     <mergeCell ref="M3:P3"/>
@@ -3523,83 +3600,6 @@
     <mergeCell ref="L8:L10"/>
     <mergeCell ref="M8:M10"/>
     <mergeCell ref="N8:N10"/>
-    <mergeCell ref="AI5:AK5"/>
-    <mergeCell ref="AO5:AQ5"/>
-    <mergeCell ref="AR5:BG5"/>
-    <mergeCell ref="BH5:CI5"/>
-    <mergeCell ref="CJ5:CO5"/>
-    <mergeCell ref="AL5:AN5"/>
-    <mergeCell ref="CP5:CP7"/>
-    <mergeCell ref="AR6:AX6"/>
-    <mergeCell ref="AY6:BC6"/>
-    <mergeCell ref="BD6:BF6"/>
-    <mergeCell ref="BH6:BR6"/>
-    <mergeCell ref="CO6:CO7"/>
-    <mergeCell ref="CJ6:CJ7"/>
-    <mergeCell ref="CK6:CN6"/>
-    <mergeCell ref="AI7:AK7"/>
-    <mergeCell ref="AO7:AQ7"/>
-    <mergeCell ref="BS6:CA6"/>
-    <mergeCell ref="CB6:CI6"/>
-    <mergeCell ref="CP8:CP10"/>
-    <mergeCell ref="AH9:AH10"/>
-    <mergeCell ref="BG9:BG10"/>
-    <mergeCell ref="CI9:CI10"/>
-    <mergeCell ref="CC8:CC10"/>
-    <mergeCell ref="CD8:CD10"/>
-    <mergeCell ref="CE8:CH10"/>
-    <mergeCell ref="CJ8:CJ10"/>
-    <mergeCell ref="CK8:CK10"/>
-    <mergeCell ref="CL8:CL10"/>
-    <mergeCell ref="BR8:BR10"/>
-    <mergeCell ref="BS8:BS10"/>
-    <mergeCell ref="BT8:BT10"/>
-    <mergeCell ref="BU8:BU10"/>
-    <mergeCell ref="BV8:BY10"/>
-    <mergeCell ref="BF8:BF10"/>
-    <mergeCell ref="BH8:BH10"/>
-    <mergeCell ref="BI8:BI10"/>
-    <mergeCell ref="AO8:AO10"/>
-    <mergeCell ref="AI8:AI10"/>
-    <mergeCell ref="AJ8:AJ10"/>
-    <mergeCell ref="AK8:AK10"/>
-    <mergeCell ref="BE8:BE10"/>
-    <mergeCell ref="AP8:AP10"/>
-    <mergeCell ref="AQ8:AQ10"/>
-    <mergeCell ref="AL7:AN7"/>
-    <mergeCell ref="AL8:AL10"/>
-    <mergeCell ref="AM8:AM10"/>
-    <mergeCell ref="AN8:AN10"/>
-    <mergeCell ref="O8:O10"/>
-    <mergeCell ref="P8:P10"/>
-    <mergeCell ref="Q8:Q10"/>
-    <mergeCell ref="R8:R10"/>
-    <mergeCell ref="S8:S10"/>
-    <mergeCell ref="T8:T10"/>
-    <mergeCell ref="V8:V10"/>
-    <mergeCell ref="W8:W10"/>
-    <mergeCell ref="X8:X10"/>
-    <mergeCell ref="Y8:Y10"/>
-    <mergeCell ref="AB8:AB10"/>
-    <mergeCell ref="AC8:AC10"/>
-    <mergeCell ref="AD8:AD10"/>
-    <mergeCell ref="AE8:AE10"/>
-    <mergeCell ref="CM8:CM10"/>
-    <mergeCell ref="CN8:CN10"/>
-    <mergeCell ref="CB8:CB10"/>
-    <mergeCell ref="BO8:BO10"/>
-    <mergeCell ref="CO8:CO10"/>
-    <mergeCell ref="AR8:AR10"/>
-    <mergeCell ref="AS8:AS10"/>
-    <mergeCell ref="AT8:AT10"/>
-    <mergeCell ref="AU8:AU10"/>
-    <mergeCell ref="AX8:AX10"/>
-    <mergeCell ref="AY8:AY10"/>
-    <mergeCell ref="AZ8:AZ10"/>
-    <mergeCell ref="BA8:BA10"/>
-    <mergeCell ref="BD8:BD10"/>
-    <mergeCell ref="BJ8:BJ10"/>
-    <mergeCell ref="BK8:BN10"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
fix 3 type report
</commit_message>
<xml_diff>
--- a/src/main/resources/templates/summaryReportForm3.xlsx
+++ b/src/main/resources/templates/summaryReportForm3.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="21231"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F39A44D4-1B1D-4568-BC45-C71964FAC7FB}" xr6:coauthVersionLast="40" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F41BEED9-2841-4863-BF6B-066F1B11CBB0}" xr6:coauthVersionLast="40" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -259,15 +259,6 @@
     <t>$dist_value48</t>
   </si>
   <si>
-    <t>$dist_value51</t>
-  </si>
-  <si>
-    <t>$dist_value52</t>
-  </si>
-  <si>
-    <t>$dist_value53</t>
-  </si>
-  <si>
     <t>$dist_value56</t>
   </si>
   <si>
@@ -310,27 +301,6 @@
     <t>$dist_value72</t>
   </si>
   <si>
-    <t>$dist_value75</t>
-  </si>
-  <si>
-    <t>$dist_value76</t>
-  </si>
-  <si>
-    <t>$dist_value77</t>
-  </si>
-  <si>
-    <t>$dist_value78</t>
-  </si>
-  <si>
-    <t>$dist_value79</t>
-  </si>
-  <si>
-    <t>$dist_value80</t>
-  </si>
-  <si>
-    <t>$dist_value81</t>
-  </si>
-  <si>
     <t>$dist_value83</t>
   </si>
   <si>
@@ -568,15 +538,6 @@
     <t>$prod_pct_value48_value46</t>
   </si>
   <si>
-    <t>$prod_value51</t>
-  </si>
-  <si>
-    <t>$prod_value52</t>
-  </si>
-  <si>
-    <t>$prod_value53</t>
-  </si>
-  <si>
     <t>$prod_sub_value53_value52</t>
   </si>
   <si>
@@ -637,27 +598,6 @@
     <t>$prod_pct_value68_value66</t>
   </si>
   <si>
-    <t>$prod_value75</t>
-  </si>
-  <si>
-    <t>$prod_value76</t>
-  </si>
-  <si>
-    <t>$prod_value77</t>
-  </si>
-  <si>
-    <t>$prod_value78</t>
-  </si>
-  <si>
-    <t>$prod_value79</t>
-  </si>
-  <si>
-    <t>$prod_value80</t>
-  </si>
-  <si>
-    <t>$prod_value81</t>
-  </si>
-  <si>
     <t>$prod_sub_value77_value76</t>
   </si>
   <si>
@@ -719,6 +659,66 @@
   </si>
   <si>
     <t>$dist_pdc_value17_value3</t>
+  </si>
+  <si>
+    <t>$prod_pdc_value46_value39</t>
+  </si>
+  <si>
+    <t>$prod_pdc_value47_value40</t>
+  </si>
+  <si>
+    <t>$prod_pdc_value48_value41</t>
+  </si>
+  <si>
+    <t>$dist_pdc_value46_value39</t>
+  </si>
+  <si>
+    <t>$dist_pdc_value47_value40</t>
+  </si>
+  <si>
+    <t>$dist_pdc_value48_value41</t>
+  </si>
+  <si>
+    <t>$prod_pdc_value66_value55</t>
+  </si>
+  <si>
+    <t>$prod_pdc_value67_value56</t>
+  </si>
+  <si>
+    <t>$prod_pdc_value68_value57</t>
+  </si>
+  <si>
+    <t>$prod_pdc_value69_value58</t>
+  </si>
+  <si>
+    <t>$prod_pdc_value70_value59</t>
+  </si>
+  <si>
+    <t>$prod_pdc_value71_value60</t>
+  </si>
+  <si>
+    <t>$prod_pdc_value72_value61</t>
+  </si>
+  <si>
+    <t>$dist_pdc_value66_value55</t>
+  </si>
+  <si>
+    <t>$dist_pdc_value67_value56</t>
+  </si>
+  <si>
+    <t>$dist_pdc_value68_value57</t>
+  </si>
+  <si>
+    <t>$dist_pdc_value69_value58</t>
+  </si>
+  <si>
+    <t>$dist_pdc_value70_value59</t>
+  </si>
+  <si>
+    <t>$dist_pdc_value71_value60</t>
+  </si>
+  <si>
+    <t>$dist_pdc_value72_value61</t>
   </si>
 </sst>
 </file>
@@ -1368,6 +1368,153 @@
     <xf numFmtId="164" fontId="4" fillId="0" borderId="32" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="3" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1377,49 +1524,10 @@
     <xf numFmtId="49" fontId="4" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="49" fontId="4" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="49" fontId="1" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="4" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1427,114 +1535,6 @@
     </xf>
     <xf numFmtId="49" fontId="4" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="29" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="19" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="28" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="27" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1825,235 +1825,235 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:94" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B1" s="36" t="s">
+      <c r="B1" s="85" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="36"/>
-      <c r="D1" s="36"/>
-      <c r="E1" s="36"/>
-      <c r="F1" s="36"/>
-      <c r="G1" s="36"/>
-      <c r="H1" s="36"/>
-      <c r="I1" s="36"/>
-      <c r="J1" s="36"/>
-      <c r="K1" s="36"/>
-      <c r="L1" s="36"/>
-      <c r="M1" s="36"/>
-      <c r="N1" s="36"/>
-      <c r="O1" s="36"/>
-      <c r="P1" s="36"/>
-      <c r="Q1" s="36"/>
-      <c r="R1" s="36"/>
-      <c r="S1" s="36"/>
-      <c r="T1" s="36"/>
-      <c r="U1" s="36"/>
-      <c r="V1" s="36"/>
-      <c r="W1" s="36"/>
-      <c r="X1" s="36"/>
-      <c r="Y1" s="36"/>
-      <c r="Z1" s="36"/>
-      <c r="AA1" s="36"/>
+      <c r="C1" s="85"/>
+      <c r="D1" s="85"/>
+      <c r="E1" s="85"/>
+      <c r="F1" s="85"/>
+      <c r="G1" s="85"/>
+      <c r="H1" s="85"/>
+      <c r="I1" s="85"/>
+      <c r="J1" s="85"/>
+      <c r="K1" s="85"/>
+      <c r="L1" s="85"/>
+      <c r="M1" s="85"/>
+      <c r="N1" s="85"/>
+      <c r="O1" s="85"/>
+      <c r="P1" s="85"/>
+      <c r="Q1" s="85"/>
+      <c r="R1" s="85"/>
+      <c r="S1" s="85"/>
+      <c r="T1" s="85"/>
+      <c r="U1" s="85"/>
+      <c r="V1" s="85"/>
+      <c r="W1" s="85"/>
+      <c r="X1" s="85"/>
+      <c r="Y1" s="85"/>
+      <c r="Z1" s="85"/>
+      <c r="AA1" s="85"/>
     </row>
     <row r="2" spans="1:94" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="B2" s="36" t="s">
+      <c r="B2" s="85" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="36"/>
-      <c r="D2" s="36"/>
-      <c r="E2" s="36"/>
-      <c r="F2" s="36"/>
-      <c r="G2" s="36"/>
-      <c r="H2" s="36"/>
-      <c r="I2" s="36"/>
-      <c r="J2" s="36"/>
-      <c r="K2" s="36"/>
-      <c r="L2" s="36"/>
-      <c r="M2" s="36"/>
-      <c r="N2" s="36"/>
-      <c r="O2" s="36"/>
-      <c r="P2" s="36"/>
-      <c r="Q2" s="36"/>
-      <c r="R2" s="36"/>
-      <c r="S2" s="36"/>
-      <c r="T2" s="36"/>
-      <c r="U2" s="36"/>
-      <c r="V2" s="36"/>
-      <c r="W2" s="36"/>
-      <c r="X2" s="36"/>
-      <c r="Y2" s="36"/>
-      <c r="Z2" s="36"/>
-      <c r="AA2" s="36"/>
+      <c r="C2" s="85"/>
+      <c r="D2" s="85"/>
+      <c r="E2" s="85"/>
+      <c r="F2" s="85"/>
+      <c r="G2" s="85"/>
+      <c r="H2" s="85"/>
+      <c r="I2" s="85"/>
+      <c r="J2" s="85"/>
+      <c r="K2" s="85"/>
+      <c r="L2" s="85"/>
+      <c r="M2" s="85"/>
+      <c r="N2" s="85"/>
+      <c r="O2" s="85"/>
+      <c r="P2" s="85"/>
+      <c r="Q2" s="85"/>
+      <c r="R2" s="85"/>
+      <c r="S2" s="85"/>
+      <c r="T2" s="85"/>
+      <c r="U2" s="85"/>
+      <c r="V2" s="85"/>
+      <c r="W2" s="85"/>
+      <c r="X2" s="85"/>
+      <c r="Y2" s="85"/>
+      <c r="Z2" s="85"/>
+      <c r="AA2" s="85"/>
       <c r="AB2" s="3"/>
     </row>
     <row r="3" spans="1:94" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="L3" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="M3" s="37" t="s">
-        <v>228</v>
-      </c>
-      <c r="N3" s="37"/>
-      <c r="O3" s="37"/>
-      <c r="P3" s="37"/>
+      <c r="M3" s="86" t="s">
+        <v>208</v>
+      </c>
+      <c r="N3" s="86"/>
+      <c r="O3" s="86"/>
+      <c r="P3" s="86"/>
     </row>
     <row r="4" spans="1:94" s="2" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="5" spans="1:94" s="2" customFormat="1" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="38" t="s">
+      <c r="A5" s="87" t="s">
         <v>3</v>
       </c>
-      <c r="B5" s="41" t="s">
+      <c r="B5" s="88" t="s">
         <v>4</v>
       </c>
-      <c r="C5" s="44" t="s">
+      <c r="C5" s="66" t="s">
         <v>5</v>
       </c>
-      <c r="D5" s="45"/>
-      <c r="E5" s="45"/>
-      <c r="F5" s="45"/>
-      <c r="G5" s="45"/>
-      <c r="H5" s="45"/>
-      <c r="I5" s="45"/>
-      <c r="J5" s="45"/>
-      <c r="K5" s="45"/>
-      <c r="L5" s="45"/>
-      <c r="M5" s="45"/>
-      <c r="N5" s="45"/>
-      <c r="O5" s="45"/>
-      <c r="P5" s="45"/>
-      <c r="Q5" s="45"/>
-      <c r="R5" s="45"/>
-      <c r="S5" s="45"/>
-      <c r="T5" s="45"/>
-      <c r="U5" s="45"/>
-      <c r="V5" s="45"/>
-      <c r="W5" s="45"/>
-      <c r="X5" s="45"/>
-      <c r="Y5" s="45"/>
-      <c r="Z5" s="45"/>
-      <c r="AA5" s="45"/>
-      <c r="AB5" s="45"/>
-      <c r="AC5" s="45"/>
-      <c r="AD5" s="45"/>
-      <c r="AE5" s="45"/>
-      <c r="AF5" s="45"/>
-      <c r="AG5" s="45"/>
-      <c r="AH5" s="45"/>
-      <c r="AI5" s="58" t="s">
+      <c r="D5" s="65"/>
+      <c r="E5" s="65"/>
+      <c r="F5" s="65"/>
+      <c r="G5" s="65"/>
+      <c r="H5" s="65"/>
+      <c r="I5" s="65"/>
+      <c r="J5" s="65"/>
+      <c r="K5" s="65"/>
+      <c r="L5" s="65"/>
+      <c r="M5" s="65"/>
+      <c r="N5" s="65"/>
+      <c r="O5" s="65"/>
+      <c r="P5" s="65"/>
+      <c r="Q5" s="65"/>
+      <c r="R5" s="65"/>
+      <c r="S5" s="65"/>
+      <c r="T5" s="65"/>
+      <c r="U5" s="65"/>
+      <c r="V5" s="65"/>
+      <c r="W5" s="65"/>
+      <c r="X5" s="65"/>
+      <c r="Y5" s="65"/>
+      <c r="Z5" s="65"/>
+      <c r="AA5" s="65"/>
+      <c r="AB5" s="65"/>
+      <c r="AC5" s="65"/>
+      <c r="AD5" s="65"/>
+      <c r="AE5" s="65"/>
+      <c r="AF5" s="65"/>
+      <c r="AG5" s="65"/>
+      <c r="AH5" s="65"/>
+      <c r="AI5" s="59" t="s">
         <v>6</v>
       </c>
-      <c r="AJ5" s="59"/>
-      <c r="AK5" s="60"/>
-      <c r="AL5" s="58" t="s">
+      <c r="AJ5" s="60"/>
+      <c r="AK5" s="61"/>
+      <c r="AL5" s="59" t="s">
         <v>43</v>
       </c>
-      <c r="AM5" s="59"/>
-      <c r="AN5" s="60"/>
-      <c r="AO5" s="61" t="s">
+      <c r="AM5" s="60"/>
+      <c r="AN5" s="61"/>
+      <c r="AO5" s="62" t="s">
         <v>7</v>
       </c>
-      <c r="AP5" s="62"/>
-      <c r="AQ5" s="63"/>
-      <c r="AR5" s="45" t="s">
+      <c r="AP5" s="63"/>
+      <c r="AQ5" s="64"/>
+      <c r="AR5" s="65" t="s">
         <v>8</v>
       </c>
-      <c r="AS5" s="45"/>
-      <c r="AT5" s="45"/>
-      <c r="AU5" s="45"/>
-      <c r="AV5" s="45"/>
-      <c r="AW5" s="45"/>
-      <c r="AX5" s="45"/>
-      <c r="AY5" s="45"/>
-      <c r="AZ5" s="45"/>
-      <c r="BA5" s="45"/>
-      <c r="BB5" s="45"/>
-      <c r="BC5" s="45"/>
-      <c r="BD5" s="45"/>
-      <c r="BE5" s="45"/>
-      <c r="BF5" s="45"/>
-      <c r="BG5" s="45"/>
-      <c r="BH5" s="44" t="s">
+      <c r="AS5" s="65"/>
+      <c r="AT5" s="65"/>
+      <c r="AU5" s="65"/>
+      <c r="AV5" s="65"/>
+      <c r="AW5" s="65"/>
+      <c r="AX5" s="65"/>
+      <c r="AY5" s="65"/>
+      <c r="AZ5" s="65"/>
+      <c r="BA5" s="65"/>
+      <c r="BB5" s="65"/>
+      <c r="BC5" s="65"/>
+      <c r="BD5" s="65"/>
+      <c r="BE5" s="65"/>
+      <c r="BF5" s="65"/>
+      <c r="BG5" s="65"/>
+      <c r="BH5" s="66" t="s">
         <v>9</v>
       </c>
-      <c r="BI5" s="45"/>
-      <c r="BJ5" s="45"/>
-      <c r="BK5" s="45"/>
-      <c r="BL5" s="45"/>
-      <c r="BM5" s="45"/>
-      <c r="BN5" s="45"/>
-      <c r="BO5" s="45"/>
-      <c r="BP5" s="45"/>
-      <c r="BQ5" s="45"/>
-      <c r="BR5" s="45"/>
-      <c r="BS5" s="45"/>
-      <c r="BT5" s="45"/>
-      <c r="BU5" s="45"/>
-      <c r="BV5" s="45"/>
-      <c r="BW5" s="45"/>
-      <c r="BX5" s="45"/>
-      <c r="BY5" s="45"/>
-      <c r="BZ5" s="45"/>
-      <c r="CA5" s="45"/>
-      <c r="CB5" s="45"/>
-      <c r="CC5" s="45"/>
-      <c r="CD5" s="45"/>
-      <c r="CE5" s="45"/>
-      <c r="CF5" s="45"/>
-      <c r="CG5" s="45"/>
-      <c r="CH5" s="45"/>
-      <c r="CI5" s="64"/>
-      <c r="CJ5" s="65" t="s">
+      <c r="BI5" s="65"/>
+      <c r="BJ5" s="65"/>
+      <c r="BK5" s="65"/>
+      <c r="BL5" s="65"/>
+      <c r="BM5" s="65"/>
+      <c r="BN5" s="65"/>
+      <c r="BO5" s="65"/>
+      <c r="BP5" s="65"/>
+      <c r="BQ5" s="65"/>
+      <c r="BR5" s="65"/>
+      <c r="BS5" s="65"/>
+      <c r="BT5" s="65"/>
+      <c r="BU5" s="65"/>
+      <c r="BV5" s="65"/>
+      <c r="BW5" s="65"/>
+      <c r="BX5" s="65"/>
+      <c r="BY5" s="65"/>
+      <c r="BZ5" s="65"/>
+      <c r="CA5" s="65"/>
+      <c r="CB5" s="65"/>
+      <c r="CC5" s="65"/>
+      <c r="CD5" s="65"/>
+      <c r="CE5" s="65"/>
+      <c r="CF5" s="65"/>
+      <c r="CG5" s="65"/>
+      <c r="CH5" s="65"/>
+      <c r="CI5" s="67"/>
+      <c r="CJ5" s="68" t="s">
         <v>10</v>
       </c>
-      <c r="CK5" s="65"/>
-      <c r="CL5" s="65"/>
-      <c r="CM5" s="65"/>
-      <c r="CN5" s="65"/>
-      <c r="CO5" s="65"/>
-      <c r="CP5" s="66" t="s">
+      <c r="CK5" s="68"/>
+      <c r="CL5" s="68"/>
+      <c r="CM5" s="68"/>
+      <c r="CN5" s="68"/>
+      <c r="CO5" s="68"/>
+      <c r="CP5" s="69" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="6" spans="1:94" s="2" customFormat="1" ht="39.950000000000003" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="39"/>
-      <c r="B6" s="42"/>
-      <c r="C6" s="46" t="s">
+      <c r="A6" s="57"/>
+      <c r="B6" s="46"/>
+      <c r="C6" s="89" t="s">
         <v>12</v>
       </c>
-      <c r="D6" s="47"/>
-      <c r="E6" s="47"/>
-      <c r="F6" s="47"/>
-      <c r="G6" s="47"/>
-      <c r="H6" s="47"/>
-      <c r="I6" s="47"/>
-      <c r="J6" s="47"/>
-      <c r="K6" s="47"/>
-      <c r="L6" s="47"/>
-      <c r="M6" s="47"/>
-      <c r="N6" s="47"/>
-      <c r="O6" s="47"/>
-      <c r="P6" s="47"/>
-      <c r="Q6" s="48" t="s">
+      <c r="D6" s="72"/>
+      <c r="E6" s="72"/>
+      <c r="F6" s="72"/>
+      <c r="G6" s="72"/>
+      <c r="H6" s="72"/>
+      <c r="I6" s="72"/>
+      <c r="J6" s="72"/>
+      <c r="K6" s="72"/>
+      <c r="L6" s="72"/>
+      <c r="M6" s="72"/>
+      <c r="N6" s="72"/>
+      <c r="O6" s="72"/>
+      <c r="P6" s="72"/>
+      <c r="Q6" s="78" t="s">
         <v>13</v>
       </c>
-      <c r="R6" s="48"/>
-      <c r="S6" s="48"/>
-      <c r="T6" s="48"/>
-      <c r="U6" s="48"/>
-      <c r="V6" s="48"/>
-      <c r="W6" s="48"/>
-      <c r="X6" s="48"/>
-      <c r="Y6" s="48"/>
-      <c r="Z6" s="48"/>
-      <c r="AA6" s="48"/>
-      <c r="AB6" s="48"/>
-      <c r="AC6" s="48" t="s">
+      <c r="R6" s="78"/>
+      <c r="S6" s="78"/>
+      <c r="T6" s="78"/>
+      <c r="U6" s="78"/>
+      <c r="V6" s="78"/>
+      <c r="W6" s="78"/>
+      <c r="X6" s="78"/>
+      <c r="Y6" s="78"/>
+      <c r="Z6" s="78"/>
+      <c r="AA6" s="78"/>
+      <c r="AB6" s="78"/>
+      <c r="AC6" s="78" t="s">
         <v>14</v>
       </c>
-      <c r="AD6" s="48"/>
-      <c r="AE6" s="48"/>
-      <c r="AF6" s="48"/>
-      <c r="AG6" s="48"/>
-      <c r="AH6" s="49"/>
+      <c r="AD6" s="78"/>
+      <c r="AE6" s="78"/>
+      <c r="AF6" s="78"/>
+      <c r="AG6" s="78"/>
+      <c r="AH6" s="74"/>
       <c r="AI6" s="5" t="s">
         <v>12</v>
       </c>
@@ -2081,94 +2081,94 @@
       <c r="AQ6" s="14" t="s">
         <v>15</v>
       </c>
-      <c r="AR6" s="47" t="s">
+      <c r="AR6" s="72" t="s">
         <v>12</v>
       </c>
-      <c r="AS6" s="47"/>
-      <c r="AT6" s="47"/>
-      <c r="AU6" s="47"/>
-      <c r="AV6" s="47"/>
-      <c r="AW6" s="47"/>
-      <c r="AX6" s="69"/>
-      <c r="AY6" s="49" t="s">
+      <c r="AS6" s="72"/>
+      <c r="AT6" s="72"/>
+      <c r="AU6" s="72"/>
+      <c r="AV6" s="72"/>
+      <c r="AW6" s="72"/>
+      <c r="AX6" s="73"/>
+      <c r="AY6" s="74" t="s">
         <v>13</v>
       </c>
-      <c r="AZ6" s="52"/>
-      <c r="BA6" s="52"/>
-      <c r="BB6" s="52"/>
-      <c r="BC6" s="53"/>
-      <c r="BD6" s="49" t="s">
+      <c r="AZ6" s="75"/>
+      <c r="BA6" s="75"/>
+      <c r="BB6" s="75"/>
+      <c r="BC6" s="76"/>
+      <c r="BD6" s="74" t="s">
         <v>14</v>
       </c>
-      <c r="BE6" s="52"/>
-      <c r="BF6" s="52"/>
+      <c r="BE6" s="75"/>
+      <c r="BF6" s="75"/>
       <c r="BG6" s="6"/>
-      <c r="BH6" s="70" t="s">
+      <c r="BH6" s="77" t="s">
         <v>12</v>
       </c>
-      <c r="BI6" s="52"/>
-      <c r="BJ6" s="52"/>
-      <c r="BK6" s="52"/>
-      <c r="BL6" s="52"/>
-      <c r="BM6" s="52"/>
-      <c r="BN6" s="52"/>
-      <c r="BO6" s="52"/>
-      <c r="BP6" s="52"/>
-      <c r="BQ6" s="52"/>
-      <c r="BR6" s="53"/>
-      <c r="BS6" s="48" t="s">
+      <c r="BI6" s="75"/>
+      <c r="BJ6" s="75"/>
+      <c r="BK6" s="75"/>
+      <c r="BL6" s="75"/>
+      <c r="BM6" s="75"/>
+      <c r="BN6" s="75"/>
+      <c r="BO6" s="75"/>
+      <c r="BP6" s="75"/>
+      <c r="BQ6" s="75"/>
+      <c r="BR6" s="76"/>
+      <c r="BS6" s="78" t="s">
         <v>13</v>
       </c>
-      <c r="BT6" s="48"/>
-      <c r="BU6" s="48"/>
-      <c r="BV6" s="48"/>
-      <c r="BW6" s="48"/>
-      <c r="BX6" s="48"/>
-      <c r="BY6" s="48"/>
-      <c r="BZ6" s="48"/>
-      <c r="CA6" s="48"/>
-      <c r="CB6" s="48" t="s">
+      <c r="BT6" s="78"/>
+      <c r="BU6" s="78"/>
+      <c r="BV6" s="78"/>
+      <c r="BW6" s="78"/>
+      <c r="BX6" s="78"/>
+      <c r="BY6" s="78"/>
+      <c r="BZ6" s="78"/>
+      <c r="CA6" s="78"/>
+      <c r="CB6" s="78" t="s">
         <v>14</v>
       </c>
-      <c r="CC6" s="48"/>
-      <c r="CD6" s="48"/>
-      <c r="CE6" s="49"/>
-      <c r="CF6" s="49"/>
-      <c r="CG6" s="49"/>
-      <c r="CH6" s="49"/>
-      <c r="CI6" s="79"/>
-      <c r="CJ6" s="71" t="s">
+      <c r="CC6" s="78"/>
+      <c r="CD6" s="78"/>
+      <c r="CE6" s="74"/>
+      <c r="CF6" s="74"/>
+      <c r="CG6" s="74"/>
+      <c r="CH6" s="74"/>
+      <c r="CI6" s="84"/>
+      <c r="CJ6" s="79" t="s">
         <v>16</v>
       </c>
-      <c r="CK6" s="73" t="s">
+      <c r="CK6" s="81" t="s">
         <v>17</v>
       </c>
-      <c r="CL6" s="74"/>
-      <c r="CM6" s="74"/>
-      <c r="CN6" s="75"/>
-      <c r="CO6" s="48" t="s">
+      <c r="CL6" s="82"/>
+      <c r="CM6" s="82"/>
+      <c r="CN6" s="83"/>
+      <c r="CO6" s="78" t="s">
         <v>18</v>
       </c>
-      <c r="CP6" s="67"/>
+      <c r="CP6" s="70"/>
     </row>
     <row r="7" spans="1:94" s="2" customFormat="1" ht="56.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="39"/>
-      <c r="B7" s="42"/>
+      <c r="A7" s="57"/>
+      <c r="B7" s="46"/>
       <c r="C7" s="9" t="s">
         <v>19</v>
       </c>
       <c r="D7" s="8" t="s">
         <v>20</v>
       </c>
-      <c r="E7" s="49" t="s">
+      <c r="E7" s="74" t="s">
         <v>21</v>
       </c>
-      <c r="F7" s="52"/>
-      <c r="G7" s="52"/>
-      <c r="H7" s="52"/>
-      <c r="I7" s="52"/>
-      <c r="J7" s="52"/>
-      <c r="K7" s="53"/>
+      <c r="F7" s="75"/>
+      <c r="G7" s="75"/>
+      <c r="H7" s="75"/>
+      <c r="I7" s="75"/>
+      <c r="J7" s="75"/>
+      <c r="K7" s="76"/>
       <c r="L7" s="8" t="s">
         <v>22</v>
       </c>
@@ -2190,15 +2190,15 @@
       <c r="R7" s="8" t="s">
         <v>20</v>
       </c>
-      <c r="S7" s="49" t="s">
+      <c r="S7" s="74" t="s">
         <v>27</v>
       </c>
-      <c r="T7" s="52"/>
-      <c r="U7" s="52"/>
-      <c r="V7" s="52"/>
-      <c r="W7" s="52"/>
-      <c r="X7" s="52"/>
-      <c r="Y7" s="53"/>
+      <c r="T7" s="75"/>
+      <c r="U7" s="75"/>
+      <c r="V7" s="75"/>
+      <c r="W7" s="75"/>
+      <c r="X7" s="75"/>
+      <c r="Y7" s="76"/>
       <c r="Z7" s="10" t="s">
         <v>24</v>
       </c>
@@ -2226,21 +2226,21 @@
       <c r="AH7" s="15" t="s">
         <v>29</v>
       </c>
-      <c r="AI7" s="76" t="s">
+      <c r="AI7" s="48" t="s">
         <v>27</v>
       </c>
-      <c r="AJ7" s="77"/>
-      <c r="AK7" s="78"/>
-      <c r="AL7" s="76" t="s">
+      <c r="AJ7" s="49"/>
+      <c r="AK7" s="50"/>
+      <c r="AL7" s="48" t="s">
         <v>27</v>
       </c>
-      <c r="AM7" s="77"/>
-      <c r="AN7" s="78"/>
-      <c r="AO7" s="53" t="s">
+      <c r="AM7" s="49"/>
+      <c r="AN7" s="50"/>
+      <c r="AO7" s="76" t="s">
         <v>27</v>
       </c>
-      <c r="AP7" s="48"/>
-      <c r="AQ7" s="79"/>
+      <c r="AP7" s="78"/>
+      <c r="AQ7" s="84"/>
       <c r="AR7" s="7" t="s">
         <v>19</v>
       </c>
@@ -2373,7 +2373,7 @@
       <c r="CI7" s="12" t="s">
         <v>29</v>
       </c>
-      <c r="CJ7" s="72"/>
+      <c r="CJ7" s="80"/>
       <c r="CK7" s="8" t="s">
         <v>34</v>
       </c>
@@ -2386,79 +2386,79 @@
       <c r="CN7" s="8" t="s">
         <v>37</v>
       </c>
-      <c r="CO7" s="48"/>
-      <c r="CP7" s="68"/>
+      <c r="CO7" s="78"/>
+      <c r="CP7" s="71"/>
     </row>
     <row r="8" spans="1:94" s="2" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="39"/>
-      <c r="B8" s="42"/>
-      <c r="C8" s="50" t="s">
+      <c r="A8" s="57"/>
+      <c r="B8" s="46"/>
+      <c r="C8" s="51" t="s">
         <v>38</v>
       </c>
-      <c r="D8" s="54" t="s">
-        <v>229</v>
-      </c>
-      <c r="E8" s="56" t="s">
-        <v>229</v>
-      </c>
-      <c r="F8" s="56" t="s">
+      <c r="D8" s="90" t="s">
+        <v>209</v>
+      </c>
+      <c r="E8" s="36" t="s">
+        <v>209</v>
+      </c>
+      <c r="F8" s="36" t="s">
         <v>35</v>
       </c>
-      <c r="G8" s="56" t="s">
+      <c r="G8" s="36" t="s">
         <v>36</v>
       </c>
-      <c r="H8" s="56" t="s">
+      <c r="H8" s="36" t="s">
         <v>39</v>
       </c>
-      <c r="I8" s="56" t="s">
+      <c r="I8" s="36" t="s">
         <v>40</v>
       </c>
-      <c r="J8" s="56" t="s">
+      <c r="J8" s="36" t="s">
         <v>34</v>
       </c>
-      <c r="K8" s="56" t="s">
+      <c r="K8" s="36" t="s">
         <v>41</v>
       </c>
-      <c r="L8" s="56" t="s">
-        <v>229</v>
-      </c>
-      <c r="M8" s="56" t="s">
-        <v>229</v>
-      </c>
-      <c r="N8" s="56" t="s">
-        <v>229</v>
-      </c>
-      <c r="O8" s="57" t="s">
+      <c r="L8" s="36" t="s">
+        <v>209</v>
+      </c>
+      <c r="M8" s="36" t="s">
+        <v>209</v>
+      </c>
+      <c r="N8" s="36" t="s">
+        <v>209</v>
+      </c>
+      <c r="O8" s="37" t="s">
         <v>42</v>
       </c>
-      <c r="P8" s="56" t="s">
-        <v>229</v>
-      </c>
-      <c r="Q8" s="56" t="s">
+      <c r="P8" s="36" t="s">
+        <v>209</v>
+      </c>
+      <c r="Q8" s="36" t="s">
         <v>38</v>
       </c>
-      <c r="R8" s="56" t="s">
-        <v>229</v>
-      </c>
-      <c r="S8" s="56" t="s">
-        <v>229</v>
-      </c>
-      <c r="T8" s="56" t="s">
+      <c r="R8" s="36" t="s">
+        <v>209</v>
+      </c>
+      <c r="S8" s="36" t="s">
+        <v>209</v>
+      </c>
+      <c r="T8" s="36" t="s">
         <v>35</v>
       </c>
-      <c r="U8" s="56" t="s">
+      <c r="U8" s="36" t="s">
         <v>36</v>
       </c>
-      <c r="V8" s="56" t="s">
+      <c r="V8" s="36" t="s">
         <v>39</v>
       </c>
-      <c r="W8" s="56" t="s">
+      <c r="W8" s="36" t="s">
         <v>40</v>
       </c>
-      <c r="X8" s="56" t="s">
+      <c r="X8" s="36" t="s">
         <v>34</v>
       </c>
-      <c r="Y8" s="56" t="s">
+      <c r="Y8" s="36" t="s">
         <v>41</v>
       </c>
       <c r="Z8" s="16" t="s">
@@ -2467,17 +2467,17 @@
       <c r="AA8" s="16" t="s">
         <v>42</v>
       </c>
-      <c r="AB8" s="56" t="s">
-        <v>229</v>
-      </c>
-      <c r="AC8" s="56" t="s">
+      <c r="AB8" s="36" t="s">
+        <v>209</v>
+      </c>
+      <c r="AC8" s="36" t="s">
         <v>38</v>
       </c>
-      <c r="AD8" s="56" t="s">
-        <v>229</v>
-      </c>
-      <c r="AE8" s="56" t="s">
-        <v>229</v>
+      <c r="AD8" s="36" t="s">
+        <v>209</v>
+      </c>
+      <c r="AE8" s="36" t="s">
+        <v>209</v>
       </c>
       <c r="AF8" s="16" t="s">
         <v>42</v>
@@ -2488,44 +2488,44 @@
       <c r="AH8" s="15" t="s">
         <v>42</v>
       </c>
-      <c r="AI8" s="50" t="s">
-        <v>229</v>
-      </c>
-      <c r="AJ8" s="56" t="s">
-        <v>229</v>
-      </c>
-      <c r="AK8" s="89" t="s">
-        <v>229</v>
-      </c>
-      <c r="AL8" s="50" t="s">
-        <v>229</v>
-      </c>
-      <c r="AM8" s="56" t="s">
-        <v>229</v>
-      </c>
-      <c r="AN8" s="89" t="s">
-        <v>229</v>
-      </c>
-      <c r="AO8" s="88" t="s">
-        <v>229</v>
-      </c>
-      <c r="AP8" s="56" t="s">
-        <v>229</v>
-      </c>
-      <c r="AQ8" s="42" t="s">
-        <v>229</v>
-      </c>
-      <c r="AR8" s="88" t="s">
+      <c r="AI8" s="51" t="s">
+        <v>209</v>
+      </c>
+      <c r="AJ8" s="36" t="s">
+        <v>209</v>
+      </c>
+      <c r="AK8" s="53" t="s">
+        <v>209</v>
+      </c>
+      <c r="AL8" s="51" t="s">
+        <v>209</v>
+      </c>
+      <c r="AM8" s="36" t="s">
+        <v>209</v>
+      </c>
+      <c r="AN8" s="53" t="s">
+        <v>209</v>
+      </c>
+      <c r="AO8" s="38" t="s">
+        <v>209</v>
+      </c>
+      <c r="AP8" s="36" t="s">
+        <v>209</v>
+      </c>
+      <c r="AQ8" s="46" t="s">
+        <v>209</v>
+      </c>
+      <c r="AR8" s="38" t="s">
         <v>38</v>
       </c>
-      <c r="AS8" s="56" t="s">
-        <v>229</v>
-      </c>
-      <c r="AT8" s="56" t="s">
-        <v>229</v>
-      </c>
-      <c r="AU8" s="56" t="s">
-        <v>229</v>
+      <c r="AS8" s="36" t="s">
+        <v>209</v>
+      </c>
+      <c r="AT8" s="36" t="s">
+        <v>209</v>
+      </c>
+      <c r="AU8" s="36" t="s">
+        <v>209</v>
       </c>
       <c r="AV8" s="16" t="s">
         <v>42</v>
@@ -2533,17 +2533,17 @@
       <c r="AW8" s="16" t="s">
         <v>42</v>
       </c>
-      <c r="AX8" s="56" t="s">
-        <v>229</v>
-      </c>
-      <c r="AY8" s="56" t="s">
+      <c r="AX8" s="36" t="s">
+        <v>209</v>
+      </c>
+      <c r="AY8" s="36" t="s">
         <v>38</v>
       </c>
-      <c r="AZ8" s="56" t="s">
-        <v>229</v>
-      </c>
-      <c r="BA8" s="56" t="s">
-        <v>229</v>
+      <c r="AZ8" s="36" t="s">
+        <v>209</v>
+      </c>
+      <c r="BA8" s="36" t="s">
+        <v>209</v>
       </c>
       <c r="BB8" s="16" t="s">
         <v>42</v>
@@ -2551,35 +2551,35 @@
       <c r="BC8" s="16" t="s">
         <v>42</v>
       </c>
-      <c r="BD8" s="56" t="s">
+      <c r="BD8" s="36" t="s">
         <v>38</v>
       </c>
-      <c r="BE8" s="56" t="s">
-        <v>229</v>
-      </c>
-      <c r="BF8" s="56" t="s">
-        <v>229</v>
+      <c r="BE8" s="36" t="s">
+        <v>209</v>
+      </c>
+      <c r="BF8" s="36" t="s">
+        <v>209</v>
       </c>
       <c r="BG8" s="15" t="s">
         <v>42</v>
       </c>
-      <c r="BH8" s="39" t="s">
+      <c r="BH8" s="57" t="s">
         <v>38</v>
       </c>
-      <c r="BI8" s="56" t="s">
-        <v>229</v>
-      </c>
-      <c r="BJ8" s="56" t="s">
-        <v>229</v>
-      </c>
-      <c r="BK8" s="80" t="s">
-        <v>229</v>
-      </c>
-      <c r="BL8" s="83"/>
-      <c r="BM8" s="83"/>
-      <c r="BN8" s="84"/>
-      <c r="BO8" s="56" t="s">
-        <v>229</v>
+      <c r="BI8" s="36" t="s">
+        <v>209</v>
+      </c>
+      <c r="BJ8" s="36" t="s">
+        <v>209</v>
+      </c>
+      <c r="BK8" s="40" t="s">
+        <v>209</v>
+      </c>
+      <c r="BL8" s="41"/>
+      <c r="BM8" s="41"/>
+      <c r="BN8" s="39"/>
+      <c r="BO8" s="36" t="s">
+        <v>209</v>
       </c>
       <c r="BP8" s="16" t="s">
         <v>42</v>
@@ -2587,315 +2587,315 @@
       <c r="BQ8" s="15" t="s">
         <v>42</v>
       </c>
-      <c r="BR8" s="56" t="s">
-        <v>229</v>
-      </c>
-      <c r="BS8" s="56" t="s">
+      <c r="BR8" s="36" t="s">
+        <v>209</v>
+      </c>
+      <c r="BS8" s="36" t="s">
         <v>38</v>
       </c>
-      <c r="BT8" s="56" t="s">
-        <v>229</v>
-      </c>
-      <c r="BU8" s="56" t="s">
-        <v>229</v>
-      </c>
-      <c r="BV8" s="80" t="s">
-        <v>229</v>
-      </c>
-      <c r="BW8" s="83"/>
-      <c r="BX8" s="83"/>
-      <c r="BY8" s="84"/>
+      <c r="BT8" s="36" t="s">
+        <v>209</v>
+      </c>
+      <c r="BU8" s="36" t="s">
+        <v>209</v>
+      </c>
+      <c r="BV8" s="40" t="s">
+        <v>209</v>
+      </c>
+      <c r="BW8" s="41"/>
+      <c r="BX8" s="41"/>
+      <c r="BY8" s="39"/>
       <c r="BZ8" s="16" t="s">
         <v>42</v>
       </c>
       <c r="CA8" s="16" t="s">
         <v>42</v>
       </c>
-      <c r="CB8" s="56" t="s">
+      <c r="CB8" s="36" t="s">
         <v>38</v>
       </c>
-      <c r="CC8" s="56" t="s">
-        <v>229</v>
-      </c>
-      <c r="CD8" s="56" t="s">
-        <v>229</v>
-      </c>
-      <c r="CE8" s="80" t="s">
-        <v>229</v>
-      </c>
-      <c r="CF8" s="83"/>
-      <c r="CG8" s="83"/>
-      <c r="CH8" s="84"/>
+      <c r="CC8" s="36" t="s">
+        <v>209</v>
+      </c>
+      <c r="CD8" s="36" t="s">
+        <v>209</v>
+      </c>
+      <c r="CE8" s="40" t="s">
+        <v>209</v>
+      </c>
+      <c r="CF8" s="41"/>
+      <c r="CG8" s="41"/>
+      <c r="CH8" s="39"/>
       <c r="CI8" s="17" t="s">
         <v>42</v>
       </c>
-      <c r="CJ8" s="56" t="s">
-        <v>229</v>
-      </c>
-      <c r="CK8" s="56" t="s">
-        <v>229</v>
-      </c>
-      <c r="CL8" s="56" t="s">
-        <v>229</v>
-      </c>
-      <c r="CM8" s="56" t="s">
-        <v>229</v>
-      </c>
-      <c r="CN8" s="56" t="s">
-        <v>229</v>
-      </c>
-      <c r="CO8" s="56" t="s">
-        <v>229</v>
-      </c>
-      <c r="CP8" s="56" t="s">
-        <v>229</v>
+      <c r="CJ8" s="36" t="s">
+        <v>209</v>
+      </c>
+      <c r="CK8" s="36" t="s">
+        <v>209</v>
+      </c>
+      <c r="CL8" s="36" t="s">
+        <v>209</v>
+      </c>
+      <c r="CM8" s="36" t="s">
+        <v>209</v>
+      </c>
+      <c r="CN8" s="36" t="s">
+        <v>209</v>
+      </c>
+      <c r="CO8" s="36" t="s">
+        <v>209</v>
+      </c>
+      <c r="CP8" s="36" t="s">
+        <v>209</v>
       </c>
     </row>
     <row r="9" spans="1:94" s="2" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="39"/>
-      <c r="B9" s="42"/>
-      <c r="C9" s="50"/>
-      <c r="D9" s="54"/>
-      <c r="E9" s="56"/>
-      <c r="F9" s="56"/>
-      <c r="G9" s="56"/>
-      <c r="H9" s="56"/>
-      <c r="I9" s="56"/>
-      <c r="J9" s="56"/>
-      <c r="K9" s="56"/>
-      <c r="L9" s="56"/>
-      <c r="M9" s="56"/>
-      <c r="N9" s="56"/>
-      <c r="O9" s="91"/>
-      <c r="P9" s="56"/>
-      <c r="Q9" s="56"/>
-      <c r="R9" s="56"/>
-      <c r="S9" s="56"/>
-      <c r="T9" s="56"/>
-      <c r="U9" s="56"/>
-      <c r="V9" s="56"/>
-      <c r="W9" s="56"/>
-      <c r="X9" s="56"/>
-      <c r="Y9" s="56"/>
+      <c r="A9" s="57"/>
+      <c r="B9" s="46"/>
+      <c r="C9" s="51"/>
+      <c r="D9" s="90"/>
+      <c r="E9" s="36"/>
+      <c r="F9" s="36"/>
+      <c r="G9" s="36"/>
+      <c r="H9" s="36"/>
+      <c r="I9" s="36"/>
+      <c r="J9" s="36"/>
+      <c r="K9" s="36"/>
+      <c r="L9" s="36"/>
+      <c r="M9" s="36"/>
+      <c r="N9" s="36"/>
+      <c r="O9" s="55"/>
+      <c r="P9" s="36"/>
+      <c r="Q9" s="36"/>
+      <c r="R9" s="36"/>
+      <c r="S9" s="36"/>
+      <c r="T9" s="36"/>
+      <c r="U9" s="36"/>
+      <c r="V9" s="36"/>
+      <c r="W9" s="36"/>
+      <c r="X9" s="36"/>
+      <c r="Y9" s="36"/>
       <c r="Z9" s="18" t="s">
-        <v>229</v>
+        <v>209</v>
       </c>
       <c r="AA9" s="18" t="s">
-        <v>229</v>
-      </c>
-      <c r="AB9" s="56"/>
-      <c r="AC9" s="56"/>
-      <c r="AD9" s="56"/>
-      <c r="AE9" s="56"/>
+        <v>209</v>
+      </c>
+      <c r="AB9" s="36"/>
+      <c r="AC9" s="36"/>
+      <c r="AD9" s="36"/>
+      <c r="AE9" s="36"/>
       <c r="AF9" s="18" t="s">
-        <v>229</v>
+        <v>209</v>
       </c>
       <c r="AG9" s="18" t="s">
-        <v>229</v>
-      </c>
-      <c r="AH9" s="80" t="s">
-        <v>229</v>
-      </c>
-      <c r="AI9" s="50"/>
-      <c r="AJ9" s="56"/>
-      <c r="AK9" s="89"/>
-      <c r="AL9" s="50"/>
-      <c r="AM9" s="56"/>
-      <c r="AN9" s="89"/>
-      <c r="AO9" s="88"/>
-      <c r="AP9" s="56"/>
-      <c r="AQ9" s="42"/>
-      <c r="AR9" s="88"/>
-      <c r="AS9" s="56"/>
-      <c r="AT9" s="56"/>
-      <c r="AU9" s="56"/>
+        <v>209</v>
+      </c>
+      <c r="AH9" s="40" t="s">
+        <v>209</v>
+      </c>
+      <c r="AI9" s="51"/>
+      <c r="AJ9" s="36"/>
+      <c r="AK9" s="53"/>
+      <c r="AL9" s="51"/>
+      <c r="AM9" s="36"/>
+      <c r="AN9" s="53"/>
+      <c r="AO9" s="38"/>
+      <c r="AP9" s="36"/>
+      <c r="AQ9" s="46"/>
+      <c r="AR9" s="38"/>
+      <c r="AS9" s="36"/>
+      <c r="AT9" s="36"/>
+      <c r="AU9" s="36"/>
       <c r="AV9" s="18" t="s">
-        <v>229</v>
+        <v>209</v>
       </c>
       <c r="AW9" s="18" t="s">
-        <v>229</v>
-      </c>
-      <c r="AX9" s="56"/>
-      <c r="AY9" s="56"/>
-      <c r="AZ9" s="56"/>
-      <c r="BA9" s="56"/>
+        <v>209</v>
+      </c>
+      <c r="AX9" s="36"/>
+      <c r="AY9" s="36"/>
+      <c r="AZ9" s="36"/>
+      <c r="BA9" s="36"/>
       <c r="BB9" s="18" t="s">
-        <v>229</v>
+        <v>209</v>
       </c>
       <c r="BC9" s="18" t="s">
-        <v>229</v>
-      </c>
-      <c r="BD9" s="56"/>
-      <c r="BE9" s="56"/>
-      <c r="BF9" s="56"/>
-      <c r="BG9" s="43" t="s">
-        <v>229</v>
-      </c>
-      <c r="BH9" s="39"/>
-      <c r="BI9" s="56"/>
-      <c r="BJ9" s="56"/>
-      <c r="BK9" s="81"/>
-      <c r="BL9" s="85"/>
-      <c r="BM9" s="85"/>
-      <c r="BN9" s="86"/>
-      <c r="BO9" s="56"/>
+        <v>209</v>
+      </c>
+      <c r="BD9" s="36"/>
+      <c r="BE9" s="36"/>
+      <c r="BF9" s="36"/>
+      <c r="BG9" s="47" t="s">
+        <v>209</v>
+      </c>
+      <c r="BH9" s="57"/>
+      <c r="BI9" s="36"/>
+      <c r="BJ9" s="36"/>
+      <c r="BK9" s="42"/>
+      <c r="BL9" s="43"/>
+      <c r="BM9" s="43"/>
+      <c r="BN9" s="44"/>
+      <c r="BO9" s="36"/>
       <c r="BP9" s="18" t="s">
-        <v>229</v>
+        <v>209</v>
       </c>
       <c r="BQ9" s="18" t="s">
-        <v>229</v>
-      </c>
-      <c r="BR9" s="56"/>
-      <c r="BS9" s="56"/>
-      <c r="BT9" s="56"/>
-      <c r="BU9" s="56"/>
-      <c r="BV9" s="81"/>
-      <c r="BW9" s="85"/>
-      <c r="BX9" s="85"/>
-      <c r="BY9" s="86"/>
+        <v>209</v>
+      </c>
+      <c r="BR9" s="36"/>
+      <c r="BS9" s="36"/>
+      <c r="BT9" s="36"/>
+      <c r="BU9" s="36"/>
+      <c r="BV9" s="42"/>
+      <c r="BW9" s="43"/>
+      <c r="BX9" s="43"/>
+      <c r="BY9" s="44"/>
       <c r="BZ9" s="18" t="s">
-        <v>229</v>
+        <v>209</v>
       </c>
       <c r="CA9" s="18" t="s">
-        <v>229</v>
-      </c>
-      <c r="CB9" s="56"/>
-      <c r="CC9" s="56"/>
-      <c r="CD9" s="56"/>
-      <c r="CE9" s="81"/>
-      <c r="CF9" s="85"/>
-      <c r="CG9" s="85"/>
-      <c r="CH9" s="86"/>
-      <c r="CI9" s="43" t="s">
-        <v>229</v>
-      </c>
-      <c r="CJ9" s="56"/>
-      <c r="CK9" s="56"/>
-      <c r="CL9" s="56"/>
-      <c r="CM9" s="56"/>
-      <c r="CN9" s="56"/>
-      <c r="CO9" s="56"/>
-      <c r="CP9" s="56"/>
+        <v>209</v>
+      </c>
+      <c r="CB9" s="36"/>
+      <c r="CC9" s="36"/>
+      <c r="CD9" s="36"/>
+      <c r="CE9" s="42"/>
+      <c r="CF9" s="43"/>
+      <c r="CG9" s="43"/>
+      <c r="CH9" s="44"/>
+      <c r="CI9" s="47" t="s">
+        <v>209</v>
+      </c>
+      <c r="CJ9" s="36"/>
+      <c r="CK9" s="36"/>
+      <c r="CL9" s="36"/>
+      <c r="CM9" s="36"/>
+      <c r="CN9" s="36"/>
+      <c r="CO9" s="36"/>
+      <c r="CP9" s="36"/>
     </row>
     <row r="10" spans="1:94" s="2" customFormat="1" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="40"/>
-      <c r="B10" s="43"/>
-      <c r="C10" s="51"/>
-      <c r="D10" s="55"/>
-      <c r="E10" s="57"/>
-      <c r="F10" s="57"/>
-      <c r="G10" s="57"/>
-      <c r="H10" s="57"/>
-      <c r="I10" s="57"/>
-      <c r="J10" s="57"/>
-      <c r="K10" s="57"/>
-      <c r="L10" s="57"/>
-      <c r="M10" s="57"/>
-      <c r="N10" s="57"/>
-      <c r="O10" s="91"/>
-      <c r="P10" s="57"/>
-      <c r="Q10" s="57"/>
-      <c r="R10" s="57"/>
-      <c r="S10" s="57"/>
-      <c r="T10" s="57"/>
-      <c r="U10" s="57"/>
-      <c r="V10" s="57"/>
-      <c r="W10" s="57"/>
-      <c r="X10" s="57"/>
-      <c r="Y10" s="57"/>
+      <c r="A10" s="58"/>
+      <c r="B10" s="47"/>
+      <c r="C10" s="52"/>
+      <c r="D10" s="91"/>
+      <c r="E10" s="37"/>
+      <c r="F10" s="37"/>
+      <c r="G10" s="37"/>
+      <c r="H10" s="37"/>
+      <c r="I10" s="37"/>
+      <c r="J10" s="37"/>
+      <c r="K10" s="37"/>
+      <c r="L10" s="37"/>
+      <c r="M10" s="37"/>
+      <c r="N10" s="37"/>
+      <c r="O10" s="55"/>
+      <c r="P10" s="37"/>
+      <c r="Q10" s="37"/>
+      <c r="R10" s="37"/>
+      <c r="S10" s="37"/>
+      <c r="T10" s="37"/>
+      <c r="U10" s="37"/>
+      <c r="V10" s="37"/>
+      <c r="W10" s="37"/>
+      <c r="X10" s="37"/>
+      <c r="Y10" s="37"/>
       <c r="Z10" s="19" t="s">
-        <v>229</v>
+        <v>209</v>
       </c>
       <c r="AA10" s="19" t="s">
         <v>38</v>
       </c>
-      <c r="AB10" s="57"/>
-      <c r="AC10" s="57"/>
-      <c r="AD10" s="57"/>
-      <c r="AE10" s="57"/>
+      <c r="AB10" s="37"/>
+      <c r="AC10" s="37"/>
+      <c r="AD10" s="37"/>
+      <c r="AE10" s="37"/>
       <c r="AF10" s="19" t="s">
-        <v>229</v>
+        <v>209</v>
       </c>
       <c r="AG10" s="19" t="s">
         <v>38</v>
       </c>
-      <c r="AH10" s="81"/>
-      <c r="AI10" s="51"/>
-      <c r="AJ10" s="57"/>
-      <c r="AK10" s="90"/>
-      <c r="AL10" s="51"/>
-      <c r="AM10" s="57"/>
-      <c r="AN10" s="90"/>
-      <c r="AO10" s="84"/>
-      <c r="AP10" s="57"/>
-      <c r="AQ10" s="43"/>
-      <c r="AR10" s="84"/>
-      <c r="AS10" s="57"/>
-      <c r="AT10" s="57"/>
-      <c r="AU10" s="57"/>
+      <c r="AH10" s="42"/>
+      <c r="AI10" s="52"/>
+      <c r="AJ10" s="37"/>
+      <c r="AK10" s="54"/>
+      <c r="AL10" s="52"/>
+      <c r="AM10" s="37"/>
+      <c r="AN10" s="54"/>
+      <c r="AO10" s="39"/>
+      <c r="AP10" s="37"/>
+      <c r="AQ10" s="47"/>
+      <c r="AR10" s="39"/>
+      <c r="AS10" s="37"/>
+      <c r="AT10" s="37"/>
+      <c r="AU10" s="37"/>
       <c r="AV10" s="19" t="s">
-        <v>229</v>
+        <v>209</v>
       </c>
       <c r="AW10" s="19" t="s">
         <v>38</v>
       </c>
-      <c r="AX10" s="57"/>
-      <c r="AY10" s="57"/>
-      <c r="AZ10" s="57"/>
-      <c r="BA10" s="57"/>
+      <c r="AX10" s="37"/>
+      <c r="AY10" s="37"/>
+      <c r="AZ10" s="37"/>
+      <c r="BA10" s="37"/>
       <c r="BB10" s="19" t="s">
-        <v>229</v>
+        <v>209</v>
       </c>
       <c r="BC10" s="19" t="s">
         <v>38</v>
       </c>
-      <c r="BD10" s="57"/>
-      <c r="BE10" s="57"/>
-      <c r="BF10" s="57"/>
-      <c r="BG10" s="82"/>
-      <c r="BH10" s="40"/>
-      <c r="BI10" s="57"/>
-      <c r="BJ10" s="57"/>
-      <c r="BK10" s="81"/>
-      <c r="BL10" s="87"/>
-      <c r="BM10" s="87"/>
-      <c r="BN10" s="86"/>
-      <c r="BO10" s="57"/>
+      <c r="BD10" s="37"/>
+      <c r="BE10" s="37"/>
+      <c r="BF10" s="37"/>
+      <c r="BG10" s="56"/>
+      <c r="BH10" s="58"/>
+      <c r="BI10" s="37"/>
+      <c r="BJ10" s="37"/>
+      <c r="BK10" s="42"/>
+      <c r="BL10" s="45"/>
+      <c r="BM10" s="45"/>
+      <c r="BN10" s="44"/>
+      <c r="BO10" s="37"/>
       <c r="BP10" s="19" t="s">
-        <v>229</v>
+        <v>209</v>
       </c>
       <c r="BQ10" s="19" t="s">
         <v>38</v>
       </c>
-      <c r="BR10" s="57"/>
-      <c r="BS10" s="57"/>
-      <c r="BT10" s="57"/>
-      <c r="BU10" s="57"/>
-      <c r="BV10" s="81"/>
-      <c r="BW10" s="87"/>
-      <c r="BX10" s="87"/>
-      <c r="BY10" s="86"/>
+      <c r="BR10" s="37"/>
+      <c r="BS10" s="37"/>
+      <c r="BT10" s="37"/>
+      <c r="BU10" s="37"/>
+      <c r="BV10" s="42"/>
+      <c r="BW10" s="45"/>
+      <c r="BX10" s="45"/>
+      <c r="BY10" s="44"/>
       <c r="BZ10" s="19" t="s">
-        <v>229</v>
+        <v>209</v>
       </c>
       <c r="CA10" s="19" t="s">
         <v>38</v>
       </c>
-      <c r="CB10" s="57"/>
-      <c r="CC10" s="57"/>
-      <c r="CD10" s="57"/>
-      <c r="CE10" s="81"/>
-      <c r="CF10" s="87"/>
-      <c r="CG10" s="87"/>
-      <c r="CH10" s="86"/>
-      <c r="CI10" s="82"/>
-      <c r="CJ10" s="57"/>
-      <c r="CK10" s="57"/>
-      <c r="CL10" s="57"/>
-      <c r="CM10" s="57"/>
-      <c r="CN10" s="57"/>
-      <c r="CO10" s="57"/>
-      <c r="CP10" s="57"/>
+      <c r="CB10" s="37"/>
+      <c r="CC10" s="37"/>
+      <c r="CD10" s="37"/>
+      <c r="CE10" s="42"/>
+      <c r="CF10" s="45"/>
+      <c r="CG10" s="45"/>
+      <c r="CH10" s="44"/>
+      <c r="CI10" s="56"/>
+      <c r="CJ10" s="37"/>
+      <c r="CK10" s="37"/>
+      <c r="CL10" s="37"/>
+      <c r="CM10" s="37"/>
+      <c r="CN10" s="37"/>
+      <c r="CO10" s="37"/>
+      <c r="CP10" s="37"/>
     </row>
     <row r="11" spans="1:94" s="1" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A11" s="22" t="s">
@@ -2936,13 +2936,13 @@
         <v>55</v>
       </c>
       <c r="N11" s="29" t="s">
-        <v>110</v>
+        <v>100</v>
       </c>
       <c r="O11" s="29" t="s">
-        <v>111</v>
+        <v>101</v>
       </c>
       <c r="P11" s="29" t="s">
-        <v>112</v>
+        <v>102</v>
       </c>
       <c r="Q11" s="29" t="s">
         <v>56</v>
@@ -2972,31 +2972,31 @@
         <v>64</v>
       </c>
       <c r="Z11" s="29" t="s">
-        <v>113</v>
+        <v>103</v>
       </c>
       <c r="AA11" s="29" t="s">
-        <v>114</v>
+        <v>104</v>
       </c>
       <c r="AB11" s="29" t="s">
         <v>65</v>
       </c>
       <c r="AC11" s="29" t="s">
-        <v>230</v>
+        <v>210</v>
       </c>
       <c r="AD11" s="29" t="s">
-        <v>231</v>
+        <v>211</v>
       </c>
       <c r="AE11" s="29" t="s">
-        <v>232</v>
+        <v>212</v>
       </c>
       <c r="AF11" s="29" t="s">
-        <v>115</v>
+        <v>105</v>
       </c>
       <c r="AG11" s="29" t="s">
-        <v>116</v>
+        <v>106</v>
       </c>
       <c r="AH11" s="24" t="s">
-        <v>117</v>
+        <v>107</v>
       </c>
       <c r="AI11" s="28" t="s">
         <v>66</v>
@@ -3005,7 +3005,7 @@
         <v>67</v>
       </c>
       <c r="AK11" s="26" t="s">
-        <v>222</v>
+        <v>202</v>
       </c>
       <c r="AL11" s="24" t="s">
         <v>68</v>
@@ -3014,7 +3014,7 @@
         <v>69</v>
       </c>
       <c r="AN11" s="26" t="s">
-        <v>223</v>
+        <v>203</v>
       </c>
       <c r="AO11" s="31" t="s">
         <v>70</v>
@@ -3023,7 +3023,7 @@
         <v>71</v>
       </c>
       <c r="AQ11" s="26" t="s">
-        <v>224</v>
+        <v>204</v>
       </c>
       <c r="AR11" s="30" t="s">
         <v>72</v>
@@ -3038,13 +3038,13 @@
         <v>75</v>
       </c>
       <c r="AV11" s="29" t="s">
-        <v>118</v>
+        <v>108</v>
       </c>
       <c r="AW11" s="29" t="s">
-        <v>119</v>
+        <v>109</v>
       </c>
       <c r="AX11" s="29" t="s">
-        <v>120</v>
+        <v>110</v>
       </c>
       <c r="AY11" s="29" t="s">
         <v>76</v>
@@ -3056,450 +3056,457 @@
         <v>78</v>
       </c>
       <c r="BB11" s="29" t="s">
-        <v>121</v>
+        <v>111</v>
       </c>
       <c r="BC11" s="29" t="s">
-        <v>122</v>
+        <v>112</v>
       </c>
       <c r="BD11" s="29" t="s">
+        <v>216</v>
+      </c>
+      <c r="BE11" s="29" t="s">
+        <v>217</v>
+      </c>
+      <c r="BF11" s="29" t="s">
+        <v>218</v>
+      </c>
+      <c r="BG11" s="24" t="s">
+        <v>113</v>
+      </c>
+      <c r="BH11" s="28" t="s">
+        <v>200</v>
+      </c>
+      <c r="BI11" s="29" t="s">
         <v>79</v>
       </c>
-      <c r="BE11" s="29" t="s">
+      <c r="BJ11" s="29" t="s">
         <v>80</v>
       </c>
-      <c r="BF11" s="29" t="s">
+      <c r="BK11" s="29" t="s">
         <v>81</v>
       </c>
-      <c r="BG11" s="24" t="s">
-        <v>123</v>
-      </c>
-      <c r="BH11" s="28" t="s">
-        <v>220</v>
-      </c>
-      <c r="BI11" s="29" t="s">
+      <c r="BL11" s="29" t="s">
         <v>82</v>
       </c>
-      <c r="BJ11" s="29" t="s">
+      <c r="BM11" s="29" t="s">
         <v>83</v>
       </c>
-      <c r="BK11" s="29" t="s">
+      <c r="BN11" s="29" t="s">
         <v>84</v>
       </c>
-      <c r="BL11" s="29" t="s">
+      <c r="BO11" s="29" t="s">
         <v>85</v>
       </c>
-      <c r="BM11" s="29" t="s">
+      <c r="BP11" s="29" t="s">
+        <v>114</v>
+      </c>
+      <c r="BQ11" s="29" t="s">
+        <v>115</v>
+      </c>
+      <c r="BR11" s="29" t="s">
+        <v>116</v>
+      </c>
+      <c r="BS11" s="29" t="s">
         <v>86</v>
       </c>
-      <c r="BN11" s="29" t="s">
+      <c r="BT11" s="29" t="s">
         <v>87</v>
       </c>
-      <c r="BO11" s="29" t="s">
+      <c r="BU11" s="29" t="s">
         <v>88</v>
       </c>
-      <c r="BP11" s="29" t="s">
-        <v>124</v>
-      </c>
-      <c r="BQ11" s="29" t="s">
-        <v>125</v>
-      </c>
-      <c r="BR11" s="29" t="s">
-        <v>126</v>
-      </c>
-      <c r="BS11" s="29" t="s">
+      <c r="BV11" s="29" t="s">
         <v>89</v>
       </c>
-      <c r="BT11" s="29" t="s">
+      <c r="BW11" s="29" t="s">
         <v>90</v>
       </c>
-      <c r="BU11" s="29" t="s">
+      <c r="BX11" s="29" t="s">
         <v>91</v>
       </c>
-      <c r="BV11" s="29" t="s">
+      <c r="BY11" s="29" t="s">
         <v>92</v>
       </c>
-      <c r="BW11" s="29" t="s">
+      <c r="BZ11" s="29" t="s">
+        <v>117</v>
+      </c>
+      <c r="CA11" s="29" t="s">
+        <v>118</v>
+      </c>
+      <c r="CB11" s="29" t="s">
+        <v>226</v>
+      </c>
+      <c r="CC11" s="29" t="s">
+        <v>227</v>
+      </c>
+      <c r="CD11" s="29" t="s">
+        <v>228</v>
+      </c>
+      <c r="CE11" s="29" t="s">
+        <v>229</v>
+      </c>
+      <c r="CF11" s="29" t="s">
+        <v>230</v>
+      </c>
+      <c r="CG11" s="29" t="s">
+        <v>231</v>
+      </c>
+      <c r="CH11" s="29" t="s">
+        <v>232</v>
+      </c>
+      <c r="CI11" s="26" t="s">
+        <v>119</v>
+      </c>
+      <c r="CJ11" s="31" t="s">
         <v>93</v>
       </c>
-      <c r="BX11" s="29" t="s">
+      <c r="CK11" s="29" t="s">
         <v>94</v>
       </c>
-      <c r="BY11" s="29" t="s">
+      <c r="CL11" s="29" t="s">
         <v>95</v>
       </c>
-      <c r="BZ11" s="29" t="s">
-        <v>127</v>
-      </c>
-      <c r="CA11" s="29" t="s">
-        <v>128</v>
-      </c>
-      <c r="CB11" s="29" t="s">
+      <c r="CM11" s="29" t="s">
         <v>96</v>
       </c>
-      <c r="CC11" s="29" t="s">
+      <c r="CN11" s="29" t="s">
         <v>97</v>
       </c>
-      <c r="CD11" s="29" t="s">
+      <c r="CO11" s="29" t="s">
         <v>98</v>
       </c>
-      <c r="CE11" s="29" t="s">
+      <c r="CP11" s="26" t="s">
         <v>99</v>
-      </c>
-      <c r="CF11" s="29" t="s">
-        <v>100</v>
-      </c>
-      <c r="CG11" s="29" t="s">
-        <v>101</v>
-      </c>
-      <c r="CH11" s="29" t="s">
-        <v>102</v>
-      </c>
-      <c r="CI11" s="26" t="s">
-        <v>129</v>
-      </c>
-      <c r="CJ11" s="31" t="s">
-        <v>103</v>
-      </c>
-      <c r="CK11" s="29" t="s">
-        <v>104</v>
-      </c>
-      <c r="CL11" s="29" t="s">
-        <v>105</v>
-      </c>
-      <c r="CM11" s="29" t="s">
-        <v>106</v>
-      </c>
-      <c r="CN11" s="29" t="s">
-        <v>107</v>
-      </c>
-      <c r="CO11" s="29" t="s">
-        <v>108</v>
-      </c>
-      <c r="CP11" s="26" t="s">
-        <v>109</v>
       </c>
     </row>
     <row r="12" spans="1:94" s="13" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="20" t="s">
+        <v>121</v>
+      </c>
+      <c r="B12" s="21" t="s">
+        <v>120</v>
+      </c>
+      <c r="C12" s="32" t="s">
+        <v>122</v>
+      </c>
+      <c r="D12" s="33" t="s">
+        <v>123</v>
+      </c>
+      <c r="E12" s="33" t="s">
+        <v>124</v>
+      </c>
+      <c r="F12" s="33" t="s">
+        <v>125</v>
+      </c>
+      <c r="G12" s="33" t="s">
+        <v>126</v>
+      </c>
+      <c r="H12" s="33" t="s">
+        <v>127</v>
+      </c>
+      <c r="I12" s="33" t="s">
+        <v>128</v>
+      </c>
+      <c r="J12" s="33" t="s">
+        <v>129</v>
+      </c>
+      <c r="K12" s="33" t="s">
+        <v>130</v>
+      </c>
+      <c r="L12" s="33" t="s">
         <v>131</v>
       </c>
-      <c r="B12" s="21" t="s">
-        <v>130</v>
-      </c>
-      <c r="C12" s="32" t="s">
+      <c r="M12" s="33" t="s">
         <v>132</v>
       </c>
-      <c r="D12" s="33" t="s">
+      <c r="N12" s="33" t="s">
         <v>133</v>
       </c>
-      <c r="E12" s="33" t="s">
+      <c r="O12" s="33" t="s">
         <v>134</v>
       </c>
-      <c r="F12" s="33" t="s">
+      <c r="P12" s="33" t="s">
         <v>135</v>
       </c>
-      <c r="G12" s="33" t="s">
+      <c r="Q12" s="33" t="s">
         <v>136</v>
       </c>
-      <c r="H12" s="33" t="s">
+      <c r="R12" s="34" t="s">
         <v>137</v>
       </c>
-      <c r="I12" s="33" t="s">
+      <c r="S12" s="33" t="s">
         <v>138</v>
       </c>
-      <c r="J12" s="33" t="s">
+      <c r="T12" s="33" t="s">
         <v>139</v>
       </c>
-      <c r="K12" s="33" t="s">
+      <c r="U12" s="33" t="s">
         <v>140</v>
       </c>
-      <c r="L12" s="33" t="s">
+      <c r="V12" s="33" t="s">
         <v>141</v>
       </c>
-      <c r="M12" s="33" t="s">
+      <c r="W12" s="33" t="s">
         <v>142</v>
       </c>
-      <c r="N12" s="33" t="s">
+      <c r="X12" s="33" t="s">
         <v>143</v>
       </c>
-      <c r="O12" s="33" t="s">
+      <c r="Y12" s="33" t="s">
         <v>144</v>
       </c>
-      <c r="P12" s="33" t="s">
+      <c r="Z12" s="33" t="s">
         <v>145</v>
       </c>
-      <c r="Q12" s="33" t="s">
+      <c r="AA12" s="33" t="s">
         <v>146</v>
       </c>
-      <c r="R12" s="34" t="s">
+      <c r="AB12" s="33" t="s">
         <v>147</v>
       </c>
-      <c r="S12" s="33" t="s">
+      <c r="AC12" s="33" t="s">
         <v>148</v>
       </c>
-      <c r="T12" s="33" t="s">
+      <c r="AD12" s="33" t="s">
         <v>149</v>
       </c>
-      <c r="U12" s="33" t="s">
+      <c r="AE12" s="33" t="s">
         <v>150</v>
       </c>
-      <c r="V12" s="33" t="s">
+      <c r="AF12" s="33" t="s">
         <v>151</v>
       </c>
-      <c r="W12" s="33" t="s">
+      <c r="AG12" s="33" t="s">
         <v>152</v>
       </c>
-      <c r="X12" s="33" t="s">
+      <c r="AH12" s="25" t="s">
         <v>153</v>
       </c>
-      <c r="Y12" s="33" t="s">
+      <c r="AI12" s="32" t="s">
         <v>154</v>
       </c>
-      <c r="Z12" s="33" t="s">
+      <c r="AJ12" s="33" t="s">
         <v>155</v>
       </c>
-      <c r="AA12" s="33" t="s">
+      <c r="AK12" s="27" t="s">
+        <v>205</v>
+      </c>
+      <c r="AL12" s="25" t="s">
         <v>156</v>
       </c>
-      <c r="AB12" s="33" t="s">
+      <c r="AM12" s="25" t="s">
         <v>157</v>
       </c>
-      <c r="AC12" s="33" t="s">
+      <c r="AN12" s="27" t="s">
+        <v>206</v>
+      </c>
+      <c r="AO12" s="35" t="s">
         <v>158</v>
       </c>
-      <c r="AD12" s="33" t="s">
+      <c r="AP12" s="33" t="s">
         <v>159</v>
       </c>
-      <c r="AE12" s="33" t="s">
+      <c r="AQ12" s="27" t="s">
+        <v>207</v>
+      </c>
+      <c r="AR12" s="34" t="s">
         <v>160</v>
       </c>
-      <c r="AF12" s="33" t="s">
+      <c r="AS12" s="33" t="s">
         <v>161</v>
       </c>
-      <c r="AG12" s="33" t="s">
+      <c r="AT12" s="33" t="s">
         <v>162</v>
       </c>
-      <c r="AH12" s="25" t="s">
+      <c r="AU12" s="33" t="s">
         <v>163</v>
       </c>
-      <c r="AI12" s="32" t="s">
+      <c r="AV12" s="33" t="s">
         <v>164</v>
       </c>
-      <c r="AJ12" s="33" t="s">
+      <c r="AW12" s="33" t="s">
         <v>165</v>
       </c>
-      <c r="AK12" s="27" t="s">
+      <c r="AX12" s="33" t="s">
+        <v>166</v>
+      </c>
+      <c r="AY12" s="33" t="s">
+        <v>167</v>
+      </c>
+      <c r="AZ12" s="33" t="s">
+        <v>168</v>
+      </c>
+      <c r="BA12" s="33" t="s">
+        <v>169</v>
+      </c>
+      <c r="BB12" s="33" t="s">
+        <v>170</v>
+      </c>
+      <c r="BC12" s="33" t="s">
+        <v>171</v>
+      </c>
+      <c r="BD12" s="33" t="s">
+        <v>213</v>
+      </c>
+      <c r="BE12" s="33" t="s">
+        <v>214</v>
+      </c>
+      <c r="BF12" s="33" t="s">
+        <v>215</v>
+      </c>
+      <c r="BG12" s="25" t="s">
+        <v>172</v>
+      </c>
+      <c r="BH12" s="32" t="s">
+        <v>201</v>
+      </c>
+      <c r="BI12" s="33" t="s">
+        <v>173</v>
+      </c>
+      <c r="BJ12" s="33" t="s">
+        <v>174</v>
+      </c>
+      <c r="BK12" s="33" t="s">
+        <v>175</v>
+      </c>
+      <c r="BL12" s="33" t="s">
+        <v>176</v>
+      </c>
+      <c r="BM12" s="33" t="s">
+        <v>177</v>
+      </c>
+      <c r="BN12" s="33" t="s">
+        <v>178</v>
+      </c>
+      <c r="BO12" s="33" t="s">
+        <v>179</v>
+      </c>
+      <c r="BP12" s="33" t="s">
+        <v>180</v>
+      </c>
+      <c r="BQ12" s="33" t="s">
+        <v>181</v>
+      </c>
+      <c r="BR12" s="33" t="s">
+        <v>182</v>
+      </c>
+      <c r="BS12" s="33" t="s">
+        <v>183</v>
+      </c>
+      <c r="BT12" s="33" t="s">
+        <v>184</v>
+      </c>
+      <c r="BU12" s="33" t="s">
+        <v>185</v>
+      </c>
+      <c r="BV12" s="33" t="s">
+        <v>186</v>
+      </c>
+      <c r="BW12" s="33" t="s">
+        <v>187</v>
+      </c>
+      <c r="BX12" s="33" t="s">
+        <v>188</v>
+      </c>
+      <c r="BY12" s="33" t="s">
+        <v>189</v>
+      </c>
+      <c r="BZ12" s="33" t="s">
+        <v>190</v>
+      </c>
+      <c r="CA12" s="33" t="s">
+        <v>191</v>
+      </c>
+      <c r="CB12" s="33" t="s">
+        <v>219</v>
+      </c>
+      <c r="CC12" s="33" t="s">
+        <v>220</v>
+      </c>
+      <c r="CD12" s="33" t="s">
+        <v>221</v>
+      </c>
+      <c r="CE12" s="33" t="s">
+        <v>222</v>
+      </c>
+      <c r="CF12" s="33" t="s">
+        <v>223</v>
+      </c>
+      <c r="CG12" s="33" t="s">
+        <v>224</v>
+      </c>
+      <c r="CH12" s="33" t="s">
         <v>225</v>
       </c>
-      <c r="AL12" s="25" t="s">
-        <v>166</v>
-      </c>
-      <c r="AM12" s="25" t="s">
-        <v>167</v>
-      </c>
-      <c r="AN12" s="27" t="s">
-        <v>226</v>
-      </c>
-      <c r="AO12" s="35" t="s">
-        <v>168</v>
-      </c>
-      <c r="AP12" s="33" t="s">
-        <v>169</v>
-      </c>
-      <c r="AQ12" s="27" t="s">
-        <v>227</v>
-      </c>
-      <c r="AR12" s="34" t="s">
-        <v>170</v>
-      </c>
-      <c r="AS12" s="33" t="s">
-        <v>171</v>
-      </c>
-      <c r="AT12" s="33" t="s">
-        <v>172</v>
-      </c>
-      <c r="AU12" s="33" t="s">
-        <v>173</v>
-      </c>
-      <c r="AV12" s="33" t="s">
-        <v>174</v>
-      </c>
-      <c r="AW12" s="33" t="s">
-        <v>175</v>
-      </c>
-      <c r="AX12" s="33" t="s">
-        <v>176</v>
-      </c>
-      <c r="AY12" s="33" t="s">
-        <v>177</v>
-      </c>
-      <c r="AZ12" s="33" t="s">
-        <v>178</v>
-      </c>
-      <c r="BA12" s="33" t="s">
-        <v>179</v>
-      </c>
-      <c r="BB12" s="33" t="s">
-        <v>180</v>
-      </c>
-      <c r="BC12" s="33" t="s">
-        <v>181</v>
-      </c>
-      <c r="BD12" s="33" t="s">
-        <v>182</v>
-      </c>
-      <c r="BE12" s="33" t="s">
-        <v>183</v>
-      </c>
-      <c r="BF12" s="33" t="s">
-        <v>184</v>
-      </c>
-      <c r="BG12" s="25" t="s">
-        <v>185</v>
-      </c>
-      <c r="BH12" s="32" t="s">
-        <v>221</v>
-      </c>
-      <c r="BI12" s="33" t="s">
-        <v>186</v>
-      </c>
-      <c r="BJ12" s="33" t="s">
-        <v>187</v>
-      </c>
-      <c r="BK12" s="33" t="s">
-        <v>188</v>
-      </c>
-      <c r="BL12" s="33" t="s">
-        <v>189</v>
-      </c>
-      <c r="BM12" s="33" t="s">
-        <v>190</v>
-      </c>
-      <c r="BN12" s="33" t="s">
-        <v>191</v>
-      </c>
-      <c r="BO12" s="33" t="s">
+      <c r="CI12" s="27" t="s">
         <v>192</v>
       </c>
-      <c r="BP12" s="33" t="s">
+      <c r="CJ12" s="35" t="s">
         <v>193</v>
       </c>
-      <c r="BQ12" s="33" t="s">
+      <c r="CK12" s="33" t="s">
         <v>194</v>
       </c>
-      <c r="BR12" s="33" t="s">
+      <c r="CL12" s="33" t="s">
         <v>195</v>
       </c>
-      <c r="BS12" s="33" t="s">
+      <c r="CM12" s="33" t="s">
         <v>196</v>
       </c>
-      <c r="BT12" s="33" t="s">
+      <c r="CN12" s="33" t="s">
         <v>197</v>
       </c>
-      <c r="BU12" s="33" t="s">
+      <c r="CO12" s="33" t="s">
         <v>198</v>
       </c>
-      <c r="BV12" s="33" t="s">
+      <c r="CP12" s="33" t="s">
         <v>199</v>
-      </c>
-      <c r="BW12" s="33" t="s">
-        <v>200</v>
-      </c>
-      <c r="BX12" s="33" t="s">
-        <v>201</v>
-      </c>
-      <c r="BY12" s="33" t="s">
-        <v>202</v>
-      </c>
-      <c r="BZ12" s="33" t="s">
-        <v>203</v>
-      </c>
-      <c r="CA12" s="33" t="s">
-        <v>204</v>
-      </c>
-      <c r="CB12" s="33" t="s">
-        <v>205</v>
-      </c>
-      <c r="CC12" s="33" t="s">
-        <v>206</v>
-      </c>
-      <c r="CD12" s="33" t="s">
-        <v>207</v>
-      </c>
-      <c r="CE12" s="33" t="s">
-        <v>208</v>
-      </c>
-      <c r="CF12" s="33" t="s">
-        <v>209</v>
-      </c>
-      <c r="CG12" s="33" t="s">
-        <v>210</v>
-      </c>
-      <c r="CH12" s="33" t="s">
-        <v>211</v>
-      </c>
-      <c r="CI12" s="27" t="s">
-        <v>212</v>
-      </c>
-      <c r="CJ12" s="35" t="s">
-        <v>213</v>
-      </c>
-      <c r="CK12" s="33" t="s">
-        <v>214</v>
-      </c>
-      <c r="CL12" s="33" t="s">
-        <v>215</v>
-      </c>
-      <c r="CM12" s="33" t="s">
-        <v>216</v>
-      </c>
-      <c r="CN12" s="33" t="s">
-        <v>217</v>
-      </c>
-      <c r="CO12" s="33" t="s">
-        <v>218</v>
-      </c>
-      <c r="CP12" s="33" t="s">
-        <v>219</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="101">
-    <mergeCell ref="CM8:CM10"/>
-    <mergeCell ref="CN8:CN10"/>
-    <mergeCell ref="CB8:CB10"/>
-    <mergeCell ref="BO8:BO10"/>
-    <mergeCell ref="CO8:CO10"/>
-    <mergeCell ref="AR8:AR10"/>
-    <mergeCell ref="AS8:AS10"/>
-    <mergeCell ref="AT8:AT10"/>
-    <mergeCell ref="AU8:AU10"/>
-    <mergeCell ref="AX8:AX10"/>
-    <mergeCell ref="AY8:AY10"/>
-    <mergeCell ref="AZ8:AZ10"/>
-    <mergeCell ref="BA8:BA10"/>
-    <mergeCell ref="BD8:BD10"/>
-    <mergeCell ref="BJ8:BJ10"/>
-    <mergeCell ref="BK8:BN10"/>
-    <mergeCell ref="AQ8:AQ10"/>
-    <mergeCell ref="AL7:AN7"/>
-    <mergeCell ref="AL8:AL10"/>
-    <mergeCell ref="AM8:AM10"/>
-    <mergeCell ref="AN8:AN10"/>
-    <mergeCell ref="O8:O10"/>
-    <mergeCell ref="P8:P10"/>
-    <mergeCell ref="Q8:Q10"/>
-    <mergeCell ref="R8:R10"/>
-    <mergeCell ref="S8:S10"/>
-    <mergeCell ref="T8:T10"/>
-    <mergeCell ref="V8:V10"/>
-    <mergeCell ref="W8:W10"/>
-    <mergeCell ref="X8:X10"/>
-    <mergeCell ref="Y8:Y10"/>
-    <mergeCell ref="AB8:AB10"/>
-    <mergeCell ref="AC8:AC10"/>
-    <mergeCell ref="AD8:AD10"/>
-    <mergeCell ref="AE8:AE10"/>
+    <mergeCell ref="B1:AA1"/>
+    <mergeCell ref="B2:AA2"/>
+    <mergeCell ref="M3:P3"/>
+    <mergeCell ref="A5:A10"/>
+    <mergeCell ref="B5:B10"/>
+    <mergeCell ref="C5:AH5"/>
+    <mergeCell ref="C6:P6"/>
+    <mergeCell ref="Q6:AB6"/>
+    <mergeCell ref="AC6:AH6"/>
+    <mergeCell ref="C8:C10"/>
+    <mergeCell ref="E7:K7"/>
+    <mergeCell ref="S7:Y7"/>
+    <mergeCell ref="D8:D10"/>
+    <mergeCell ref="E8:E10"/>
+    <mergeCell ref="F8:F10"/>
+    <mergeCell ref="G8:G10"/>
+    <mergeCell ref="I8:I10"/>
+    <mergeCell ref="H8:H10"/>
+    <mergeCell ref="U8:U10"/>
+    <mergeCell ref="J8:J10"/>
+    <mergeCell ref="K8:K10"/>
+    <mergeCell ref="L8:L10"/>
+    <mergeCell ref="M8:M10"/>
+    <mergeCell ref="N8:N10"/>
+    <mergeCell ref="AI5:AK5"/>
+    <mergeCell ref="AO5:AQ5"/>
+    <mergeCell ref="AR5:BG5"/>
+    <mergeCell ref="BH5:CI5"/>
+    <mergeCell ref="CJ5:CO5"/>
+    <mergeCell ref="AL5:AN5"/>
+    <mergeCell ref="CP5:CP7"/>
+    <mergeCell ref="AR6:AX6"/>
+    <mergeCell ref="AY6:BC6"/>
+    <mergeCell ref="BD6:BF6"/>
+    <mergeCell ref="BH6:BR6"/>
+    <mergeCell ref="CO6:CO7"/>
+    <mergeCell ref="CJ6:CJ7"/>
+    <mergeCell ref="CK6:CN6"/>
+    <mergeCell ref="AI7:AK7"/>
+    <mergeCell ref="AO7:AQ7"/>
+    <mergeCell ref="BS6:CA6"/>
+    <mergeCell ref="CB6:CI6"/>
     <mergeCell ref="CP8:CP10"/>
     <mergeCell ref="AH9:AH10"/>
     <mergeCell ref="BG9:BG10"/>
@@ -3524,48 +3531,41 @@
     <mergeCell ref="AK8:AK10"/>
     <mergeCell ref="BE8:BE10"/>
     <mergeCell ref="AP8:AP10"/>
-    <mergeCell ref="AI5:AK5"/>
-    <mergeCell ref="AO5:AQ5"/>
-    <mergeCell ref="AR5:BG5"/>
-    <mergeCell ref="BH5:CI5"/>
-    <mergeCell ref="CJ5:CO5"/>
-    <mergeCell ref="AL5:AN5"/>
-    <mergeCell ref="CP5:CP7"/>
-    <mergeCell ref="AR6:AX6"/>
-    <mergeCell ref="AY6:BC6"/>
-    <mergeCell ref="BD6:BF6"/>
-    <mergeCell ref="BH6:BR6"/>
-    <mergeCell ref="CO6:CO7"/>
-    <mergeCell ref="CJ6:CJ7"/>
-    <mergeCell ref="CK6:CN6"/>
-    <mergeCell ref="AI7:AK7"/>
-    <mergeCell ref="AO7:AQ7"/>
-    <mergeCell ref="BS6:CA6"/>
-    <mergeCell ref="CB6:CI6"/>
-    <mergeCell ref="B1:AA1"/>
-    <mergeCell ref="B2:AA2"/>
-    <mergeCell ref="M3:P3"/>
-    <mergeCell ref="A5:A10"/>
-    <mergeCell ref="B5:B10"/>
-    <mergeCell ref="C5:AH5"/>
-    <mergeCell ref="C6:P6"/>
-    <mergeCell ref="Q6:AB6"/>
-    <mergeCell ref="AC6:AH6"/>
-    <mergeCell ref="C8:C10"/>
-    <mergeCell ref="E7:K7"/>
-    <mergeCell ref="S7:Y7"/>
-    <mergeCell ref="D8:D10"/>
-    <mergeCell ref="E8:E10"/>
-    <mergeCell ref="F8:F10"/>
-    <mergeCell ref="G8:G10"/>
-    <mergeCell ref="I8:I10"/>
-    <mergeCell ref="H8:H10"/>
-    <mergeCell ref="U8:U10"/>
-    <mergeCell ref="J8:J10"/>
-    <mergeCell ref="K8:K10"/>
-    <mergeCell ref="L8:L10"/>
-    <mergeCell ref="M8:M10"/>
-    <mergeCell ref="N8:N10"/>
+    <mergeCell ref="AQ8:AQ10"/>
+    <mergeCell ref="AL7:AN7"/>
+    <mergeCell ref="AL8:AL10"/>
+    <mergeCell ref="AM8:AM10"/>
+    <mergeCell ref="AN8:AN10"/>
+    <mergeCell ref="O8:O10"/>
+    <mergeCell ref="P8:P10"/>
+    <mergeCell ref="Q8:Q10"/>
+    <mergeCell ref="R8:R10"/>
+    <mergeCell ref="S8:S10"/>
+    <mergeCell ref="T8:T10"/>
+    <mergeCell ref="V8:V10"/>
+    <mergeCell ref="W8:W10"/>
+    <mergeCell ref="X8:X10"/>
+    <mergeCell ref="Y8:Y10"/>
+    <mergeCell ref="AB8:AB10"/>
+    <mergeCell ref="AC8:AC10"/>
+    <mergeCell ref="AD8:AD10"/>
+    <mergeCell ref="AE8:AE10"/>
+    <mergeCell ref="CM8:CM10"/>
+    <mergeCell ref="CN8:CN10"/>
+    <mergeCell ref="CB8:CB10"/>
+    <mergeCell ref="BO8:BO10"/>
+    <mergeCell ref="CO8:CO10"/>
+    <mergeCell ref="AR8:AR10"/>
+    <mergeCell ref="AS8:AS10"/>
+    <mergeCell ref="AT8:AT10"/>
+    <mergeCell ref="AU8:AU10"/>
+    <mergeCell ref="AX8:AX10"/>
+    <mergeCell ref="AY8:AY10"/>
+    <mergeCell ref="AZ8:AZ10"/>
+    <mergeCell ref="BA8:BA10"/>
+    <mergeCell ref="BD8:BD10"/>
+    <mergeCell ref="BJ8:BJ10"/>
+    <mergeCell ref="BK8:BN10"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>